<commit_message>
Update configuration templates and logging settings
- Updated 'ImportTemplate.xlsx' with new data.
- Removed obsolete 'jira-config.json'
</commit_message>
<xml_diff>
--- a/resources/templates/ImportTemplate.xlsx
+++ b/resources/templates/ImportTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workdir\DeerHide\sources\jira-toolkit\rsc\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jules/Workdir/sources/jira-toolkit/resources/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9471506-A60E-4104-83CF-1148AC344A3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8715B6CB-C258-0246-816F-293FA3525AAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13152" yWindow="6060" windowWidth="17568" windowHeight="12420" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
+    <workbookView xWindow="16820" yWindow="10420" windowWidth="17560" windowHeight="12420" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset" sheetId="1" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="111">
   <si>
     <t>IssueType</t>
   </si>
@@ -245,9 +245,6 @@
     <t>Creation Marker</t>
   </si>
   <si>
-    <t>JV</t>
-  </si>
-  <si>
     <t>Issue Type</t>
   </si>
   <si>
@@ -399,6 +396,12 @@
   </si>
   <si>
     <t>pod_test</t>
+  </si>
+  <si>
+    <t>tst</t>
+  </si>
+  <si>
+    <t>a</t>
   </si>
 </sst>
 </file>
@@ -922,7 +925,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -953,6 +956,15 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="16" applyAlignment="1">
       <alignment horizontal="left" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -999,7 +1011,291 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="56">
+  <dxfs count="88">
+    <dxf>
+      <fill>
+        <patternFill patternType="darkUp"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDAF2D0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2CEEF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <color theme="0" tint="-0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFF9B1AB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF99CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF6699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="darkUp"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDAF2D0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2CEEF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <color theme="0" tint="-0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFF9B1AB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF99CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF6699"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="darkUp"/>
@@ -1320,63 +1616,63 @@
 <file path=xl/namedSheetViews/namedSheetView1.xml><?xml version="1.0" encoding="utf-8"?>
 <namedSheetViews xmlns="http://schemas.microsoft.com/office/spreadsheetml/2019/namedsheetviews" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <namedSheetView name="View1" id="{77233F75-225A-4D7F-8A86-543E0A8C6E58}">
-    <nsvFilter filterId="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" ref="A1:AJ3" tableId="1"/>
+    <nsvFilter filterId="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" ref="A1:AJ5" tableId="1"/>
   </namedSheetView>
 </namedSheetViews>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" name="JiraDataset" displayName="JiraDataset" ref="A1:AJ3" totalsRowShown="0" headerRowDxfId="55" dataDxfId="54">
-  <autoFilter ref="A1:AJ3" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" name="JiraDataset" displayName="JiraDataset" ref="A1:AJ5" totalsRowShown="0" headerRowDxfId="87" dataDxfId="86">
+  <autoFilter ref="A1:AJ5" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}"/>
   <tableColumns count="36">
-    <tableColumn id="3" xr3:uid="{AF2EC907-349C-4651-852D-6E39C61E17FF}" name="Priority" dataDxfId="53"/>
-    <tableColumn id="2" xr3:uid="{E90C51F2-4386-421F-A3E4-E2CA9D43D396}" name="IssueType" dataDxfId="52"/>
-    <tableColumn id="1" xr3:uid="{BBAD373B-BA13-47E4-9F74-565F4D9E9680}" name="Summary" dataDxfId="51"/>
-    <tableColumn id="4" xr3:uid="{026E5B97-FAFC-4E46-860E-0B0C976B1148}" name="Issue Key" dataDxfId="50"/>
-    <tableColumn id="5" xr3:uid="{A2C262E8-D544-4669-99F1-151EDE081654}" name="Description" dataDxfId="49"/>
-    <tableColumn id="7" xr3:uid="{0FAD1ACC-432E-462C-8B89-71540710BCB5}" name="FixVersion" dataDxfId="48">
+    <tableColumn id="3" xr3:uid="{AF2EC907-349C-4651-852D-6E39C61E17FF}" name="Priority" dataDxfId="85"/>
+    <tableColumn id="2" xr3:uid="{E90C51F2-4386-421F-A3E4-E2CA9D43D396}" name="IssueType" dataDxfId="84"/>
+    <tableColumn id="1" xr3:uid="{BBAD373B-BA13-47E4-9F74-565F4D9E9680}" name="Summary" dataDxfId="83"/>
+    <tableColumn id="4" xr3:uid="{026E5B97-FAFC-4E46-860E-0B0C976B1148}" name="Issue Key" dataDxfId="82"/>
+    <tableColumn id="5" xr3:uid="{A2C262E8-D544-4669-99F1-151EDE081654}" name="Description" dataDxfId="81"/>
+    <tableColumn id="7" xr3:uid="{0FAD1ACC-432E-462C-8B89-71540710BCB5}" name="FixVersion" dataDxfId="80">
       <calculatedColumnFormula>Config!$G$4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="28" xr3:uid="{07F3030C-7187-4B16-BBDB-798304851975}" name="Assignee.Name" dataDxfId="47"/>
-    <tableColumn id="8" xr3:uid="{8C7FB8DB-A85B-4189-93D8-0F0D4EEEF81B}" name="Component" dataDxfId="46"/>
-    <tableColumn id="9" xr3:uid="{DC5101A8-1204-44D2-BC2C-FEE1A4EFE7C1}" name="Sprint Name" dataDxfId="45"/>
-    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="44"/>
-    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="43"/>
-    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="42"/>
-    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="41"/>
-    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="40">
+    <tableColumn id="28" xr3:uid="{07F3030C-7187-4B16-BBDB-798304851975}" name="Assignee.Name" dataDxfId="79"/>
+    <tableColumn id="8" xr3:uid="{8C7FB8DB-A85B-4189-93D8-0F0D4EEEF81B}" name="Component" dataDxfId="78"/>
+    <tableColumn id="9" xr3:uid="{DC5101A8-1204-44D2-BC2C-FEE1A4EFE7C1}" name="Sprint Name" dataDxfId="77"/>
+    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="76"/>
+    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="75"/>
+    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="74"/>
+    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="73"/>
+    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="72">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[IssueType]]="Epic",JiraDataset[[#This Row],[Summary]],"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="27" xr3:uid="{911C8FDC-5528-43FC-BDF4-D4761F03C0E5}" name="Child-Issue" dataDxfId="39"/>
-    <tableColumn id="41" xr3:uid="{AB248E07-9BFA-42CC-BC41-B4234F677BFB}" name="Child-Issue1" dataDxfId="38"/>
-    <tableColumn id="29" xr3:uid="{89D12135-F3E3-4253-844F-1B9A54169953}" name="Child-Issue2" dataDxfId="37"/>
-    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="36"/>
-    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="35"/>
-    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="34"/>
-    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="33"/>
-    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="32"/>
-    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="31"/>
-    <tableColumn id="18" xr3:uid="{16B98070-7F8A-4FC7-AD99-EA81D0BD26AB}" name="Labels6" dataDxfId="30"/>
-    <tableColumn id="19" xr3:uid="{016EAEF4-8EA9-408B-9F1A-ECFB17E81C77}" name="Labels7" dataDxfId="29"/>
-    <tableColumn id="26" xr3:uid="{8263F9EC-BF0A-46F7-BA83-6083A4262B91}" name="Labels8" dataDxfId="28"/>
-    <tableColumn id="20" xr3:uid="{389B11C5-1B22-48C0-BCA2-72F050425FA1}" name="Labels9" dataDxfId="27"/>
-    <tableColumn id="25" xr3:uid="{AE95F8A2-F7F0-4985-9AE6-4201B9792775}" name="Labels10" dataDxfId="26"/>
-    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="25">
+    <tableColumn id="27" xr3:uid="{911C8FDC-5528-43FC-BDF4-D4761F03C0E5}" name="Child-Issue" dataDxfId="71"/>
+    <tableColumn id="41" xr3:uid="{AB248E07-9BFA-42CC-BC41-B4234F677BFB}" name="Child-Issue1" dataDxfId="70"/>
+    <tableColumn id="29" xr3:uid="{89D12135-F3E3-4253-844F-1B9A54169953}" name="Child-Issue2" dataDxfId="69"/>
+    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="68"/>
+    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="67"/>
+    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="66"/>
+    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="65"/>
+    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="64"/>
+    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="63"/>
+    <tableColumn id="18" xr3:uid="{16B98070-7F8A-4FC7-AD99-EA81D0BD26AB}" name="Labels6" dataDxfId="62"/>
+    <tableColumn id="19" xr3:uid="{016EAEF4-8EA9-408B-9F1A-ECFB17E81C77}" name="Labels7" dataDxfId="61"/>
+    <tableColumn id="26" xr3:uid="{8263F9EC-BF0A-46F7-BA83-6083A4262B91}" name="Labels8" dataDxfId="60"/>
+    <tableColumn id="20" xr3:uid="{389B11C5-1B22-48C0-BCA2-72F050425FA1}" name="Labels9" dataDxfId="59"/>
+    <tableColumn id="25" xr3:uid="{AE95F8A2-F7F0-4985-9AE6-4201B9792775}" name="Labels10" dataDxfId="58"/>
+    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="57">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], Config!$D$4:$E$9, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="24">
+    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="56">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="23">
+    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="55">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Feature Pod Label", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="22">
+    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="54">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], Config!$A$4:$B$24, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="21">
+    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="53">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Project Key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="20">
+    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="52">
       <calculatedColumnFormula array="1">IF(
   JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
   "",
@@ -1392,7 +1688,7 @@
   )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="19">
+    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="51">
       <calculatedColumnFormula array="1">IFERROR(
     _xlfn.IFS(
         JiraDataset[[#This Row],[IssueType]] = cfg_type_comment,"SKIP",
@@ -1402,7 +1698,7 @@
     cfg_type_workitem
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="18"/>
+    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="50"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1442,7 +1738,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}" name="CfgPriorities" displayName="CfgPriorities" ref="O3:O9" totalsRowShown="0">
   <autoFilter ref="O3:O9" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="17"/>
+    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="49"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1476,7 +1772,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{D4E1611F-A2CF-465D-A219-1759EA66687D}" name="Name"/>
     <tableColumn id="2" xr3:uid="{174D0D86-B1AA-4BF7-AC91-FCACFC898851}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Remark" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Remark" dataDxfId="48"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1809,43 +2105,43 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F73058B-F76D-4AAE-8108-6C4469E9D8B5}">
-  <dimension ref="A1:AK3"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AK5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.7109375" customWidth="1"/>
-    <col min="4" max="4" width="11.85546875" hidden="1" customWidth="1"/>
+    <col min="1" max="2" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.6640625" customWidth="1"/>
+    <col min="4" max="4" width="11.83203125" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="33" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="46.28515625" customWidth="1"/>
-    <col min="7" max="7" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.5703125" customWidth="1"/>
+    <col min="6" max="6" width="46.33203125" customWidth="1"/>
+    <col min="7" max="7" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.5" customWidth="1"/>
     <col min="9" max="9" width="14" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.28515625" customWidth="1"/>
-    <col min="13" max="13" width="14.42578125" customWidth="1"/>
-    <col min="14" max="14" width="14.28515625" customWidth="1"/>
+    <col min="10" max="11" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.33203125" customWidth="1"/>
+    <col min="13" max="13" width="14.5" customWidth="1"/>
+    <col min="14" max="14" width="14.33203125" customWidth="1"/>
     <col min="15" max="15" width="0" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="22.28515625" hidden="1" customWidth="1"/>
-    <col min="17" max="17" width="12.85546875" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="12.42578125" customWidth="1"/>
-    <col min="19" max="19" width="15.5703125" customWidth="1"/>
-    <col min="20" max="20" width="12.85546875" customWidth="1"/>
+    <col min="16" max="16" width="22.33203125" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="12.83203125" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="12.5" customWidth="1"/>
+    <col min="19" max="19" width="15.5" customWidth="1"/>
+    <col min="20" max="20" width="12.83203125" customWidth="1"/>
     <col min="21" max="21" width="10" customWidth="1"/>
     <col min="22" max="22" width="10" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="10" customWidth="1"/>
-    <col min="24" max="24" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="10.1640625" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="10" customWidth="1" outlineLevel="1"/>
     <col min="31" max="31" width="10" customWidth="1"/>
-    <col min="32" max="32" width="8.7109375" customWidth="1" outlineLevel="1"/>
-    <col min="33" max="34" width="13.140625" customWidth="1" outlineLevel="1"/>
-    <col min="35" max="35" width="11.42578125" customWidth="1" outlineLevel="1"/>
-    <col min="36" max="37" width="13.7109375" customWidth="1" outlineLevel="1"/>
-    <col min="38" max="38" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="18.7109375" customWidth="1"/>
-    <col min="41" max="41" width="87.28515625" customWidth="1"/>
+    <col min="32" max="32" width="8.6640625" customWidth="1" outlineLevel="1"/>
+    <col min="33" max="34" width="13.1640625" customWidth="1" outlineLevel="1"/>
+    <col min="35" max="35" width="11.5" customWidth="1" outlineLevel="1"/>
+    <col min="36" max="37" width="13.6640625" customWidth="1" outlineLevel="1"/>
+    <col min="38" max="38" width="36.5" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="18.6640625" customWidth="1"/>
+    <col min="41" max="41" width="87.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>1</v>
       </c>
@@ -1880,7 +2176,7 @@
         <v>10</v>
       </c>
       <c r="L1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M1" s="3" t="s">
         <v>11</v>
@@ -1955,7 +2251,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
         <v>33</v>
@@ -1972,7 +2268,7 @@
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
       <c r="J2" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="K2" s="3">
         <v>1</v>
@@ -2047,7 +2343,7 @@
       </c>
       <c r="AJ2" s="3"/>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>53</v>
       </c>
@@ -2055,26 +2351,26 @@
         <v>42</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>58</v>
+        <v>105</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>47</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="K3" s="3">
         <v>2</v>
@@ -2113,7 +2409,7 @@
       </c>
       <c r="AF3" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], Config!$A$4:$B$24, 2, FALSE), ""))</f>
-        <v/>
+        <v>712020:e4e815aa-df03-418a-9760-3e70901b6ec5</v>
       </c>
       <c r="AG3" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Project Key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
@@ -2149,71 +2445,245 @@
       </c>
       <c r="AJ3" s="3"/>
     </row>
+    <row r="4" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A4" s="13"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="14" t="str">
+        <f>Config!$G$4</f>
+        <v>JITTP Version 1</v>
+      </c>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="15"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="15" t="str">
+        <f>IF(JiraDataset[[#This Row],[IssueType]]="Epic",JiraDataset[[#This Row],[Summary]],"")</f>
+        <v/>
+      </c>
+      <c r="O4" s="3"/>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3"/>
+      <c r="T4" s="3"/>
+      <c r="U4" s="3"/>
+      <c r="V4" s="3"/>
+      <c r="W4" s="3"/>
+      <c r="X4" s="3"/>
+      <c r="Y4" s="3"/>
+      <c r="Z4" s="3"/>
+      <c r="AA4" s="3"/>
+      <c r="AB4" s="3"/>
+      <c r="AC4" s="15" t="str">
+        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], Config!$D$4:$E$9, 2, FALSE), ""))</f>
+        <v/>
+      </c>
+      <c r="AD4" s="15" t="str">
+        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
+        <v>imported</v>
+      </c>
+      <c r="AE4" s="8" t="str">
+        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Feature Pod Label", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
+        <v>pod_test</v>
+      </c>
+      <c r="AF4" s="15" t="str">
+        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], Config!$A$4:$B$24, 2, FALSE), ""))</f>
+        <v/>
+      </c>
+      <c r="AG4" s="15" t="str">
+        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Project Key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
+        <v>JITTP2</v>
+      </c>
+      <c r="AH4" s="15" t="str" cm="1">
+        <f t="array" ref="AH4">IF(
+  JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
+  "",
+  _xlfn.LET(
+    _xlpm.p, _xlfn.TEXTSPLIT(JiraDataset[[#This Row],[Estimate]], " "),
+    _xlpm.getVal, _xlfn.LAMBDA(_xlpm.u, IFERROR(VALUE(LEFT(_xlfn._xlws.FILTER(_xlpm.p, RIGHT(_xlpm.p,1)=_xlpm.u), LEN(_xlfn._xlws.FILTER(_xlpm.p, RIGHT(_xlpm.p,1)=_xlpm.u))-1)), 0)),
+    _xlpm.w, _xlpm.getVal("w"),
+    _xlpm.d, _xlpm.getVal("d"),
+    _xlpm.h, _xlpm.getVal("h"),
+    _xlpm.m, _xlpm.getVal("m"),
+    _xlpm.seconds, _xlpm.w*144000 + _xlpm.d*28800 + _xlpm.h*3600 + _xlpm.m*60,
+    IF(_xlpm.seconds=0, "", _xlpm.seconds*60)
+  )
+)</f>
+        <v/>
+      </c>
+      <c r="AI4" s="15" t="str" cm="1">
+        <f t="array" ref="AI4">IFERROR(
+    _xlfn.IFS(
+        JiraDataset[[#This Row],[IssueType]] = cfg_type_comment,"SKIP",
+        JiraDataset[[#This Row],[IssueType]] = cfg_type_skip,"SKIP",
+        JiraDataset[[#This Row],[IssueType]] = cfg_type_note,"SKIP"
+    ),
+    cfg_type_workitem
+)</f>
+        <v>WorkItem</v>
+      </c>
+      <c r="AJ4" s="3"/>
+    </row>
+    <row r="5" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A5" s="13"/>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="14" t="str">
+        <f>Config!$G$4</f>
+        <v>JITTP Version 1</v>
+      </c>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="L5" s="15"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="15" t="str">
+        <f>IF(JiraDataset[[#This Row],[IssueType]]="Epic",JiraDataset[[#This Row],[Summary]],"")</f>
+        <v/>
+      </c>
+      <c r="O5" s="3"/>
+      <c r="P5" s="3"/>
+      <c r="Q5" s="3"/>
+      <c r="R5" s="3"/>
+      <c r="S5" s="3"/>
+      <c r="T5" s="3"/>
+      <c r="U5" s="3"/>
+      <c r="V5" s="3"/>
+      <c r="W5" s="3"/>
+      <c r="X5" s="3"/>
+      <c r="Y5" s="3"/>
+      <c r="Z5" s="3"/>
+      <c r="AA5" s="3"/>
+      <c r="AB5" s="3"/>
+      <c r="AC5" s="15" t="str">
+        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], Config!$D$4:$E$9, 2, FALSE), ""))</f>
+        <v/>
+      </c>
+      <c r="AD5" s="15" t="str">
+        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
+        <v>imported</v>
+      </c>
+      <c r="AE5" s="8" t="str">
+        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Feature Pod Label", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
+        <v>pod_test</v>
+      </c>
+      <c r="AF5" s="15" t="str">
+        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], Config!$A$4:$B$24, 2, FALSE), ""))</f>
+        <v/>
+      </c>
+      <c r="AG5" s="15" t="str">
+        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Project Key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
+        <v>JITTP2</v>
+      </c>
+      <c r="AH5" s="15" t="str" cm="1">
+        <f t="array" ref="AH5">IF(
+  JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
+  "",
+  _xlfn.LET(
+    _xlpm.p, _xlfn.TEXTSPLIT(JiraDataset[[#This Row],[Estimate]], " "),
+    _xlpm.getVal, _xlfn.LAMBDA(_xlpm.u, IFERROR(VALUE(LEFT(_xlfn._xlws.FILTER(_xlpm.p, RIGHT(_xlpm.p,1)=_xlpm.u), LEN(_xlfn._xlws.FILTER(_xlpm.p, RIGHT(_xlpm.p,1)=_xlpm.u))-1)), 0)),
+    _xlpm.w, _xlpm.getVal("w"),
+    _xlpm.d, _xlpm.getVal("d"),
+    _xlpm.h, _xlpm.getVal("h"),
+    _xlpm.m, _xlpm.getVal("m"),
+    _xlpm.seconds, _xlpm.w*144000 + _xlpm.d*28800 + _xlpm.h*3600 + _xlpm.m*60,
+    IF(_xlpm.seconds=0, "", _xlpm.seconds*60)
+  )
+)</f>
+        <v/>
+      </c>
+      <c r="AI5" s="15" t="str" cm="1">
+        <f t="array" ref="AI5">IFERROR(
+    _xlfn.IFS(
+        JiraDataset[[#This Row],[IssueType]] = cfg_type_comment,"SKIP",
+        JiraDataset[[#This Row],[IssueType]] = cfg_type_skip,"SKIP",
+        JiraDataset[[#This Row],[IssueType]] = cfg_type_note,"SKIP"
+    ),
+    cfg_type_workitem
+)</f>
+        <v>WorkItem</v>
+      </c>
+      <c r="AJ5" s="3"/>
+    </row>
   </sheetData>
   <protectedRanges>
     <protectedRange sqref="A1:A1048576 D4:N1048576 P4:AD1048576 C1:AB3" name="User Input"/>
     <protectedRange algorithmName="SHA-512" hashValue="tpheD+JLADkhiyalt6vInlMwkILPZx4PVQN/k2vmwjOBdYUuHaXCrwtObHeFz5dJh9f853O84pZ1Rn9Ujz33+A==" saltValue="9ir5NB4CJc/69S/Eh84/mA==" spinCount="100000" sqref="AC1:AI3 AE4:AK1048576" name="Computed values"/>
   </protectedRanges>
   <phoneticPr fontId="18" type="noConversion"/>
-  <conditionalFormatting sqref="A2:A3 C2:C3">
-    <cfRule type="containsText" dxfId="15" priority="429" operator="containsText" text="blocker">
+  <conditionalFormatting sqref="A2:A5 C2:C5">
+    <cfRule type="containsText" dxfId="47" priority="429" operator="containsText" text="blocker">
       <formula>NOT(ISERROR(SEARCH("blocker",A2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="430" operator="containsText" text="critical">
+    <cfRule type="containsText" dxfId="46" priority="430" operator="containsText" text="critical">
       <formula>NOT(ISERROR(SEARCH("critical",A2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="13" priority="431" operator="containsText" text="High">
+    <cfRule type="containsText" dxfId="45" priority="431" operator="containsText" text="High">
       <formula>NOT(ISERROR(SEARCH("High",A2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="12" priority="432" operator="containsText" text="Medium">
+    <cfRule type="containsText" dxfId="44" priority="432" operator="containsText" text="Medium">
       <formula>NOT(ISERROR(SEARCH("Medium",A2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:A3">
-    <cfRule type="containsBlanks" dxfId="11" priority="493">
+  <conditionalFormatting sqref="A2:A5">
+    <cfRule type="containsBlanks" dxfId="43" priority="493">
       <formula>LEN(TRIM(A2))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:AJ3">
-    <cfRule type="expression" dxfId="10" priority="409" stopIfTrue="1">
+  <conditionalFormatting sqref="A2:AJ5">
+    <cfRule type="expression" dxfId="42" priority="409" stopIfTrue="1">
       <formula>$B2=cfg_type_comment</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="410">
+    <cfRule type="expression" dxfId="41" priority="410">
       <formula>$B2=cfg_type_skip</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="411">
+    <cfRule type="expression" dxfId="40" priority="411">
       <formula>$B2=cfg_type_note</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2:B3">
-    <cfRule type="containsText" dxfId="7" priority="413" operator="containsText" text="epic">
+  <conditionalFormatting sqref="B2:B5">
+    <cfRule type="containsText" dxfId="39" priority="413" operator="containsText" text="epic">
       <formula>NOT(ISERROR(SEARCH("epic",B2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="427" operator="containsText" text="story">
+    <cfRule type="containsText" dxfId="38" priority="427" operator="containsText" text="story">
       <formula>NOT(ISERROR(SEARCH("story",B2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="5" priority="433" operator="containsText" text="task">
+    <cfRule type="containsText" dxfId="37" priority="433" operator="containsText" text="task">
       <formula>NOT(ISERROR(SEARCH("task",B2)))</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="4" priority="492">
+    <cfRule type="containsBlanks" dxfId="36" priority="492">
       <formula>LEN(TRIM(B2))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2:AJ3">
-    <cfRule type="expression" dxfId="3" priority="1">
+  <conditionalFormatting sqref="B2:AJ5">
+    <cfRule type="expression" dxfId="35" priority="1">
       <formula>$B2="Epic"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="2">
+    <cfRule type="expression" dxfId="34" priority="2">
       <formula>$B2="Story"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C3">
-    <cfRule type="containsBlanks" dxfId="1" priority="494">
+  <conditionalFormatting sqref="C2:C5">
+    <cfRule type="containsBlanks" dxfId="33" priority="494">
       <formula>LEN(TRIM(C2))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:L3">
-    <cfRule type="containsBlanks" dxfId="0" priority="412">
+  <conditionalFormatting sqref="K2:L5">
+    <cfRule type="containsBlanks" dxfId="32" priority="412">
       <formula>LEN(TRIM(K2))=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2222,37 +2692,37 @@
       <formula1>1</formula1>
       <formula2>1000</formula2>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="J2:J3" xr:uid="{386E3B68-2486-4DDE-BEB1-45F897521149}"/>
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" promptTitle="Warning" prompt="This field should be the Issue ID or Issue Key of the child tasks. (upstream linkage is not possible)._x000a__x000a__x000a_To link Epics and Stories, use the Epic Link from the Story Issue." sqref="O2:Q3" xr:uid="{D7BD960D-9CEA-4120-B2E3-2AE0D4661093}">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="J2:J5" xr:uid="{386E3B68-2486-4DDE-BEB1-45F897521149}"/>
+    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" promptTitle="Warning" prompt="This field should be the Issue ID or Issue Key of the child tasks. (upstream linkage is not possible)._x000a__x000a__x000a_To link Epics and Stories, use the Epic Link from the Story Issue." sqref="O2:Q5" xr:uid="{D7BD960D-9CEA-4120-B2E3-2AE0D4661093}">
       <formula1>1</formula1>
       <formula2>1000</formula2>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Note" prompt="The content of this column will be ignored during the Jira import." sqref="AJ2:AJ3" xr:uid="{2DA3EDB6-7635-4349-8860-B614B5B71275}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Permissions" prompt="Updating Existing Issues requires global admin permissions" sqref="D2:D3" xr:uid="{D5E4A4BB-53C8-42DF-9B52-F5E00AC6407B}"/>
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" promptTitle="Warning" prompt="Use the Issue ID value to link this work item to an Epic_x000a__x000a_Story Issues are not Child-Issues and should have Epic Link instead. " sqref="M2:M3" xr:uid="{16C14239-D6AA-4935-8809-57760481D8F1}">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Note" prompt="The content of this column will be ignored during the Jira import." sqref="AJ2:AJ5" xr:uid="{2DA3EDB6-7635-4349-8860-B614B5B71275}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Permissions" prompt="Updating Existing Issues requires global admin permissions" sqref="D2:D5" xr:uid="{D5E4A4BB-53C8-42DF-9B52-F5E00AC6407B}"/>
+    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" promptTitle="Warning" prompt="Use the Issue ID value to link this work item to an Epic_x000a__x000a_Story Issues are not Child-Issues and should have Epic Link instead. " sqref="M2:M5" xr:uid="{16C14239-D6AA-4935-8809-57760481D8F1}">
       <formula1>1</formula1>
       <formula2>1000</formula2>
     </dataValidation>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="It must be a number (integer). This reference is only used during the import process." sqref="K1" xr:uid="{9C637146-F2E3-4D08-87A8-F70FD358E47E}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Use the Issue ID value to link this work item to an Epic_x000a__x000a_Story Issues are not Child-Issues and should have Epic Link instead. " sqref="M1" xr:uid="{A61138FD-C2B2-49D2-810B-69EAE2230B73}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="This field should be the Issue ID or Issue Key of the child tasks. (upstream linkage is not possible)._x000a__x000a__x000a_To link Epics and Stories, use the Epic Link from the Story Issue." sqref="O1:Q1" xr:uid="{BE6B7503-A11A-4130-9D63-988F0CFED80E}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="AUTOMATIC FIELD" prompt="Do not manually edit these!" sqref="AF2:AH3 AC2:AC3 AF1:AH1" xr:uid="{893DA5FE-9FD0-4D28-BBD0-3D7AEDECEACB}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="H2:H3" xr:uid="{65EDED96-6789-400B-B504-6BC3F5A79E70}">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="AUTOMATIC FIELD" prompt="Do not manually edit these!" sqref="AC2:AC5 AF1:AH5" xr:uid="{893DA5FE-9FD0-4D28-BBD0-3D7AEDECEACB}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="H2:H5" xr:uid="{65EDED96-6789-400B-B504-6BC3F5A79E70}">
       <formula1>INDIRECT("CfgComponents[Component.Name]")</formula1>
     </dataValidation>
-    <dataValidation type="list" errorStyle="warning" showErrorMessage="1" error="must be a valid fixversion" sqref="G2:G3" xr:uid="{44FDC20A-8BF5-49B5-9D2C-3A1FE5A7D835}">
+    <dataValidation type="list" errorStyle="warning" showErrorMessage="1" error="must be a valid fixversion" sqref="G2:G5" xr:uid="{44FDC20A-8BF5-49B5-9D2C-3A1FE5A7D835}">
       <formula1>INDIRECT("CfgAssignees[Asssignee.Name]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="I2:I3" xr:uid="{A898E2E7-BC45-4B88-BA1E-4AAA377361D4}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="I2:I5" xr:uid="{A898E2E7-BC45-4B88-BA1E-4AAA377361D4}">
       <formula1>INDIRECT("CfgSprints[Sprint.Name]")</formula1>
     </dataValidation>
     <dataValidation allowBlank="1" showErrorMessage="1" promptTitle="Warning" prompt="Field only used for Epic Issues, so they can be referenced in Story Issues via the Epic Link field.," sqref="N2:N3 L2:L3" xr:uid="{541AD292-0123-4B65-9663-081991FDF0C1}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Field only used for Epic Issues, so they can be referenced in Story Issues via the Epic Link field.," sqref="L1" xr:uid="{64C73155-DEE7-497D-8A98-01E54655ACA8}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="It must be a number (integer) or the Work Item key. This reference is only used during the import process to set the parent." sqref="L1" xr:uid="{8A2BE248-5762-43AD-9C47-C5A92A2E2357}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Field only used for Epic work item, so they can be referenced in Story work items via the Epic Link field. _x000a_DC Only" sqref="N1" xr:uid="{E8F6E005-1F9B-40F3-B24C-E2A3D286C532}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="Creation Marker (Config Sheet)" prompt="Do not manually edit these!" sqref="AD1:AD3" xr:uid="{412C516D-E091-4DDD-9C14-C33AC653C143}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="Feature Pod Label (Config Sheet)" prompt="Do not manually edit these!" sqref="AE1:AE3" xr:uid="{D2234141-379F-4413-AB08-6835BD9FF967}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="AUTOMATIC FIELD" prompt="Do not manually edit these! SKIP types won't be imported into Jira" sqref="AI1:AI3" xr:uid="{5A336857-7D14-4900-8734-BED680BE5154}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="Creation Marker (Config Sheet)" prompt="Do not manually edit these!" sqref="AD1:AD5" xr:uid="{412C516D-E091-4DDD-9C14-C33AC653C143}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="Feature Pod Label (Config Sheet)" prompt="Do not manually edit these!" sqref="AE1:AE5" xr:uid="{D2234141-379F-4413-AB08-6835BD9FF967}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="AUTOMATIC FIELD" prompt="Do not manually edit these! SKIP types won't be imported into Jira" sqref="AI1:AI5" xr:uid="{5A336857-7D14-4900-8734-BED680BE5154}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2266,19 +2736,19 @@
           <x14:formula1>
             <xm:f>Config!$O$4:$O$10</xm:f>
           </x14:formula1>
-          <xm:sqref>A2:A3</xm:sqref>
+          <xm:sqref>A2:A5</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Issue Type" xr:uid="{28BF52BF-C0B0-4D22-B02F-F1408D5A055B}">
           <x14:formula1>
             <xm:f>Config!$U$4:$U$33</xm:f>
           </x14:formula1>
-          <xm:sqref>B2:B3</xm:sqref>
+          <xm:sqref>B2:B5</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" xr:uid="{7708D6E2-1D6B-41D8-A9EE-0E87219BA8EA}">
           <x14:formula1>
             <xm:f>Config!$G$4:$G$8</xm:f>
           </x14:formula1>
-          <xm:sqref>F2:F3</xm:sqref>
+          <xm:sqref>F2:F5</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2289,90 +2759,90 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2D54512-1380-4F02-BB23-352387C91232}">
   <dimension ref="A1:V21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="29.7109375" customWidth="1"/>
+    <col min="1" max="1" width="29.6640625" customWidth="1"/>
     <col min="2" max="2" width="49" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.28515625" customWidth="1"/>
-    <col min="4" max="5" width="18.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.28515625" customWidth="1"/>
-    <col min="7" max="7" width="18.5703125" customWidth="1"/>
-    <col min="8" max="8" width="4.28515625" customWidth="1"/>
-    <col min="9" max="9" width="19.140625" customWidth="1"/>
-    <col min="10" max="10" width="4.28515625" customWidth="1"/>
-    <col min="11" max="11" width="18.5703125" customWidth="1"/>
-    <col min="12" max="12" width="4.28515625" customWidth="1"/>
-    <col min="13" max="13" width="17.5703125" customWidth="1"/>
-    <col min="14" max="14" width="4.28515625" customWidth="1"/>
-    <col min="15" max="15" width="18.7109375" customWidth="1"/>
-    <col min="16" max="16" width="4.28515625" customWidth="1"/>
-    <col min="17" max="18" width="18.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.33203125" customWidth="1"/>
+    <col min="4" max="5" width="18.6640625" customWidth="1"/>
+    <col min="6" max="6" width="4.33203125" customWidth="1"/>
+    <col min="7" max="7" width="18.5" customWidth="1"/>
+    <col min="8" max="8" width="4.33203125" customWidth="1"/>
+    <col min="9" max="9" width="19.1640625" customWidth="1"/>
+    <col min="10" max="10" width="4.33203125" customWidth="1"/>
+    <col min="11" max="11" width="18.5" customWidth="1"/>
+    <col min="12" max="12" width="4.33203125" customWidth="1"/>
+    <col min="13" max="13" width="17.5" customWidth="1"/>
+    <col min="14" max="14" width="4.33203125" customWidth="1"/>
+    <col min="15" max="15" width="18.6640625" customWidth="1"/>
+    <col min="16" max="16" width="4.33203125" customWidth="1"/>
+    <col min="17" max="18" width="18.6640625" customWidth="1"/>
     <col min="19" max="19" width="35" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="22.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:22" ht="22" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B1" s="11"/>
       <c r="D1" s="11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E1" s="11"/>
       <c r="G1" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K1" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="M1" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="O1" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="M1" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="O1" s="6" t="s">
-        <v>60</v>
-      </c>
       <c r="Q1" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="R1" s="11"/>
       <c r="S1" s="11"/>
       <c r="U1" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="7"/>
       <c r="D2" s="12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E2" s="12"/>
       <c r="F2" s="7"/>
       <c r="G2" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H2" s="10"/>
       <c r="I2" s="10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J2" s="10"/>
       <c r="K2" s="12" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="L2" s="12"/>
       <c r="M2" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="N2" s="9"/>
       <c r="O2" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="P2" s="10"/>
       <c r="Q2" s="12"/>
@@ -2380,54 +2850,54 @@
       <c r="S2" s="9"/>
       <c r="T2" s="7"/>
       <c r="U2" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="V2" s="9"/>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" t="s">
         <v>65</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D3" t="s">
         <v>66</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>67</v>
       </c>
-      <c r="E3" t="s">
-        <v>68</v>
-      </c>
       <c r="G3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="K3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O3" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>60</v>
+      </c>
+      <c r="R3" t="s">
+        <v>61</v>
+      </c>
+      <c r="S3" t="s">
+        <v>77</v>
+      </c>
+      <c r="U3" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="Q3" t="s">
-        <v>61</v>
-      </c>
-      <c r="R3" t="s">
-        <v>62</v>
-      </c>
-      <c r="S3" t="s">
-        <v>78</v>
-      </c>
-      <c r="U3" s="5" t="s">
-        <v>73</v>
-      </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B4" t="s">
         <v>50</v>
@@ -2439,10 +2909,10 @@
         <v>1</v>
       </c>
       <c r="G4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K4" t="s">
         <v>39</v>
@@ -2457,7 +2927,7 @@
         <v>31</v>
       </c>
       <c r="R4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="S4" s="7"/>
       <c r="U4" t="str" cm="1">
@@ -2465,9 +2935,9 @@
         <v>Story</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B5" t="s">
         <v>51</v>
@@ -2479,10 +2949,10 @@
         <v>2</v>
       </c>
       <c r="G5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="K5" t="s">
         <v>37</v>
@@ -2500,25 +2970,25 @@
         <v>40</v>
       </c>
       <c r="S5" s="7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="U5" t="str">
         <f ca="1"/>
         <v>Task</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B6" t="s">
         <v>52</v>
       </c>
       <c r="G6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K6" t="s">
         <v>41</v>
@@ -2533,21 +3003,21 @@
         <v>49</v>
       </c>
       <c r="R6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="S6" s="7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="U6" t="str">
         <f ca="1"/>
         <v>Bug</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="I7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="K7" t="s">
         <v>42</v>
@@ -2563,11 +3033,11 @@
         <v>Epic</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="I8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O8" s="1" t="s">
         <v>55</v>
@@ -2577,11 +3047,11 @@
         <v>Comment</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="I9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="O9" s="1" t="s">
         <v>56</v>
@@ -2591,18 +3061,18 @@
         <v>Skip</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="I10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="U10" t="str">
         <f ca="1"/>
         <v>Note</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
       <c r="U11" t="str">
@@ -2610,43 +3080,43 @@
         <v>WorkItem</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.2">
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
     </row>
-    <row r="19" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
     </row>
-    <row r="20" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
     </row>
-    <row r="21" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
     </row>
@@ -2677,6 +3147,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FB038601AF41D04A88A4BD446922F1A8" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e8d32171d27ae41230d53456f24efae5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c471fd26-9765-4fbe-b6fd-c17c1e55c974" xmlns:ns3="9df69692-83aa-4c55-88c1-62abad05f4fe" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f2fb84de5621acf32f385a2ba90fb29" ns2:_="" ns3:_="">
     <xsd:import namespace="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
@@ -2905,27 +3395,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FFE630F-6530-4863-AB67-8477539A0000}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
+    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2C983B91-58B3-4C2C-AC55-FFEC9F0DB5F6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2942,23 +3431,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FFE630F-6530-4863-AB67-8477539A0000}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
-    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Fix: Missing formulas in the import template
</commit_message>
<xml_diff>
--- a/resources/templates/ImportTemplate.xlsx
+++ b/resources/templates/ImportTemplate.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jules/Workdir/sources/jira-toolkit/resources/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tom_48_97\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8715B6CB-C258-0246-816F-293FA3525AAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CB533E1-F127-4B9B-ACDE-FE3A52926206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16820" yWindow="10420" windowWidth="17560" windowHeight="12420" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
+    <workbookView xWindow="1116" yWindow="1116" windowWidth="23040" windowHeight="13560" activeTab="1" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
   </bookViews>
   <sheets>
-    <sheet name="Dataset" sheetId="1" r:id="rId1"/>
+    <sheet name="Dataset2" sheetId="1" r:id="rId1"/>
     <sheet name="Config" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="110">
   <si>
     <t>IssueType</t>
   </si>
@@ -245,6 +245,9 @@
     <t>Creation Marker</t>
   </si>
   <si>
+    <t>JV</t>
+  </si>
+  <si>
     <t>Issue Type</t>
   </si>
   <si>
@@ -396,12 +399,6 @@
   </si>
   <si>
     <t>pod_test</t>
-  </si>
-  <si>
-    <t>tst</t>
-  </si>
-  <si>
-    <t>a</t>
   </si>
 </sst>
 </file>
@@ -925,7 +922,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -956,15 +953,6 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="16" applyAlignment="1">
       <alignment horizontal="left" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1011,291 +999,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="88">
-    <dxf>
-      <fill>
-        <patternFill patternType="darkUp"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDAF2D0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2CEEF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.89996032593768116"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <strike val="0"/>
-        <color theme="0" tint="-0.34998626667073579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFF9B1AB"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCC99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9999"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF99CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="darkUp"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDAF2D0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2CEEF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.89996032593768116"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <strike val="0"/>
-        <color theme="0" tint="-0.34998626667073579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFF9B1AB"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCC99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9999"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF99CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6699"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="56">
     <dxf>
       <fill>
         <patternFill patternType="darkUp"/>
@@ -1616,63 +1320,63 @@
 <file path=xl/namedSheetViews/namedSheetView1.xml><?xml version="1.0" encoding="utf-8"?>
 <namedSheetViews xmlns="http://schemas.microsoft.com/office/spreadsheetml/2019/namedsheetviews" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <namedSheetView name="View1" id="{77233F75-225A-4D7F-8A86-543E0A8C6E58}">
-    <nsvFilter filterId="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" ref="A1:AJ5" tableId="1"/>
+    <nsvFilter filterId="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" ref="A1:AJ3" tableId="1"/>
   </namedSheetView>
 </namedSheetViews>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" name="JiraDataset" displayName="JiraDataset" ref="A1:AJ5" totalsRowShown="0" headerRowDxfId="87" dataDxfId="86">
-  <autoFilter ref="A1:AJ5" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" name="JiraDataset" displayName="JiraDataset" ref="A1:AJ3" totalsRowShown="0" headerRowDxfId="55" dataDxfId="54">
+  <autoFilter ref="A1:AJ3" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}"/>
   <tableColumns count="36">
-    <tableColumn id="3" xr3:uid="{AF2EC907-349C-4651-852D-6E39C61E17FF}" name="Priority" dataDxfId="85"/>
-    <tableColumn id="2" xr3:uid="{E90C51F2-4386-421F-A3E4-E2CA9D43D396}" name="IssueType" dataDxfId="84"/>
-    <tableColumn id="1" xr3:uid="{BBAD373B-BA13-47E4-9F74-565F4D9E9680}" name="Summary" dataDxfId="83"/>
-    <tableColumn id="4" xr3:uid="{026E5B97-FAFC-4E46-860E-0B0C976B1148}" name="Issue Key" dataDxfId="82"/>
-    <tableColumn id="5" xr3:uid="{A2C262E8-D544-4669-99F1-151EDE081654}" name="Description" dataDxfId="81"/>
-    <tableColumn id="7" xr3:uid="{0FAD1ACC-432E-462C-8B89-71540710BCB5}" name="FixVersion" dataDxfId="80">
+    <tableColumn id="3" xr3:uid="{AF2EC907-349C-4651-852D-6E39C61E17FF}" name="Priority" dataDxfId="53"/>
+    <tableColumn id="2" xr3:uid="{E90C51F2-4386-421F-A3E4-E2CA9D43D396}" name="IssueType" dataDxfId="52"/>
+    <tableColumn id="1" xr3:uid="{BBAD373B-BA13-47E4-9F74-565F4D9E9680}" name="Summary" dataDxfId="51"/>
+    <tableColumn id="4" xr3:uid="{026E5B97-FAFC-4E46-860E-0B0C976B1148}" name="Issue Key" dataDxfId="50"/>
+    <tableColumn id="5" xr3:uid="{A2C262E8-D544-4669-99F1-151EDE081654}" name="Description" dataDxfId="49"/>
+    <tableColumn id="7" xr3:uid="{0FAD1ACC-432E-462C-8B89-71540710BCB5}" name="FixVersion" dataDxfId="48">
       <calculatedColumnFormula>Config!$G$4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="28" xr3:uid="{07F3030C-7187-4B16-BBDB-798304851975}" name="Assignee.Name" dataDxfId="79"/>
-    <tableColumn id="8" xr3:uid="{8C7FB8DB-A85B-4189-93D8-0F0D4EEEF81B}" name="Component" dataDxfId="78"/>
-    <tableColumn id="9" xr3:uid="{DC5101A8-1204-44D2-BC2C-FEE1A4EFE7C1}" name="Sprint Name" dataDxfId="77"/>
-    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="76"/>
-    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="75"/>
-    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="74"/>
-    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="73"/>
-    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="72">
+    <tableColumn id="28" xr3:uid="{07F3030C-7187-4B16-BBDB-798304851975}" name="Assignee.Name" dataDxfId="47"/>
+    <tableColumn id="8" xr3:uid="{8C7FB8DB-A85B-4189-93D8-0F0D4EEEF81B}" name="Component" dataDxfId="46"/>
+    <tableColumn id="9" xr3:uid="{DC5101A8-1204-44D2-BC2C-FEE1A4EFE7C1}" name="Sprint Name" dataDxfId="45"/>
+    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="44"/>
+    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="43"/>
+    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="42"/>
+    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="41"/>
+    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="40">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[IssueType]]="Epic",JiraDataset[[#This Row],[Summary]],"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="27" xr3:uid="{911C8FDC-5528-43FC-BDF4-D4761F03C0E5}" name="Child-Issue" dataDxfId="71"/>
-    <tableColumn id="41" xr3:uid="{AB248E07-9BFA-42CC-BC41-B4234F677BFB}" name="Child-Issue1" dataDxfId="70"/>
-    <tableColumn id="29" xr3:uid="{89D12135-F3E3-4253-844F-1B9A54169953}" name="Child-Issue2" dataDxfId="69"/>
-    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="68"/>
-    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="67"/>
-    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="66"/>
-    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="65"/>
-    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="64"/>
-    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="63"/>
-    <tableColumn id="18" xr3:uid="{16B98070-7F8A-4FC7-AD99-EA81D0BD26AB}" name="Labels6" dataDxfId="62"/>
-    <tableColumn id="19" xr3:uid="{016EAEF4-8EA9-408B-9F1A-ECFB17E81C77}" name="Labels7" dataDxfId="61"/>
-    <tableColumn id="26" xr3:uid="{8263F9EC-BF0A-46F7-BA83-6083A4262B91}" name="Labels8" dataDxfId="60"/>
-    <tableColumn id="20" xr3:uid="{389B11C5-1B22-48C0-BCA2-72F050425FA1}" name="Labels9" dataDxfId="59"/>
-    <tableColumn id="25" xr3:uid="{AE95F8A2-F7F0-4985-9AE6-4201B9792775}" name="Labels10" dataDxfId="58"/>
-    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="57">
+    <tableColumn id="27" xr3:uid="{911C8FDC-5528-43FC-BDF4-D4761F03C0E5}" name="Child-Issue" dataDxfId="39"/>
+    <tableColumn id="41" xr3:uid="{AB248E07-9BFA-42CC-BC41-B4234F677BFB}" name="Child-Issue1" dataDxfId="38"/>
+    <tableColumn id="29" xr3:uid="{89D12135-F3E3-4253-844F-1B9A54169953}" name="Child-Issue2" dataDxfId="37"/>
+    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="36"/>
+    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="35"/>
+    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="34"/>
+    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="33"/>
+    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="32"/>
+    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="31"/>
+    <tableColumn id="18" xr3:uid="{16B98070-7F8A-4FC7-AD99-EA81D0BD26AB}" name="Labels6" dataDxfId="30"/>
+    <tableColumn id="19" xr3:uid="{016EAEF4-8EA9-408B-9F1A-ECFB17E81C77}" name="Labels7" dataDxfId="29"/>
+    <tableColumn id="26" xr3:uid="{8263F9EC-BF0A-46F7-BA83-6083A4262B91}" name="Labels8" dataDxfId="28"/>
+    <tableColumn id="20" xr3:uid="{389B11C5-1B22-48C0-BCA2-72F050425FA1}" name="Labels9" dataDxfId="27"/>
+    <tableColumn id="25" xr3:uid="{AE95F8A2-F7F0-4985-9AE6-4201B9792775}" name="Labels10" dataDxfId="26"/>
+    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="25">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], Config!$D$4:$E$9, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="56">
+    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="24">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="55">
+    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="23">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Feature Pod Label", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="54">
+    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="22">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], Config!$A$4:$B$24, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="53">
+    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="21">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Project Key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="52">
+    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="20">
       <calculatedColumnFormula array="1">IF(
   JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
   "",
@@ -1688,7 +1392,7 @@
   )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="51">
+    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="19">
       <calculatedColumnFormula array="1">IFERROR(
     _xlfn.IFS(
         JiraDataset[[#This Row],[IssueType]] = cfg_type_comment,"SKIP",
@@ -1698,7 +1402,7 @@
     cfg_type_workitem
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="50"/>
+    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1738,7 +1442,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}" name="CfgPriorities" displayName="CfgPriorities" ref="O3:O9" totalsRowShown="0">
   <autoFilter ref="O3:O9" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="49"/>
+    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1772,7 +1476,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{D4E1611F-A2CF-465D-A219-1759EA66687D}" name="Name"/>
     <tableColumn id="2" xr3:uid="{174D0D86-B1AA-4BF7-AC91-FCACFC898851}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Remark" dataDxfId="48"/>
+    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Remark" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2105,43 +1809,43 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F73058B-F76D-4AAE-8108-6C4469E9D8B5}">
-  <dimension ref="A1:AK5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:AK3"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelCol="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="12.44140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="31.6640625" customWidth="1"/>
-    <col min="4" max="4" width="11.83203125" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="11.88671875" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="33" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="46.33203125" customWidth="1"/>
-    <col min="7" max="7" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.5" customWidth="1"/>
+    <col min="7" max="7" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.5546875" customWidth="1"/>
     <col min="9" max="9" width="14" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="14.44140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="14.33203125" customWidth="1"/>
-    <col min="13" max="13" width="14.5" customWidth="1"/>
+    <col min="13" max="13" width="14.44140625" customWidth="1"/>
     <col min="14" max="14" width="14.33203125" customWidth="1"/>
     <col min="15" max="15" width="0" hidden="1" customWidth="1"/>
     <col min="16" max="16" width="22.33203125" hidden="1" customWidth="1"/>
-    <col min="17" max="17" width="12.83203125" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="12.5" customWidth="1"/>
-    <col min="19" max="19" width="15.5" customWidth="1"/>
-    <col min="20" max="20" width="12.83203125" customWidth="1"/>
+    <col min="17" max="17" width="12.88671875" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="12.44140625" customWidth="1"/>
+    <col min="19" max="19" width="15.5546875" customWidth="1"/>
+    <col min="20" max="20" width="12.88671875" customWidth="1"/>
     <col min="21" max="21" width="10" customWidth="1"/>
     <col min="22" max="22" width="10" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="10" customWidth="1"/>
-    <col min="24" max="24" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="10.109375" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="10" customWidth="1" outlineLevel="1"/>
     <col min="31" max="31" width="10" customWidth="1"/>
     <col min="32" max="32" width="8.6640625" customWidth="1" outlineLevel="1"/>
-    <col min="33" max="34" width="13.1640625" customWidth="1" outlineLevel="1"/>
-    <col min="35" max="35" width="11.5" customWidth="1" outlineLevel="1"/>
+    <col min="33" max="34" width="13.109375" customWidth="1" outlineLevel="1"/>
+    <col min="35" max="35" width="11.44140625" customWidth="1" outlineLevel="1"/>
     <col min="36" max="37" width="13.6640625" customWidth="1" outlineLevel="1"/>
-    <col min="38" max="38" width="36.5" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="36.5546875" bestFit="1" customWidth="1"/>
     <col min="40" max="40" width="18.6640625" customWidth="1"/>
     <col min="41" max="41" width="87.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>1</v>
       </c>
@@ -2176,7 +1880,7 @@
         <v>10</v>
       </c>
       <c r="L1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="M1" s="3" t="s">
         <v>11</v>
@@ -2251,7 +1955,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
         <v>33</v>
@@ -2268,7 +1972,7 @@
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
       <c r="J2" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K2" s="3">
         <v>1</v>
@@ -2343,7 +2047,7 @@
       </c>
       <c r="AJ2" s="3"/>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>53</v>
       </c>
@@ -2351,26 +2055,26 @@
         <v>42</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>105</v>
+        <v>58</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>47</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="K3" s="3">
         <v>2</v>
@@ -2409,7 +2113,7 @@
       </c>
       <c r="AF3" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], Config!$A$4:$B$24, 2, FALSE), ""))</f>
-        <v>712020:e4e815aa-df03-418a-9760-3e70901b6ec5</v>
+        <v/>
       </c>
       <c r="AG3" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Project Key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
@@ -2445,245 +2149,71 @@
       </c>
       <c r="AJ3" s="3"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="A4" s="13"/>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="14" t="str">
-        <f>Config!$G$4</f>
-        <v>JITTP Version 1</v>
-      </c>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="15"/>
-      <c r="M4" s="3"/>
-      <c r="N4" s="15" t="str">
-        <f>IF(JiraDataset[[#This Row],[IssueType]]="Epic",JiraDataset[[#This Row],[Summary]],"")</f>
-        <v/>
-      </c>
-      <c r="O4" s="3"/>
-      <c r="P4" s="3"/>
-      <c r="Q4" s="3"/>
-      <c r="R4" s="3"/>
-      <c r="S4" s="3"/>
-      <c r="T4" s="3"/>
-      <c r="U4" s="3"/>
-      <c r="V4" s="3"/>
-      <c r="W4" s="3"/>
-      <c r="X4" s="3"/>
-      <c r="Y4" s="3"/>
-      <c r="Z4" s="3"/>
-      <c r="AA4" s="3"/>
-      <c r="AB4" s="3"/>
-      <c r="AC4" s="15" t="str">
-        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], Config!$D$4:$E$9, 2, FALSE), ""))</f>
-        <v/>
-      </c>
-      <c r="AD4" s="15" t="str">
-        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
-        <v>imported</v>
-      </c>
-      <c r="AE4" s="8" t="str">
-        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Feature Pod Label", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
-        <v>pod_test</v>
-      </c>
-      <c r="AF4" s="15" t="str">
-        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], Config!$A$4:$B$24, 2, FALSE), ""))</f>
-        <v/>
-      </c>
-      <c r="AG4" s="15" t="str">
-        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Project Key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
-        <v>JITTP2</v>
-      </c>
-      <c r="AH4" s="15" t="str" cm="1">
-        <f t="array" ref="AH4">IF(
-  JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
-  "",
-  _xlfn.LET(
-    _xlpm.p, _xlfn.TEXTSPLIT(JiraDataset[[#This Row],[Estimate]], " "),
-    _xlpm.getVal, _xlfn.LAMBDA(_xlpm.u, IFERROR(VALUE(LEFT(_xlfn._xlws.FILTER(_xlpm.p, RIGHT(_xlpm.p,1)=_xlpm.u), LEN(_xlfn._xlws.FILTER(_xlpm.p, RIGHT(_xlpm.p,1)=_xlpm.u))-1)), 0)),
-    _xlpm.w, _xlpm.getVal("w"),
-    _xlpm.d, _xlpm.getVal("d"),
-    _xlpm.h, _xlpm.getVal("h"),
-    _xlpm.m, _xlpm.getVal("m"),
-    _xlpm.seconds, _xlpm.w*144000 + _xlpm.d*28800 + _xlpm.h*3600 + _xlpm.m*60,
-    IF(_xlpm.seconds=0, "", _xlpm.seconds*60)
-  )
-)</f>
-        <v/>
-      </c>
-      <c r="AI4" s="15" t="str" cm="1">
-        <f t="array" ref="AI4">IFERROR(
-    _xlfn.IFS(
-        JiraDataset[[#This Row],[IssueType]] = cfg_type_comment,"SKIP",
-        JiraDataset[[#This Row],[IssueType]] = cfg_type_skip,"SKIP",
-        JiraDataset[[#This Row],[IssueType]] = cfg_type_note,"SKIP"
-    ),
-    cfg_type_workitem
-)</f>
-        <v>WorkItem</v>
-      </c>
-      <c r="AJ4" s="3"/>
-    </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="A5" s="13"/>
-      <c r="B5" s="13"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="14" t="str">
-        <f>Config!$G$4</f>
-        <v>JITTP Version 1</v>
-      </c>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="L5" s="15"/>
-      <c r="M5" s="3"/>
-      <c r="N5" s="15" t="str">
-        <f>IF(JiraDataset[[#This Row],[IssueType]]="Epic",JiraDataset[[#This Row],[Summary]],"")</f>
-        <v/>
-      </c>
-      <c r="O5" s="3"/>
-      <c r="P5" s="3"/>
-      <c r="Q5" s="3"/>
-      <c r="R5" s="3"/>
-      <c r="S5" s="3"/>
-      <c r="T5" s="3"/>
-      <c r="U5" s="3"/>
-      <c r="V5" s="3"/>
-      <c r="W5" s="3"/>
-      <c r="X5" s="3"/>
-      <c r="Y5" s="3"/>
-      <c r="Z5" s="3"/>
-      <c r="AA5" s="3"/>
-      <c r="AB5" s="3"/>
-      <c r="AC5" s="15" t="str">
-        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], Config!$D$4:$E$9, 2, FALSE), ""))</f>
-        <v/>
-      </c>
-      <c r="AD5" s="15" t="str">
-        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
-        <v>imported</v>
-      </c>
-      <c r="AE5" s="8" t="str">
-        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Feature Pod Label", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
-        <v>pod_test</v>
-      </c>
-      <c r="AF5" s="15" t="str">
-        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], Config!$A$4:$B$24, 2, FALSE), ""))</f>
-        <v/>
-      </c>
-      <c r="AG5" s="15" t="str">
-        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Project Key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
-        <v>JITTP2</v>
-      </c>
-      <c r="AH5" s="15" t="str" cm="1">
-        <f t="array" ref="AH5">IF(
-  JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
-  "",
-  _xlfn.LET(
-    _xlpm.p, _xlfn.TEXTSPLIT(JiraDataset[[#This Row],[Estimate]], " "),
-    _xlpm.getVal, _xlfn.LAMBDA(_xlpm.u, IFERROR(VALUE(LEFT(_xlfn._xlws.FILTER(_xlpm.p, RIGHT(_xlpm.p,1)=_xlpm.u), LEN(_xlfn._xlws.FILTER(_xlpm.p, RIGHT(_xlpm.p,1)=_xlpm.u))-1)), 0)),
-    _xlpm.w, _xlpm.getVal("w"),
-    _xlpm.d, _xlpm.getVal("d"),
-    _xlpm.h, _xlpm.getVal("h"),
-    _xlpm.m, _xlpm.getVal("m"),
-    _xlpm.seconds, _xlpm.w*144000 + _xlpm.d*28800 + _xlpm.h*3600 + _xlpm.m*60,
-    IF(_xlpm.seconds=0, "", _xlpm.seconds*60)
-  )
-)</f>
-        <v/>
-      </c>
-      <c r="AI5" s="15" t="str" cm="1">
-        <f t="array" ref="AI5">IFERROR(
-    _xlfn.IFS(
-        JiraDataset[[#This Row],[IssueType]] = cfg_type_comment,"SKIP",
-        JiraDataset[[#This Row],[IssueType]] = cfg_type_skip,"SKIP",
-        JiraDataset[[#This Row],[IssueType]] = cfg_type_note,"SKIP"
-    ),
-    cfg_type_workitem
-)</f>
-        <v>WorkItem</v>
-      </c>
-      <c r="AJ5" s="3"/>
-    </row>
   </sheetData>
   <protectedRanges>
     <protectedRange sqref="A1:A1048576 D4:N1048576 P4:AD1048576 C1:AB3" name="User Input"/>
     <protectedRange algorithmName="SHA-512" hashValue="tpheD+JLADkhiyalt6vInlMwkILPZx4PVQN/k2vmwjOBdYUuHaXCrwtObHeFz5dJh9f853O84pZ1Rn9Ujz33+A==" saltValue="9ir5NB4CJc/69S/Eh84/mA==" spinCount="100000" sqref="AC1:AI3 AE4:AK1048576" name="Computed values"/>
   </protectedRanges>
   <phoneticPr fontId="18" type="noConversion"/>
-  <conditionalFormatting sqref="A2:A5 C2:C5">
-    <cfRule type="containsText" dxfId="47" priority="429" operator="containsText" text="blocker">
+  <conditionalFormatting sqref="A2:A3 C2:C3">
+    <cfRule type="containsText" dxfId="15" priority="429" operator="containsText" text="blocker">
       <formula>NOT(ISERROR(SEARCH("blocker",A2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="46" priority="430" operator="containsText" text="critical">
+    <cfRule type="containsText" dxfId="14" priority="430" operator="containsText" text="critical">
       <formula>NOT(ISERROR(SEARCH("critical",A2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="45" priority="431" operator="containsText" text="High">
+    <cfRule type="containsText" dxfId="13" priority="431" operator="containsText" text="High">
       <formula>NOT(ISERROR(SEARCH("High",A2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="44" priority="432" operator="containsText" text="Medium">
+    <cfRule type="containsText" dxfId="12" priority="432" operator="containsText" text="Medium">
       <formula>NOT(ISERROR(SEARCH("Medium",A2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:A5">
-    <cfRule type="containsBlanks" dxfId="43" priority="493">
+  <conditionalFormatting sqref="A2:A3">
+    <cfRule type="containsBlanks" dxfId="11" priority="493">
       <formula>LEN(TRIM(A2))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:AJ5">
-    <cfRule type="expression" dxfId="42" priority="409" stopIfTrue="1">
+  <conditionalFormatting sqref="A2:AJ3">
+    <cfRule type="expression" dxfId="10" priority="409" stopIfTrue="1">
       <formula>$B2=cfg_type_comment</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="41" priority="410">
+    <cfRule type="expression" dxfId="9" priority="410">
       <formula>$B2=cfg_type_skip</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="40" priority="411">
+    <cfRule type="expression" dxfId="8" priority="411">
       <formula>$B2=cfg_type_note</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2:B5">
-    <cfRule type="containsText" dxfId="39" priority="413" operator="containsText" text="epic">
+  <conditionalFormatting sqref="B2:B3">
+    <cfRule type="containsText" dxfId="7" priority="413" operator="containsText" text="epic">
       <formula>NOT(ISERROR(SEARCH("epic",B2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="38" priority="427" operator="containsText" text="story">
+    <cfRule type="containsText" dxfId="6" priority="427" operator="containsText" text="story">
       <formula>NOT(ISERROR(SEARCH("story",B2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="37" priority="433" operator="containsText" text="task">
+    <cfRule type="containsText" dxfId="5" priority="433" operator="containsText" text="task">
       <formula>NOT(ISERROR(SEARCH("task",B2)))</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="36" priority="492">
+    <cfRule type="containsBlanks" dxfId="4" priority="492">
       <formula>LEN(TRIM(B2))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2:AJ5">
-    <cfRule type="expression" dxfId="35" priority="1">
+  <conditionalFormatting sqref="B2:AJ3">
+    <cfRule type="expression" dxfId="3" priority="1">
       <formula>$B2="Epic"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="34" priority="2">
+    <cfRule type="expression" dxfId="2" priority="2">
       <formula>$B2="Story"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C5">
-    <cfRule type="containsBlanks" dxfId="33" priority="494">
+  <conditionalFormatting sqref="C2:C3">
+    <cfRule type="containsBlanks" dxfId="1" priority="494">
       <formula>LEN(TRIM(C2))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:L5">
-    <cfRule type="containsBlanks" dxfId="32" priority="412">
+  <conditionalFormatting sqref="K2:L3">
+    <cfRule type="containsBlanks" dxfId="0" priority="412">
       <formula>LEN(TRIM(K2))=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2692,37 +2222,37 @@
       <formula1>1</formula1>
       <formula2>1000</formula2>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="J2:J5" xr:uid="{386E3B68-2486-4DDE-BEB1-45F897521149}"/>
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" promptTitle="Warning" prompt="This field should be the Issue ID or Issue Key of the child tasks. (upstream linkage is not possible)._x000a__x000a__x000a_To link Epics and Stories, use the Epic Link from the Story Issue." sqref="O2:Q5" xr:uid="{D7BD960D-9CEA-4120-B2E3-2AE0D4661093}">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="J2:J3" xr:uid="{386E3B68-2486-4DDE-BEB1-45F897521149}"/>
+    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" promptTitle="Warning" prompt="This field should be the Issue ID or Issue Key of the child tasks. (upstream linkage is not possible)._x000a__x000a__x000a_To link Epics and Stories, use the Epic Link from the Story Issue." sqref="O2:Q3" xr:uid="{D7BD960D-9CEA-4120-B2E3-2AE0D4661093}">
       <formula1>1</formula1>
       <formula2>1000</formula2>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Note" prompt="The content of this column will be ignored during the Jira import." sqref="AJ2:AJ5" xr:uid="{2DA3EDB6-7635-4349-8860-B614B5B71275}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Permissions" prompt="Updating Existing Issues requires global admin permissions" sqref="D2:D5" xr:uid="{D5E4A4BB-53C8-42DF-9B52-F5E00AC6407B}"/>
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" promptTitle="Warning" prompt="Use the Issue ID value to link this work item to an Epic_x000a__x000a_Story Issues are not Child-Issues and should have Epic Link instead. " sqref="M2:M5" xr:uid="{16C14239-D6AA-4935-8809-57760481D8F1}">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Note" prompt="The content of this column will be ignored during the Jira import." sqref="AJ2:AJ3" xr:uid="{2DA3EDB6-7635-4349-8860-B614B5B71275}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Permissions" prompt="Updating Existing Issues requires global admin permissions" sqref="D2:D3" xr:uid="{D5E4A4BB-53C8-42DF-9B52-F5E00AC6407B}"/>
+    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" promptTitle="Warning" prompt="Use the Issue ID value to link this work item to an Epic_x000a__x000a_Story Issues are not Child-Issues and should have Epic Link instead. " sqref="M2:M3" xr:uid="{16C14239-D6AA-4935-8809-57760481D8F1}">
       <formula1>1</formula1>
       <formula2>1000</formula2>
     </dataValidation>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="It must be a number (integer). This reference is only used during the import process." sqref="K1" xr:uid="{9C637146-F2E3-4D08-87A8-F70FD358E47E}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Use the Issue ID value to link this work item to an Epic_x000a__x000a_Story Issues are not Child-Issues and should have Epic Link instead. " sqref="M1" xr:uid="{A61138FD-C2B2-49D2-810B-69EAE2230B73}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="This field should be the Issue ID or Issue Key of the child tasks. (upstream linkage is not possible)._x000a__x000a__x000a_To link Epics and Stories, use the Epic Link from the Story Issue." sqref="O1:Q1" xr:uid="{BE6B7503-A11A-4130-9D63-988F0CFED80E}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="AUTOMATIC FIELD" prompt="Do not manually edit these!" sqref="AC2:AC5 AF1:AH5" xr:uid="{893DA5FE-9FD0-4D28-BBD0-3D7AEDECEACB}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="H2:H5" xr:uid="{65EDED96-6789-400B-B504-6BC3F5A79E70}">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="AUTOMATIC FIELD" prompt="Do not manually edit these!" sqref="AF2:AH3 AC2:AC3 AF1:AH1" xr:uid="{893DA5FE-9FD0-4D28-BBD0-3D7AEDECEACB}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="H2:H3" xr:uid="{65EDED96-6789-400B-B504-6BC3F5A79E70}">
       <formula1>INDIRECT("CfgComponents[Component.Name]")</formula1>
     </dataValidation>
-    <dataValidation type="list" errorStyle="warning" showErrorMessage="1" error="must be a valid fixversion" sqref="G2:G5" xr:uid="{44FDC20A-8BF5-49B5-9D2C-3A1FE5A7D835}">
+    <dataValidation type="list" errorStyle="warning" showErrorMessage="1" error="must be a valid fixversion" sqref="G2:G3" xr:uid="{44FDC20A-8BF5-49B5-9D2C-3A1FE5A7D835}">
       <formula1>INDIRECT("CfgAssignees[Asssignee.Name]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="I2:I5" xr:uid="{A898E2E7-BC45-4B88-BA1E-4AAA377361D4}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="I2:I3" xr:uid="{A898E2E7-BC45-4B88-BA1E-4AAA377361D4}">
       <formula1>INDIRECT("CfgSprints[Sprint.Name]")</formula1>
     </dataValidation>
     <dataValidation allowBlank="1" showErrorMessage="1" promptTitle="Warning" prompt="Field only used for Epic Issues, so they can be referenced in Story Issues via the Epic Link field.," sqref="N2:N3 L2:L3" xr:uid="{541AD292-0123-4B65-9663-081991FDF0C1}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Field only used for Epic Issues, so they can be referenced in Story Issues via the Epic Link field.," sqref="L1" xr:uid="{64C73155-DEE7-497D-8A98-01E54655ACA8}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="It must be a number (integer) or the Work Item key. This reference is only used during the import process to set the parent." sqref="L1" xr:uid="{8A2BE248-5762-43AD-9C47-C5A92A2E2357}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Field only used for Epic work item, so they can be referenced in Story work items via the Epic Link field. _x000a_DC Only" sqref="N1" xr:uid="{E8F6E005-1F9B-40F3-B24C-E2A3D286C532}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="Creation Marker (Config Sheet)" prompt="Do not manually edit these!" sqref="AD1:AD5" xr:uid="{412C516D-E091-4DDD-9C14-C33AC653C143}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="Feature Pod Label (Config Sheet)" prompt="Do not manually edit these!" sqref="AE1:AE5" xr:uid="{D2234141-379F-4413-AB08-6835BD9FF967}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="AUTOMATIC FIELD" prompt="Do not manually edit these! SKIP types won't be imported into Jira" sqref="AI1:AI5" xr:uid="{5A336857-7D14-4900-8734-BED680BE5154}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="Creation Marker (Config Sheet)" prompt="Do not manually edit these!" sqref="AD1:AD3" xr:uid="{412C516D-E091-4DDD-9C14-C33AC653C143}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="Feature Pod Label (Config Sheet)" prompt="Do not manually edit these!" sqref="AE1:AE3" xr:uid="{D2234141-379F-4413-AB08-6835BD9FF967}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="AUTOMATIC FIELD" prompt="Do not manually edit these! SKIP types won't be imported into Jira" sqref="AI1:AI3" xr:uid="{5A336857-7D14-4900-8734-BED680BE5154}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2736,19 +2266,19 @@
           <x14:formula1>
             <xm:f>Config!$O$4:$O$10</xm:f>
           </x14:formula1>
-          <xm:sqref>A2:A5</xm:sqref>
+          <xm:sqref>A2:A3</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Issue Type" xr:uid="{28BF52BF-C0B0-4D22-B02F-F1408D5A055B}">
           <x14:formula1>
             <xm:f>Config!$U$4:$U$33</xm:f>
           </x14:formula1>
-          <xm:sqref>B2:B5</xm:sqref>
+          <xm:sqref>B2:B3</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" xr:uid="{7708D6E2-1D6B-41D8-A9EE-0E87219BA8EA}">
           <x14:formula1>
             <xm:f>Config!$G$4:$G$8</xm:f>
           </x14:formula1>
-          <xm:sqref>F2:F5</xm:sqref>
+          <xm:sqref>F2:F3</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2759,20 +2289,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2D54512-1380-4F02-BB23-352387C91232}">
   <dimension ref="A1:V21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.6640625" customWidth="1"/>
     <col min="2" max="2" width="49" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="4.33203125" customWidth="1"/>
     <col min="4" max="5" width="18.6640625" customWidth="1"/>
     <col min="6" max="6" width="4.33203125" customWidth="1"/>
-    <col min="7" max="7" width="18.5" customWidth="1"/>
+    <col min="7" max="7" width="18.5546875" customWidth="1"/>
     <col min="8" max="8" width="4.33203125" customWidth="1"/>
-    <col min="9" max="9" width="19.1640625" customWidth="1"/>
+    <col min="9" max="9" width="19.109375" customWidth="1"/>
     <col min="10" max="10" width="4.33203125" customWidth="1"/>
-    <col min="11" max="11" width="18.5" customWidth="1"/>
+    <col min="11" max="11" width="18.5546875" customWidth="1"/>
     <col min="12" max="12" width="4.33203125" customWidth="1"/>
-    <col min="13" max="13" width="17.5" customWidth="1"/>
+    <col min="13" max="13" width="17.5546875" customWidth="1"/>
     <col min="14" max="14" width="4.33203125" customWidth="1"/>
     <col min="15" max="15" width="18.6640625" customWidth="1"/>
     <col min="16" max="16" width="4.33203125" customWidth="1"/>
@@ -2781,68 +2311,68 @@
     <col min="21" max="21" width="22.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="22" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="11" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B1" s="11"/>
       <c r="D1" s="11" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E1" s="11"/>
       <c r="G1" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="I1" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="I1" s="6" t="s">
-        <v>62</v>
-      </c>
       <c r="K1" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="M1" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O1" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q1" s="11" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="R1" s="11"/>
       <c r="S1" s="11"/>
       <c r="U1" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="7"/>
       <c r="D2" s="12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E2" s="12"/>
       <c r="F2" s="7"/>
       <c r="G2" s="10" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H2" s="10"/>
       <c r="I2" s="10" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J2" s="10"/>
       <c r="K2" s="12" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="L2" s="12"/>
       <c r="M2" s="9" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="N2" s="9"/>
       <c r="O2" s="10" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="P2" s="10"/>
       <c r="Q2" s="12"/>
@@ -2850,54 +2380,54 @@
       <c r="S2" s="9"/>
       <c r="T2" s="7"/>
       <c r="U2" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="V2" s="9"/>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G3" t="s">
+        <v>75</v>
+      </c>
+      <c r="I3" t="s">
         <v>74</v>
       </c>
-      <c r="I3" t="s">
+      <c r="K3" t="s">
         <v>73</v>
       </c>
-      <c r="K3" t="s">
+      <c r="M3" t="s">
+        <v>80</v>
+      </c>
+      <c r="O3" t="s">
         <v>72</v>
       </c>
-      <c r="M3" t="s">
-        <v>79</v>
-      </c>
-      <c r="O3" t="s">
-        <v>71</v>
-      </c>
       <c r="Q3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="R3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="S3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B4" t="s">
         <v>50</v>
@@ -2909,10 +2439,10 @@
         <v>1</v>
       </c>
       <c r="G4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K4" t="s">
         <v>39</v>
@@ -2927,7 +2457,7 @@
         <v>31</v>
       </c>
       <c r="R4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="S4" s="7"/>
       <c r="U4" t="str" cm="1">
@@ -2935,9 +2465,9 @@
         <v>Story</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B5" t="s">
         <v>51</v>
@@ -2949,10 +2479,10 @@
         <v>2</v>
       </c>
       <c r="G5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K5" t="s">
         <v>37</v>
@@ -2970,25 +2500,25 @@
         <v>40</v>
       </c>
       <c r="S5" s="7" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="U5" t="str">
         <f ca="1"/>
         <v>Task</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B6" t="s">
         <v>52</v>
       </c>
       <c r="G6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="K6" t="s">
         <v>41</v>
@@ -3003,21 +2533,21 @@
         <v>49</v>
       </c>
       <c r="R6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="S6" s="7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="U6" t="str">
         <f ca="1"/>
         <v>Bug</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="I7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="K7" t="s">
         <v>42</v>
@@ -3033,11 +2563,11 @@
         <v>Epic</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="I8" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="O8" s="1" t="s">
         <v>55</v>
@@ -3047,11 +2577,11 @@
         <v>Comment</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="I9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="O9" s="1" t="s">
         <v>56</v>
@@ -3061,18 +2591,18 @@
         <v>Skip</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="I10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="U10" t="str">
         <f ca="1"/>
         <v>Note</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
       <c r="U11" t="str">
@@ -3080,43 +2610,43 @@
         <v>WorkItem</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="4:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="4:5" x14ac:dyDescent="0.3">
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="4:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="4:5" x14ac:dyDescent="0.3">
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
     </row>
-    <row r="19" spans="4:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="4:5" x14ac:dyDescent="0.3">
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
     </row>
-    <row r="20" spans="4:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="4:5" x14ac:dyDescent="0.3">
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
     </row>
-    <row r="21" spans="4:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="4:5" x14ac:dyDescent="0.3">
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
     </row>
@@ -3147,17 +2677,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -3166,7 +2685,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FB038601AF41D04A88A4BD446922F1A8" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e8d32171d27ae41230d53456f24efae5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c471fd26-9765-4fbe-b6fd-c17c1e55c974" xmlns:ns3="9df69692-83aa-4c55-88c1-62abad05f4fe" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f2fb84de5621acf32f385a2ba90fb29" ns2:_="" ns3:_="">
     <xsd:import namespace="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
@@ -3395,18 +2914,18 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FFE630F-6530-4863-AB67-8477539A0000}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
-    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -3414,7 +2933,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2C983B91-58B3-4C2C-AC55-FFEC9F0DB5F6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3431,4 +2950,15 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FFE630F-6530-4863-AB67-8477539A0000}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
+    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
JT-125 FIx missing formula in the excel template (temp)
</commit_message>
<xml_diff>
--- a/resources/templates/ImportTemplate.xlsx
+++ b/resources/templates/ImportTemplate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workdir\DeerHide\sources\jira-toolkit\resources\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6F4E5E5-CAF5-42B8-BDD6-A49043ED4875}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAB2016C-9C42-4109-8F33-1BC568D87C6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="5355" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="111">
   <si>
     <t>Priority</t>
   </si>
@@ -399,9 +399,6 @@
   </si>
   <si>
     <t>Quality Control</t>
-  </si>
-  <si>
-    <t>g</t>
   </si>
 </sst>
 </file>
@@ -501,7 +498,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -534,16 +531,13 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Accent4" xfId="2" builtinId="41"/>
     <cellStyle name="Explanatory Text" xfId="1" builtinId="53"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="72">
+  <dxfs count="56">
     <dxf>
       <fill>
         <patternFill patternType="darkUp"/>
@@ -682,6 +676,12 @@
       </fill>
     </dxf>
     <dxf>
+      <alignment horizontal="general" vertical="bottom" shrinkToFit="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
       <alignment vertical="top"/>
     </dxf>
     <dxf>
@@ -804,149 +804,6 @@
     </dxf>
     <dxf>
       <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="darkUp"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDAF2D0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2CEEF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.89996032593768116"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <i/>
-        <strike val="0"/>
-        <color theme="0" tint="-0.34998626667073579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFF9B1AB"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCC99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9999"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF99CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" shrinkToFit="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -962,57 +819,57 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="JiraDataset" displayName="JiraDataset" ref="A1:AJ4" totalsRowShown="0" headerRowDxfId="53" dataDxfId="52">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="JiraDataset" displayName="JiraDataset" ref="A1:AJ4" totalsRowShown="0" headerRowDxfId="55" dataDxfId="54">
   <autoFilter ref="A1:AJ4" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="36">
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Priority" dataDxfId="51"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="IssueType" dataDxfId="50"/>
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Summary" dataDxfId="49"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Issue Key" dataDxfId="48"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Description" dataDxfId="47"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="FixVersion" dataDxfId="46">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Priority" dataDxfId="53"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="IssueType" dataDxfId="52"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Summary" dataDxfId="51"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Issue Key" dataDxfId="50"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Description" dataDxfId="49"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="FixVersion" dataDxfId="48">
       <calculatedColumnFormula>Config!$G$4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="Assignee.Name" dataDxfId="45"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Component" dataDxfId="44"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Sprint Name" dataDxfId="43"/>
-    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0000-000028000000}" name="Estimate" dataDxfId="42"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Issue ID" dataDxfId="41"/>
-    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="Parent" dataDxfId="40"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Epic Link" dataDxfId="39"/>
-    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0000-000021000000}" name="Epic Name" dataDxfId="38">
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="Assignee.Name" dataDxfId="47"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Component" dataDxfId="46"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Sprint Name" dataDxfId="45"/>
+    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0000-000028000000}" name="Estimate" dataDxfId="44"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Issue ID" dataDxfId="43"/>
+    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="Parent" dataDxfId="42"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Epic Link" dataDxfId="41"/>
+    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0000-000021000000}" name="Epic Name" dataDxfId="40">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[IssueType]]="Epic",JiraDataset[[#This Row],[Summary]],"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0000-00001B000000}" name="Child-Issue" dataDxfId="37"/>
-    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0000-000029000000}" name="Child-Issue1" dataDxfId="36"/>
-    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0000-00001D000000}" name="Child-Issue2" dataDxfId="35"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Labels" dataDxfId="34"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Labels1" dataDxfId="33"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Labels2" dataDxfId="32"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Labels3" dataDxfId="31"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Labels4" dataDxfId="30"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Labels5" dataDxfId="29"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Labels6" dataDxfId="28"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Labels7" dataDxfId="27"/>
-    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0000-00001A000000}" name="Labels8" dataDxfId="26"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Labels9" dataDxfId="25"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="Labels10" dataDxfId="24"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Sprint" dataDxfId="23">
+    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0000-00001B000000}" name="Child-Issue" dataDxfId="39"/>
+    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0000-000029000000}" name="Child-Issue1" dataDxfId="38"/>
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0000-00001D000000}" name="Child-Issue2" dataDxfId="37"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Labels" dataDxfId="36"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Labels1" dataDxfId="35"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Labels2" dataDxfId="34"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Labels3" dataDxfId="33"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Labels4" dataDxfId="32"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Labels5" dataDxfId="31"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Labels6" dataDxfId="30"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Labels7" dataDxfId="29"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0000-00001A000000}" name="Labels8" dataDxfId="28"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Labels9" dataDxfId="27"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="Labels10" dataDxfId="26"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Sprint" dataDxfId="25">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], Config!$D$4:$E$9, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="Labels0001" dataDxfId="22">
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="Labels0001" dataDxfId="24">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0000-000027000000}" name="Labels0002" dataDxfId="21">
+    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0000-000027000000}" name="Labels0002" dataDxfId="23">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Feature Pod Label", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Assignee" dataDxfId="20">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Assignee" dataDxfId="22">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], Config!$A$4:$B$24, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="Project Key" dataDxfId="19">
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="Project Key" dataDxfId="21">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Project Key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0000-00002A000000}" name="OrigEst" dataDxfId="18">
+    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0000-00002A000000}" name="OrigEst" dataDxfId="20">
       <calculatedColumnFormula array="1">IF(
   JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
   "",
@@ -1028,7 +885,7 @@
   )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="44" xr3:uid="{00000000-0010-0000-0000-00002C000000}" name="RowType" dataDxfId="17">
+    <tableColumn id="44" xr3:uid="{00000000-0010-0000-0000-00002C000000}" name="RowType" dataDxfId="19">
       <calculatedColumnFormula array="1">IFERROR(
     _xlfn.IFS(
         JiraDataset[[#This Row],[IssueType]] = cfg_type_comment,"SKIP",
@@ -1038,7 +895,7 @@
     cfg_type_workitem
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="Note" dataDxfId="16"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="Note" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1078,7 +935,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="CfgPriorities" displayName="CfgPriorities" ref="O3:O9" totalsRowShown="0">
   <autoFilter ref="O3:O9" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Priority.Name" dataDxfId="71"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Priority.Name" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1112,7 +969,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="Name"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="Remark" dataDxfId="70"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="Remark" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1719,7 +1576,7 @@
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
-      <c r="F4" s="14" t="str">
+      <c r="F4" s="3" t="str">
         <f>Config!$G$4</f>
         <v>JITTP Version 1</v>
       </c>
@@ -1728,9 +1585,9 @@
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
-      <c r="L4" s="14"/>
+      <c r="L4" s="3"/>
       <c r="M4" s="3"/>
-      <c r="N4" s="14" t="str">
+      <c r="N4" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[IssueType]]="Epic",JiraDataset[[#This Row],[Summary]],"")</f>
         <v/>
       </c>
@@ -1748,11 +1605,11 @@
       <c r="Z4" s="3"/>
       <c r="AA4" s="3"/>
       <c r="AB4" s="3"/>
-      <c r="AC4" s="14" t="str">
+      <c r="AC4" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], Config!$D$4:$E$9, 2, FALSE), ""))</f>
         <v/>
       </c>
-      <c r="AD4" s="14" t="str">
+      <c r="AD4" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
         <v>imported</v>
       </c>
@@ -1760,15 +1617,15 @@
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Feature Pod Label", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
         <v>pod_test</v>
       </c>
-      <c r="AF4" s="14" t="str">
+      <c r="AF4" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], Config!$A$4:$B$24, 2, FALSE), ""))</f>
         <v/>
       </c>
-      <c r="AG4" s="14" t="str">
+      <c r="AG4" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Project Key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
         <v>JITTP2</v>
       </c>
-      <c r="AH4" s="14" t="str" cm="1">
+      <c r="AH4" s="3" t="str" cm="1">
         <f t="array" ref="AH4">IF(
   JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
   "",
@@ -1785,7 +1642,7 @@
 )</f>
         <v/>
       </c>
-      <c r="AI4" s="14" t="str" cm="1">
+      <c r="AI4" s="3" t="str" cm="1">
         <f t="array" ref="AI4">IFERROR(
     _xlfn.IFS(
         JiraDataset[[#This Row],[IssueType]] = cfg_type_comment,"SKIP",
@@ -1796,9 +1653,7 @@
 )</f>
         <v>WorkItem</v>
       </c>
-      <c r="AJ4" s="3" t="s">
-        <v>111</v>
-      </c>
+      <c r="AJ4" s="3"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:A4 C2:C4">

</xml_diff>

<commit_message>
Update ImportTemplate.xlsx to reflect recent changes
</commit_message>
<xml_diff>
--- a/resources/templates/ImportTemplate.xlsx
+++ b/resources/templates/ImportTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workdir\temp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workdir\DeerHide\sources\jira-toolkit\resources\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77E3885F-31A5-4652-AED3-4A4A21786D96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC33135F-B90A-4C24-BAC9-7A123C771B85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="252" yWindow="6408" windowWidth="30696" windowHeight="12420" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
+    <workbookView xWindow="5376" yWindow="5376" windowWidth="34560" windowHeight="18600" activeTab="1" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset" sheetId="1" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="110">
   <si>
     <t>IssueType</t>
   </si>
@@ -245,6 +245,9 @@
     <t>Creation Marker</t>
   </si>
   <si>
+    <t>JV</t>
+  </si>
+  <si>
     <t>Issue Type</t>
   </si>
   <si>
@@ -396,12 +399,6 @@
   </si>
   <si>
     <t>pod_test</t>
-  </si>
-  <si>
-    <t>High</t>
-  </si>
-  <si>
-    <t>Test, Task</t>
   </si>
 </sst>
 </file>
@@ -925,7 +922,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -956,15 +953,6 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="16" applyAlignment="1">
       <alignment horizontal="left" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1011,7 +999,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="72">
+  <dxfs count="56">
     <dxf>
       <fill>
         <patternFill patternType="darkUp"/>
@@ -1155,146 +1143,10 @@
       </fill>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="darkUp"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDAF2D0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2CEEF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.89996032593768116"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <strike val="0"/>
-        <color theme="0" tint="-0.34998626667073579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFF9B1AB"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCC99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9999"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF99CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6699"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
       <alignment vertical="top"/>
@@ -1437,12 +1289,6 @@
     </dxf>
     <dxf>
       <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1474,61 +1320,63 @@
 <file path=xl/namedSheetViews/namedSheetView1.xml><?xml version="1.0" encoding="utf-8"?>
 <namedSheetViews xmlns="http://schemas.microsoft.com/office/spreadsheetml/2019/namedsheetviews" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <namedSheetView name="View1" id="{77233F75-225A-4D7F-8A86-543E0A8C6E58}">
-    <nsvFilter filterId="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" ref="A1:AJ4" tableId="1"/>
+    <nsvFilter filterId="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" ref="A1:AJ3" tableId="1"/>
   </namedSheetView>
 </namedSheetViews>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" name="JiraDataset" displayName="JiraDataset" ref="A1:AJ4" totalsRowShown="0" headerRowDxfId="69" dataDxfId="68">
-  <autoFilter ref="A1:AJ4" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" name="JiraDataset" displayName="JiraDataset" ref="A1:AJ3" totalsRowShown="0" headerRowDxfId="55" dataDxfId="54">
+  <autoFilter ref="A1:AJ3" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}"/>
   <tableColumns count="36">
-    <tableColumn id="3" xr3:uid="{AF2EC907-349C-4651-852D-6E39C61E17FF}" name="Priority" dataDxfId="67"/>
-    <tableColumn id="2" xr3:uid="{E90C51F2-4386-421F-A3E4-E2CA9D43D396}" name="IssueType" dataDxfId="66"/>
-    <tableColumn id="1" xr3:uid="{BBAD373B-BA13-47E4-9F74-565F4D9E9680}" name="Summary" dataDxfId="65"/>
-    <tableColumn id="4" xr3:uid="{026E5B97-FAFC-4E46-860E-0B0C976B1148}" name="Issue Key" dataDxfId="64"/>
-    <tableColumn id="5" xr3:uid="{A2C262E8-D544-4669-99F1-151EDE081654}" name="Description" dataDxfId="63"/>
-    <tableColumn id="7" xr3:uid="{0FAD1ACC-432E-462C-8B89-71540710BCB5}" name="FixVersion" dataDxfId="62"/>
-    <tableColumn id="28" xr3:uid="{07F3030C-7187-4B16-BBDB-798304851975}" name="Assignee.Name" dataDxfId="61"/>
-    <tableColumn id="8" xr3:uid="{8C7FB8DB-A85B-4189-93D8-0F0D4EEEF81B}" name="Component" dataDxfId="60"/>
-    <tableColumn id="9" xr3:uid="{DC5101A8-1204-44D2-BC2C-FEE1A4EFE7C1}" name="Sprint Name" dataDxfId="59"/>
-    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="58"/>
-    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="57"/>
-    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="56"/>
-    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="55"/>
-    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="54">
+    <tableColumn id="3" xr3:uid="{AF2EC907-349C-4651-852D-6E39C61E17FF}" name="Priority" dataDxfId="53"/>
+    <tableColumn id="2" xr3:uid="{E90C51F2-4386-421F-A3E4-E2CA9D43D396}" name="IssueType" dataDxfId="52"/>
+    <tableColumn id="1" xr3:uid="{BBAD373B-BA13-47E4-9F74-565F4D9E9680}" name="Summary" dataDxfId="51"/>
+    <tableColumn id="4" xr3:uid="{026E5B97-FAFC-4E46-860E-0B0C976B1148}" name="Issue Key" dataDxfId="50"/>
+    <tableColumn id="5" xr3:uid="{A2C262E8-D544-4669-99F1-151EDE081654}" name="Description" dataDxfId="49"/>
+    <tableColumn id="7" xr3:uid="{0FAD1ACC-432E-462C-8B89-71540710BCB5}" name="FixVersion" dataDxfId="48">
+      <calculatedColumnFormula>Config!$G$4</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="28" xr3:uid="{07F3030C-7187-4B16-BBDB-798304851975}" name="Assignee.Name" dataDxfId="47"/>
+    <tableColumn id="8" xr3:uid="{8C7FB8DB-A85B-4189-93D8-0F0D4EEEF81B}" name="Component" dataDxfId="46"/>
+    <tableColumn id="9" xr3:uid="{DC5101A8-1204-44D2-BC2C-FEE1A4EFE7C1}" name="Sprint Name" dataDxfId="45"/>
+    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="44"/>
+    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="43"/>
+    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="42"/>
+    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="41"/>
+    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="40">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[IssueType]]="Epic",JiraDataset[[#This Row],[Summary]],"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="27" xr3:uid="{911C8FDC-5528-43FC-BDF4-D4761F03C0E5}" name="Child-Issue" dataDxfId="53"/>
-    <tableColumn id="41" xr3:uid="{AB248E07-9BFA-42CC-BC41-B4234F677BFB}" name="Child-Issue1" dataDxfId="52"/>
-    <tableColumn id="29" xr3:uid="{89D12135-F3E3-4253-844F-1B9A54169953}" name="Child-Issue2" dataDxfId="51"/>
-    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="50"/>
-    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="49"/>
-    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="48"/>
-    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="47"/>
-    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="46"/>
-    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="45"/>
-    <tableColumn id="18" xr3:uid="{16B98070-7F8A-4FC7-AD99-EA81D0BD26AB}" name="Labels6" dataDxfId="44"/>
-    <tableColumn id="19" xr3:uid="{016EAEF4-8EA9-408B-9F1A-ECFB17E81C77}" name="Labels7" dataDxfId="43"/>
-    <tableColumn id="26" xr3:uid="{8263F9EC-BF0A-46F7-BA83-6083A4262B91}" name="Labels8" dataDxfId="42"/>
-    <tableColumn id="20" xr3:uid="{389B11C5-1B22-48C0-BCA2-72F050425FA1}" name="Labels9" dataDxfId="41"/>
-    <tableColumn id="25" xr3:uid="{AE95F8A2-F7F0-4985-9AE6-4201B9792775}" name="Labels10" dataDxfId="40"/>
-    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="39">
+    <tableColumn id="27" xr3:uid="{911C8FDC-5528-43FC-BDF4-D4761F03C0E5}" name="Child-Issue" dataDxfId="39"/>
+    <tableColumn id="41" xr3:uid="{AB248E07-9BFA-42CC-BC41-B4234F677BFB}" name="Child-Issue1" dataDxfId="38"/>
+    <tableColumn id="29" xr3:uid="{89D12135-F3E3-4253-844F-1B9A54169953}" name="Child-Issue2" dataDxfId="37"/>
+    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="36"/>
+    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="35"/>
+    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="34"/>
+    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="33"/>
+    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="32"/>
+    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="31"/>
+    <tableColumn id="18" xr3:uid="{16B98070-7F8A-4FC7-AD99-EA81D0BD26AB}" name="Labels6" dataDxfId="30"/>
+    <tableColumn id="19" xr3:uid="{016EAEF4-8EA9-408B-9F1A-ECFB17E81C77}" name="Labels7" dataDxfId="29"/>
+    <tableColumn id="26" xr3:uid="{8263F9EC-BF0A-46F7-BA83-6083A4262B91}" name="Labels8" dataDxfId="28"/>
+    <tableColumn id="20" xr3:uid="{389B11C5-1B22-48C0-BCA2-72F050425FA1}" name="Labels9" dataDxfId="27"/>
+    <tableColumn id="25" xr3:uid="{AE95F8A2-F7F0-4985-9AE6-4201B9792775}" name="Labels10" dataDxfId="26"/>
+    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="25">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], Config!$D$4:$E$9, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="38">
+    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="24">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="37">
+    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="23">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Feature Pod Label", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="36">
+    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="22">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], Config!$A$4:$B$24, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="35">
+    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="21">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Project Key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="34">
+    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="20">
       <calculatedColumnFormula array="1">IF(
   JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
   "",
@@ -1544,7 +1392,7 @@
   )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="33">
+    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="19">
       <calculatedColumnFormula array="1">IFERROR(
     _xlfn.IFS(
         JiraDataset[[#This Row],[IssueType]] = cfg_type_comment,"SKIP",
@@ -1554,15 +1402,15 @@
     cfg_type_workitem
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="32"/>
+    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{93F2D14D-2ABD-4171-895D-1041B0893491}" name="CfgComponents" displayName="CfgComponents" ref="I3:I11" totalsRowShown="0">
-  <autoFilter ref="I3:I11" xr:uid="{93F2D14D-2ABD-4171-895D-1041B0893491}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{93F2D14D-2ABD-4171-895D-1041B0893491}" name="CfgComponents" displayName="CfgComponents" ref="I3:I10" totalsRowShown="0">
+  <autoFilter ref="I3:I10" xr:uid="{93F2D14D-2ABD-4171-895D-1041B0893491}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{10F6CCA4-1068-4FC8-AB82-E48B87DB0F71}" name="Component.Name"/>
   </tableColumns>
@@ -1571,8 +1419,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{7007FF9D-9384-422B-8DB3-300D782E5FE6}" name="CfgFixVersions" displayName="CfgFixVersions" ref="G3:G7" totalsRowShown="0">
-  <autoFilter ref="G3:G7" xr:uid="{7007FF9D-9384-422B-8DB3-300D782E5FE6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{7007FF9D-9384-422B-8DB3-300D782E5FE6}" name="CfgFixVersions" displayName="CfgFixVersions" ref="G3:G6" totalsRowShown="0">
+  <autoFilter ref="G3:G6" xr:uid="{7007FF9D-9384-422B-8DB3-300D782E5FE6}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{E20FAA91-E54E-42EA-9BFF-2FDA27CD5D33}" name="FixVersion.Name"/>
   </tableColumns>
@@ -1594,15 +1442,15 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}" name="CfgPriorities" displayName="CfgPriorities" ref="O3:O9" totalsRowShown="0">
   <autoFilter ref="O3:O9" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="71"/>
+    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{1EF5833D-4918-4C71-A990-1B275126361D}" name="CfgAssignees" displayName="CfgAssignees" ref="A3:B7" totalsRowShown="0">
-  <autoFilter ref="A3:B7" xr:uid="{1EF5833D-4918-4C71-A990-1B275126361D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{1EF5833D-4918-4C71-A990-1B275126361D}" name="CfgAssignees" displayName="CfgAssignees" ref="A3:B6" totalsRowShown="0">
+  <autoFilter ref="A3:B6" xr:uid="{1EF5833D-4918-4C71-A990-1B275126361D}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{7F7B4E10-E51C-443F-875D-3E6A9FD9994C}" name="Asssignee.Name"/>
     <tableColumn id="2" xr3:uid="{3A4C6F03-89A9-4E38-8288-00D055D51CD3}" name="Assignee.ID"/>
@@ -1612,8 +1460,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{72674B63-54C8-47AC-9FF0-4034C2D499BA}" name="CfgSprints" displayName="CfgSprints" ref="D3:E6" totalsRowShown="0">
-  <autoFilter ref="D3:E6" xr:uid="{72674B63-54C8-47AC-9FF0-4034C2D499BA}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{72674B63-54C8-47AC-9FF0-4034C2D499BA}" name="CfgSprints" displayName="CfgSprints" ref="D3:E5" totalsRowShown="0">
+  <autoFilter ref="D3:E5" xr:uid="{72674B63-54C8-47AC-9FF0-4034C2D499BA}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{397B719B-4CC6-4F47-8F3C-168F13ED56DA}" name="Sprint.Name"/>
     <tableColumn id="2" xr3:uid="{2FD208E7-540E-4D07-9144-6E9F3065D9DE}" name="Sprint.ID"/>
@@ -1628,7 +1476,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{D4E1611F-A2CF-465D-A219-1759EA66687D}" name="Name"/>
     <tableColumn id="2" xr3:uid="{174D0D86-B1AA-4BF7-AC91-FCACFC898851}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Remark" dataDxfId="70"/>
+    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Remark" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1961,14 +1809,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F73058B-F76D-4AAE-8108-6C4469E9D8B5}">
-  <dimension ref="A1:AK4"/>
+  <dimension ref="A1:AK3"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelCol="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="12.44140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="31.6640625" customWidth="1"/>
     <col min="4" max="4" width="11.88671875" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="33" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.5546875" customWidth="1"/>
+    <col min="6" max="6" width="46.33203125" customWidth="1"/>
     <col min="7" max="7" width="17.44140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22.5546875" customWidth="1"/>
     <col min="9" max="9" width="14" bestFit="1" customWidth="1"/>
@@ -2032,7 +1880,7 @@
         <v>10</v>
       </c>
       <c r="L1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="M1" s="3" t="s">
         <v>11</v>
@@ -2124,9 +1972,11 @@
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
       <c r="J2" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="K2" s="3"/>
+        <v>83</v>
+      </c>
+      <c r="K2" s="3">
+        <v>1</v>
+      </c>
       <c r="L2" s="3"/>
       <c r="M2" s="3"/>
       <c r="N2" s="3" t="str">
@@ -2205,21 +2055,29 @@
         <v>42</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
+        <v>98</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>47</v>
+      </c>
       <c r="J3" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="K3" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>
@@ -2241,9 +2099,9 @@
       <c r="Z3" s="3"/>
       <c r="AA3" s="3"/>
       <c r="AB3" s="3"/>
-      <c r="AC3" s="3" t="str">
+      <c r="AC3" s="3">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], Config!$D$4:$E$9, 2, FALSE), ""))</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="AD3" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
@@ -2291,161 +2149,71 @@
       </c>
       <c r="AJ3" s="3"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.3">
-      <c r="A4" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="B4" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>110</v>
-      </c>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="15">
-        <v>1</v>
-      </c>
-      <c r="M4" s="3"/>
-      <c r="N4" s="15" t="str">
-        <f>IF(JiraDataset[[#This Row],[IssueType]]="Epic",JiraDataset[[#This Row],[Summary]],"")</f>
-        <v/>
-      </c>
-      <c r="O4" s="3"/>
-      <c r="P4" s="3"/>
-      <c r="Q4" s="3"/>
-      <c r="R4" s="3"/>
-      <c r="S4" s="3"/>
-      <c r="T4" s="3"/>
-      <c r="U4" s="3"/>
-      <c r="V4" s="3"/>
-      <c r="W4" s="3"/>
-      <c r="X4" s="3"/>
-      <c r="Y4" s="3"/>
-      <c r="Z4" s="3"/>
-      <c r="AA4" s="3"/>
-      <c r="AB4" s="3"/>
-      <c r="AC4" s="15" t="str">
-        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], Config!$D$4:$E$9, 2, FALSE), ""))</f>
-        <v/>
-      </c>
-      <c r="AD4" s="15" t="str">
-        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
-        <v>imported</v>
-      </c>
-      <c r="AE4" s="8" t="str">
-        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Feature Pod Label", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
-        <v>pod_test</v>
-      </c>
-      <c r="AF4" s="15" t="str">
-        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], Config!$A$4:$B$24, 2, FALSE), ""))</f>
-        <v/>
-      </c>
-      <c r="AG4" s="15" t="str">
-        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Project Key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
-        <v>JITTP2</v>
-      </c>
-      <c r="AH4" s="15" t="str" cm="1">
-        <f t="array" ref="AH4">IF(
-  JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
-  "",
-  _xlfn.LET(
-    _xlpm.p, _xlfn.TEXTSPLIT(JiraDataset[[#This Row],[Estimate]], " "),
-    _xlpm.getVal, _xlfn.LAMBDA(_xlpm.u, IFERROR(VALUE(LEFT(_xlfn._xlws.FILTER(_xlpm.p, RIGHT(_xlpm.p,1)=_xlpm.u), LEN(_xlfn._xlws.FILTER(_xlpm.p, RIGHT(_xlpm.p,1)=_xlpm.u))-1)), 0)),
-    _xlpm.w, _xlpm.getVal("w"),
-    _xlpm.d, _xlpm.getVal("d"),
-    _xlpm.h, _xlpm.getVal("h"),
-    _xlpm.m, _xlpm.getVal("m"),
-    _xlpm.seconds, _xlpm.w*144000 + _xlpm.d*28800 + _xlpm.h*3600 + _xlpm.m*60,
-    IF(_xlpm.seconds=0, "", _xlpm.seconds*60)
-  )
-)</f>
-        <v/>
-      </c>
-      <c r="AI4" s="15" t="str" cm="1">
-        <f t="array" ref="AI4">IFERROR(
-    _xlfn.IFS(
-        JiraDataset[[#This Row],[IssueType]] = cfg_type_comment,"SKIP",
-        JiraDataset[[#This Row],[IssueType]] = cfg_type_skip,"SKIP",
-        JiraDataset[[#This Row],[IssueType]] = cfg_type_note,"SKIP"
-    ),
-    cfg_type_workitem
-)</f>
-        <v>WorkItem</v>
-      </c>
-      <c r="AJ4" s="3"/>
-    </row>
   </sheetData>
   <protectedRanges>
     <protectedRange sqref="A1:A1048576 D4:N1048576 P4:AD1048576 C1:AB3" name="User Input"/>
     <protectedRange algorithmName="SHA-512" hashValue="tpheD+JLADkhiyalt6vInlMwkILPZx4PVQN/k2vmwjOBdYUuHaXCrwtObHeFz5dJh9f853O84pZ1Rn9Ujz33+A==" saltValue="9ir5NB4CJc/69S/Eh84/mA==" spinCount="100000" sqref="AC1:AI3 AE4:AK1048576" name="Computed values"/>
   </protectedRanges>
   <phoneticPr fontId="18" type="noConversion"/>
-  <conditionalFormatting sqref="A2:A4 C2:C4">
-    <cfRule type="containsText" dxfId="31" priority="429" operator="containsText" text="blocker">
+  <conditionalFormatting sqref="A2:A3 C2:C3">
+    <cfRule type="containsText" dxfId="15" priority="429" operator="containsText" text="blocker">
       <formula>NOT(ISERROR(SEARCH("blocker",A2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="30" priority="430" operator="containsText" text="critical">
+    <cfRule type="containsText" dxfId="14" priority="430" operator="containsText" text="critical">
       <formula>NOT(ISERROR(SEARCH("critical",A2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="29" priority="431" operator="containsText" text="High">
+    <cfRule type="containsText" dxfId="13" priority="431" operator="containsText" text="High">
       <formula>NOT(ISERROR(SEARCH("High",A2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="28" priority="432" operator="containsText" text="Medium">
+    <cfRule type="containsText" dxfId="12" priority="432" operator="containsText" text="Medium">
       <formula>NOT(ISERROR(SEARCH("Medium",A2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:A4">
-    <cfRule type="containsBlanks" dxfId="27" priority="493">
+  <conditionalFormatting sqref="A2:A3">
+    <cfRule type="containsBlanks" dxfId="11" priority="493">
       <formula>LEN(TRIM(A2))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:AJ4">
-    <cfRule type="expression" dxfId="26" priority="409" stopIfTrue="1">
+  <conditionalFormatting sqref="A2:AJ3">
+    <cfRule type="expression" dxfId="10" priority="409" stopIfTrue="1">
       <formula>$B2=cfg_type_comment</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="25" priority="410">
+    <cfRule type="expression" dxfId="9" priority="410">
       <formula>$B2=cfg_type_skip</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="411">
+    <cfRule type="expression" dxfId="8" priority="411">
       <formula>$B2=cfg_type_note</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2:B4">
-    <cfRule type="containsText" dxfId="23" priority="413" operator="containsText" text="epic">
+  <conditionalFormatting sqref="B2:B3">
+    <cfRule type="containsText" dxfId="7" priority="413" operator="containsText" text="epic">
       <formula>NOT(ISERROR(SEARCH("epic",B2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="22" priority="427" operator="containsText" text="story">
+    <cfRule type="containsText" dxfId="6" priority="427" operator="containsText" text="story">
       <formula>NOT(ISERROR(SEARCH("story",B2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="21" priority="433" operator="containsText" text="task">
+    <cfRule type="containsText" dxfId="5" priority="433" operator="containsText" text="task">
       <formula>NOT(ISERROR(SEARCH("task",B2)))</formula>
     </cfRule>
-    <cfRule type="containsBlanks" dxfId="20" priority="492">
+    <cfRule type="containsBlanks" dxfId="4" priority="492">
       <formula>LEN(TRIM(B2))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2:AJ4">
-    <cfRule type="expression" dxfId="19" priority="1">
+  <conditionalFormatting sqref="B2:AJ3">
+    <cfRule type="expression" dxfId="3" priority="1">
       <formula>$B2="Epic"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="2">
+    <cfRule type="expression" dxfId="2" priority="2">
       <formula>$B2="Story"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C4">
-    <cfRule type="containsBlanks" dxfId="17" priority="494">
+  <conditionalFormatting sqref="C2:C3">
+    <cfRule type="containsBlanks" dxfId="1" priority="494">
       <formula>LEN(TRIM(C2))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:L4">
-    <cfRule type="containsBlanks" dxfId="16" priority="412">
+  <conditionalFormatting sqref="K2:L3">
+    <cfRule type="containsBlanks" dxfId="0" priority="412">
       <formula>LEN(TRIM(K2))=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2454,37 +2222,37 @@
       <formula1>1</formula1>
       <formula2>1000</formula2>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="J2:J4" xr:uid="{386E3B68-2486-4DDE-BEB1-45F897521149}"/>
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" promptTitle="Warning" prompt="This field should be the Issue ID or Issue Key of the child tasks. (upstream linkage is not possible)._x000a__x000a__x000a_To link Epics and Stories, use the Epic Link from the Story Issue." sqref="O2:Q4" xr:uid="{D7BD960D-9CEA-4120-B2E3-2AE0D4661093}">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="J2:J3" xr:uid="{386E3B68-2486-4DDE-BEB1-45F897521149}"/>
+    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" promptTitle="Warning" prompt="This field should be the Issue ID or Issue Key of the child tasks. (upstream linkage is not possible)._x000a__x000a__x000a_To link Epics and Stories, use the Epic Link from the Story Issue." sqref="O2:Q3" xr:uid="{D7BD960D-9CEA-4120-B2E3-2AE0D4661093}">
       <formula1>1</formula1>
       <formula2>1000</formula2>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Note" prompt="The content of this column will be ignored during the Jira import." sqref="AJ2:AJ4" xr:uid="{2DA3EDB6-7635-4349-8860-B614B5B71275}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Permissions" prompt="Updating Existing Issues requires global admin permissions" sqref="D2:D4" xr:uid="{D5E4A4BB-53C8-42DF-9B52-F5E00AC6407B}"/>
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" promptTitle="Warning" prompt="Use the Issue ID value to link this work item to an Epic_x000a__x000a_Story Issues are not Child-Issues and should have Epic Link instead. " sqref="M2:M4" xr:uid="{16C14239-D6AA-4935-8809-57760481D8F1}">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Note" prompt="The content of this column will be ignored during the Jira import." sqref="AJ2:AJ3" xr:uid="{2DA3EDB6-7635-4349-8860-B614B5B71275}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Permissions" prompt="Updating Existing Issues requires global admin permissions" sqref="D2:D3" xr:uid="{D5E4A4BB-53C8-42DF-9B52-F5E00AC6407B}"/>
+    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" promptTitle="Warning" prompt="Use the Issue ID value to link this work item to an Epic_x000a__x000a_Story Issues are not Child-Issues and should have Epic Link instead. " sqref="M2:M3" xr:uid="{16C14239-D6AA-4935-8809-57760481D8F1}">
       <formula1>1</formula1>
       <formula2>1000</formula2>
     </dataValidation>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="It must be a number (integer). This reference is only used during the import process." sqref="K1" xr:uid="{9C637146-F2E3-4D08-87A8-F70FD358E47E}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Use the Issue ID value to link this work item to an Epic_x000a__x000a_Story Issues are not Child-Issues and should have Epic Link instead. " sqref="M1" xr:uid="{A61138FD-C2B2-49D2-810B-69EAE2230B73}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="This field should be the Issue ID or Issue Key of the child tasks. (upstream linkage is not possible)._x000a__x000a__x000a_To link Epics and Stories, use the Epic Link from the Story Issue." sqref="O1:Q1" xr:uid="{BE6B7503-A11A-4130-9D63-988F0CFED80E}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="AUTOMATIC FIELD" prompt="Do not manually edit these!" sqref="AC2:AC4 AF1:AH4" xr:uid="{893DA5FE-9FD0-4D28-BBD0-3D7AEDECEACB}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="H2:H4" xr:uid="{65EDED96-6789-400B-B504-6BC3F5A79E70}">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="AUTOMATIC FIELD" prompt="Do not manually edit these!" sqref="AF2:AH3 AC2:AC3 AF1:AH1" xr:uid="{893DA5FE-9FD0-4D28-BBD0-3D7AEDECEACB}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="H2:H3" xr:uid="{65EDED96-6789-400B-B504-6BC3F5A79E70}">
       <formula1>INDIRECT("CfgComponents[Component.Name]")</formula1>
     </dataValidation>
-    <dataValidation type="list" errorStyle="warning" showErrorMessage="1" error="must be a valid fixversion" sqref="G2:G4" xr:uid="{44FDC20A-8BF5-49B5-9D2C-3A1FE5A7D835}">
+    <dataValidation type="list" errorStyle="warning" showErrorMessage="1" error="must be a valid fixversion" sqref="G2:G3" xr:uid="{44FDC20A-8BF5-49B5-9D2C-3A1FE5A7D835}">
       <formula1>INDIRECT("CfgAssignees[Asssignee.Name]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="I2:I4" xr:uid="{A898E2E7-BC45-4B88-BA1E-4AAA377361D4}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="I2:I3" xr:uid="{A898E2E7-BC45-4B88-BA1E-4AAA377361D4}">
       <formula1>INDIRECT("CfgSprints[Sprint.Name]")</formula1>
     </dataValidation>
     <dataValidation allowBlank="1" showErrorMessage="1" promptTitle="Warning" prompt="Field only used for Epic Issues, so they can be referenced in Story Issues via the Epic Link field.," sqref="N2:N3 L2:L3" xr:uid="{541AD292-0123-4B65-9663-081991FDF0C1}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Field only used for Epic Issues, so they can be referenced in Story Issues via the Epic Link field.," sqref="L1" xr:uid="{64C73155-DEE7-497D-8A98-01E54655ACA8}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="It must be a number (integer) or the Work Item key. This reference is only used during the import process to set the parent." sqref="L1" xr:uid="{8A2BE248-5762-43AD-9C47-C5A92A2E2357}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Field only used for Epic work item, so they can be referenced in Story work items via the Epic Link field. _x000a_DC Only" sqref="N1" xr:uid="{E8F6E005-1F9B-40F3-B24C-E2A3D286C532}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="Creation Marker (Config Sheet)" prompt="Do not manually edit these!" sqref="AD1:AD4" xr:uid="{412C516D-E091-4DDD-9C14-C33AC653C143}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="Feature Pod Label (Config Sheet)" prompt="Do not manually edit these!" sqref="AE1:AE4" xr:uid="{D2234141-379F-4413-AB08-6835BD9FF967}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="AUTOMATIC FIELD" prompt="Do not manually edit these! SKIP types won't be imported into Jira" sqref="AI1:AI4" xr:uid="{5A336857-7D14-4900-8734-BED680BE5154}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="Creation Marker (Config Sheet)" prompt="Do not manually edit these!" sqref="AD1:AD3" xr:uid="{412C516D-E091-4DDD-9C14-C33AC653C143}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="Feature Pod Label (Config Sheet)" prompt="Do not manually edit these!" sqref="AE1:AE3" xr:uid="{D2234141-379F-4413-AB08-6835BD9FF967}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="AUTOMATIC FIELD" prompt="Do not manually edit these! SKIP types won't be imported into Jira" sqref="AI1:AI3" xr:uid="{5A336857-7D14-4900-8734-BED680BE5154}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2498,19 +2266,19 @@
           <x14:formula1>
             <xm:f>Config!$O$4:$O$10</xm:f>
           </x14:formula1>
-          <xm:sqref>A2:A4</xm:sqref>
+          <xm:sqref>A2:A3</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Issue Type" xr:uid="{28BF52BF-C0B0-4D22-B02F-F1408D5A055B}">
           <x14:formula1>
             <xm:f>Config!$U$4:$U$33</xm:f>
           </x14:formula1>
-          <xm:sqref>B2:B4</xm:sqref>
+          <xm:sqref>B2:B3</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" xr:uid="{7708D6E2-1D6B-41D8-A9EE-0E87219BA8EA}">
           <x14:formula1>
             <xm:f>Config!$G$4:$G$8</xm:f>
           </x14:formula1>
-          <xm:sqref>F2:F4</xm:sqref>
+          <xm:sqref>F2:F3</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2545,66 +2313,66 @@
   <sheetData>
     <row r="1" spans="1:22" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="11" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B1" s="11"/>
       <c r="D1" s="11" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E1" s="11"/>
       <c r="G1" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="I1" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="I1" s="6" t="s">
-        <v>62</v>
-      </c>
       <c r="K1" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="M1" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O1" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q1" s="11" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="R1" s="11"/>
       <c r="S1" s="11"/>
       <c r="U1" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="7"/>
       <c r="D2" s="12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E2" s="12"/>
       <c r="F2" s="7"/>
       <c r="G2" s="10" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H2" s="10"/>
       <c r="I2" s="10" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J2" s="10"/>
       <c r="K2" s="12" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="L2" s="12"/>
       <c r="M2" s="9" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="N2" s="9"/>
       <c r="O2" s="10" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="P2" s="10"/>
       <c r="Q2" s="12"/>
@@ -2612,54 +2380,54 @@
       <c r="S2" s="9"/>
       <c r="T2" s="7"/>
       <c r="U2" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="V2" s="9"/>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G3" t="s">
+        <v>75</v>
+      </c>
+      <c r="I3" t="s">
         <v>74</v>
       </c>
-      <c r="I3" t="s">
+      <c r="K3" t="s">
         <v>73</v>
       </c>
-      <c r="K3" t="s">
+      <c r="M3" t="s">
+        <v>80</v>
+      </c>
+      <c r="O3" t="s">
         <v>72</v>
       </c>
-      <c r="M3" t="s">
-        <v>79</v>
-      </c>
-      <c r="O3" t="s">
-        <v>71</v>
-      </c>
       <c r="Q3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="R3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="S3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B4" t="s">
         <v>50</v>
@@ -2671,10 +2439,10 @@
         <v>1</v>
       </c>
       <c r="G4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K4" t="s">
         <v>39</v>
@@ -2689,7 +2457,7 @@
         <v>31</v>
       </c>
       <c r="R4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="S4" s="7"/>
       <c r="U4" t="str" cm="1">
@@ -2699,7 +2467,7 @@
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B5" t="s">
         <v>51</v>
@@ -2711,10 +2479,10 @@
         <v>2</v>
       </c>
       <c r="G5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K5" t="s">
         <v>37</v>
@@ -2732,7 +2500,7 @@
         <v>40</v>
       </c>
       <c r="S5" s="7" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="U5" t="str">
         <f ca="1"/>
@@ -2741,16 +2509,16 @@
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B6" t="s">
         <v>52</v>
       </c>
       <c r="G6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="K6" t="s">
         <v>41</v>
@@ -2759,16 +2527,16 @@
         <v>33</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>109</v>
+        <v>54</v>
       </c>
       <c r="Q6" t="s">
         <v>49</v>
       </c>
       <c r="R6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="S6" s="7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="U6" t="str">
         <f ca="1"/>
@@ -2779,7 +2547,7 @@
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="I7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="K7" t="s">
         <v>42</v>
@@ -2799,7 +2567,7 @@
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="I8" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="O8" s="1" t="s">
         <v>55</v>
@@ -2813,7 +2581,7 @@
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="I9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="O9" s="1" t="s">
         <v>56</v>
@@ -2827,7 +2595,7 @@
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="I10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="U10" t="str">
         <f ca="1"/>

</xml_diff>

<commit_message>
JT-139 refactor: simplify config_importer.json structure and update ImportTemplate.xlsx
- Removed unnecessary sections and fields from config_importer.json for clarity and maintainability.
- Cleared disabled fixers list in config_importer.json.
- Updated ImportTemplate.xlsx to reflect recent changes in configuration.
</commit_message>
<xml_diff>
--- a/resources/templates/ImportTemplate.xlsx
+++ b/resources/templates/ImportTemplate.xlsx
@@ -8,19 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workdir\DeerHide\sources\jira-toolkit\resources\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC33135F-B90A-4C24-BAC9-7A123C771B85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01FCCE72-DF9E-484F-AFA5-1709264A86F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5376" yWindow="5376" windowWidth="34560" windowHeight="18600" activeTab="1" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
+    <workbookView xWindow="1152" yWindow="1152" windowWidth="34560" windowHeight="18600" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset" sheetId="1" r:id="rId1"/>
     <sheet name="Config" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="cfg_labels_ft_label">Config!$R$6</definedName>
-    <definedName name="cfg_labels_ft_name">Config!$R$6</definedName>
-    <definedName name="cfg_labels_imported">Config!$R$5</definedName>
-    <definedName name="cfg_projectKey">Config!$R$4</definedName>
+    <definedName name="cfg_labels_ft_label">Config!$R$5</definedName>
+    <definedName name="cfg_labels_ft_name">Config!$R$5</definedName>
+    <definedName name="cfg_labels_imported">Config!$R$4</definedName>
+    <definedName name="cfg_projectKey">Config!#REF!</definedName>
     <definedName name="cfg_type_comment">Config!$M$4</definedName>
     <definedName name="cfg_type_note">Config!$M$6</definedName>
     <definedName name="cfg_type_skip">Config!$M$5</definedName>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="106">
   <si>
     <t>IssueType</t>
   </si>
@@ -191,9 +191,6 @@
     <t>Story</t>
   </si>
   <si>
-    <t>imported</t>
-  </si>
-  <si>
     <t>Bug</t>
   </si>
   <si>
@@ -233,9 +230,6 @@
     <t>Highest</t>
   </si>
   <si>
-    <t>Hight</t>
-  </si>
-  <si>
     <t>Lowest</t>
   </si>
   <si>
@@ -245,9 +239,6 @@
     <t>Creation Marker</t>
   </si>
   <si>
-    <t>JV</t>
-  </si>
-  <si>
     <t>Issue Type</t>
   </si>
   <si>
@@ -278,15 +269,6 @@
     <t>Sprint.ID</t>
   </si>
   <si>
-    <t>JITTP Version 1</t>
-  </si>
-  <si>
-    <t>JITTP Version 2</t>
-  </si>
-  <si>
-    <t>JITTP Version 3</t>
-  </si>
-  <si>
     <t>Priority.Name</t>
   </si>
   <si>
@@ -299,12 +281,6 @@
     <t>FixVersion.Name</t>
   </si>
   <si>
-    <t>SysOps</t>
-  </si>
-  <si>
-    <t>DevOps</t>
-  </si>
-  <si>
     <t>Remark</t>
   </si>
   <si>
@@ -356,12 +332,6 @@
     <t>Combined list for the table</t>
   </si>
   <si>
-    <t>1w</t>
-  </si>
-  <si>
-    <t>JITTP2</t>
-  </si>
-  <si>
     <t>Test, Epic</t>
   </si>
   <si>
@@ -371,21 +341,9 @@
     <t>Parent</t>
   </si>
   <si>
-    <t>Design</t>
-  </si>
-  <si>
     <t>Development</t>
   </si>
   <si>
-    <t>Production</t>
-  </si>
-  <si>
-    <t>Quality Assurance</t>
-  </si>
-  <si>
-    <t>Quality Control</t>
-  </si>
-  <si>
     <t>Misc Fields</t>
   </si>
   <si>
@@ -399,6 +357,36 @@
   </si>
   <si>
     <t>pod_test</t>
+  </si>
+  <si>
+    <t>jira.connection.site_address</t>
+  </si>
+  <si>
+    <t>jira.project.key</t>
+  </si>
+  <si>
+    <t>validation.skip_rowtype</t>
+  </si>
+  <si>
+    <t>validation.skip_issuetypes</t>
+  </si>
+  <si>
+    <t>["comment", "note", "skip"]</t>
+  </si>
+  <si>
+    <t>Version_Tag</t>
+  </si>
+  <si>
+    <t>PROJECT KEY</t>
+  </si>
+  <si>
+    <t>jt-imported</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Sub-Task</t>
   </si>
 </sst>
 </file>
@@ -999,7 +987,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="56">
+  <dxfs count="200">
     <dxf>
       <fill>
         <patternFill patternType="darkUp"/>
@@ -1143,10 +1131,430 @@
       </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="darkUp"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDAF2D0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2CEEF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <color theme="0" tint="-0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFF9B1AB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF99CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF6699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="darkUp"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDAF2D0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2CEEF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <color theme="0" tint="-0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFF9B1AB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF99CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF6699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="darkUp"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDAF2D0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2CEEF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <color theme="0" tint="-0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFF9B1AB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF99CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF6699"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <alignment vertical="top"/>
@@ -1289,6 +1697,864 @@
     </dxf>
     <dxf>
       <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="darkUp"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDAF2D0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2CEEF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <color theme="0" tint="-0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFF9B1AB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF99CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF6699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="darkUp"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDAF2D0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2CEEF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <color theme="0" tint="-0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFF9B1AB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF99CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF6699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="darkUp"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDAF2D0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2CEEF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <color theme="0" tint="-0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFF9B1AB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF99CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF6699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="darkUp"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDAF2D0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2CEEF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <color theme="0" tint="-0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFF9B1AB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF99CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF6699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="darkUp"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDAF2D0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2CEEF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <color theme="0" tint="-0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFF9B1AB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF99CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF6699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="darkUp"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDAF2D0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2CEEF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <color theme="0" tint="-0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFF9B1AB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF99CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF6699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1326,57 +2592,57 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" name="JiraDataset" displayName="JiraDataset" ref="A1:AJ3" totalsRowShown="0" headerRowDxfId="55" dataDxfId="54">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" name="JiraDataset" displayName="JiraDataset" ref="A1:AJ3" totalsRowShown="0" headerRowDxfId="101" dataDxfId="100">
   <autoFilter ref="A1:AJ3" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}"/>
   <tableColumns count="36">
-    <tableColumn id="3" xr3:uid="{AF2EC907-349C-4651-852D-6E39C61E17FF}" name="Priority" dataDxfId="53"/>
-    <tableColumn id="2" xr3:uid="{E90C51F2-4386-421F-A3E4-E2CA9D43D396}" name="IssueType" dataDxfId="52"/>
-    <tableColumn id="1" xr3:uid="{BBAD373B-BA13-47E4-9F74-565F4D9E9680}" name="Summary" dataDxfId="51"/>
-    <tableColumn id="4" xr3:uid="{026E5B97-FAFC-4E46-860E-0B0C976B1148}" name="Issue Key" dataDxfId="50"/>
-    <tableColumn id="5" xr3:uid="{A2C262E8-D544-4669-99F1-151EDE081654}" name="Description" dataDxfId="49"/>
-    <tableColumn id="7" xr3:uid="{0FAD1ACC-432E-462C-8B89-71540710BCB5}" name="FixVersion" dataDxfId="48">
+    <tableColumn id="3" xr3:uid="{AF2EC907-349C-4651-852D-6E39C61E17FF}" name="Priority" dataDxfId="99"/>
+    <tableColumn id="2" xr3:uid="{E90C51F2-4386-421F-A3E4-E2CA9D43D396}" name="IssueType" dataDxfId="98"/>
+    <tableColumn id="1" xr3:uid="{BBAD373B-BA13-47E4-9F74-565F4D9E9680}" name="Summary" dataDxfId="97"/>
+    <tableColumn id="4" xr3:uid="{026E5B97-FAFC-4E46-860E-0B0C976B1148}" name="Issue Key" dataDxfId="96"/>
+    <tableColumn id="5" xr3:uid="{A2C262E8-D544-4669-99F1-151EDE081654}" name="Description" dataDxfId="95"/>
+    <tableColumn id="7" xr3:uid="{0FAD1ACC-432E-462C-8B89-71540710BCB5}" name="FixVersion" dataDxfId="94">
       <calculatedColumnFormula>Config!$G$4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="28" xr3:uid="{07F3030C-7187-4B16-BBDB-798304851975}" name="Assignee.Name" dataDxfId="47"/>
-    <tableColumn id="8" xr3:uid="{8C7FB8DB-A85B-4189-93D8-0F0D4EEEF81B}" name="Component" dataDxfId="46"/>
-    <tableColumn id="9" xr3:uid="{DC5101A8-1204-44D2-BC2C-FEE1A4EFE7C1}" name="Sprint Name" dataDxfId="45"/>
-    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="44"/>
-    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="43"/>
-    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="42"/>
-    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="41"/>
-    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="40">
+    <tableColumn id="28" xr3:uid="{07F3030C-7187-4B16-BBDB-798304851975}" name="Assignee.Name" dataDxfId="93"/>
+    <tableColumn id="8" xr3:uid="{8C7FB8DB-A85B-4189-93D8-0F0D4EEEF81B}" name="Component" dataDxfId="92"/>
+    <tableColumn id="9" xr3:uid="{DC5101A8-1204-44D2-BC2C-FEE1A4EFE7C1}" name="Sprint Name" dataDxfId="91"/>
+    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="90"/>
+    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="89"/>
+    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="88"/>
+    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="87"/>
+    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="86">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[IssueType]]="Epic",JiraDataset[[#This Row],[Summary]],"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="27" xr3:uid="{911C8FDC-5528-43FC-BDF4-D4761F03C0E5}" name="Child-Issue" dataDxfId="39"/>
-    <tableColumn id="41" xr3:uid="{AB248E07-9BFA-42CC-BC41-B4234F677BFB}" name="Child-Issue1" dataDxfId="38"/>
-    <tableColumn id="29" xr3:uid="{89D12135-F3E3-4253-844F-1B9A54169953}" name="Child-Issue2" dataDxfId="37"/>
-    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="36"/>
-    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="35"/>
-    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="34"/>
-    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="33"/>
-    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="32"/>
-    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="31"/>
-    <tableColumn id="18" xr3:uid="{16B98070-7F8A-4FC7-AD99-EA81D0BD26AB}" name="Labels6" dataDxfId="30"/>
-    <tableColumn id="19" xr3:uid="{016EAEF4-8EA9-408B-9F1A-ECFB17E81C77}" name="Labels7" dataDxfId="29"/>
-    <tableColumn id="26" xr3:uid="{8263F9EC-BF0A-46F7-BA83-6083A4262B91}" name="Labels8" dataDxfId="28"/>
-    <tableColumn id="20" xr3:uid="{389B11C5-1B22-48C0-BCA2-72F050425FA1}" name="Labels9" dataDxfId="27"/>
-    <tableColumn id="25" xr3:uid="{AE95F8A2-F7F0-4985-9AE6-4201B9792775}" name="Labels10" dataDxfId="26"/>
-    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="25">
+    <tableColumn id="27" xr3:uid="{911C8FDC-5528-43FC-BDF4-D4761F03C0E5}" name="Child-Issue" dataDxfId="85"/>
+    <tableColumn id="41" xr3:uid="{AB248E07-9BFA-42CC-BC41-B4234F677BFB}" name="Child-Issue1" dataDxfId="84"/>
+    <tableColumn id="29" xr3:uid="{89D12135-F3E3-4253-844F-1B9A54169953}" name="Child-Issue2" dataDxfId="83"/>
+    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="82"/>
+    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="81"/>
+    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="80"/>
+    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="79"/>
+    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="78"/>
+    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="77"/>
+    <tableColumn id="18" xr3:uid="{16B98070-7F8A-4FC7-AD99-EA81D0BD26AB}" name="Labels6" dataDxfId="76"/>
+    <tableColumn id="19" xr3:uid="{016EAEF4-8EA9-408B-9F1A-ECFB17E81C77}" name="Labels7" dataDxfId="75"/>
+    <tableColumn id="26" xr3:uid="{8263F9EC-BF0A-46F7-BA83-6083A4262B91}" name="Labels8" dataDxfId="74"/>
+    <tableColumn id="20" xr3:uid="{389B11C5-1B22-48C0-BCA2-72F050425FA1}" name="Labels9" dataDxfId="73"/>
+    <tableColumn id="25" xr3:uid="{AE95F8A2-F7F0-4985-9AE6-4201B9792775}" name="Labels10" dataDxfId="72"/>
+    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="71">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], Config!$D$4:$E$9, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="24">
+    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="70">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="23">
+    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="69">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Feature Pod Label", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="22">
+    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="68">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], Config!$A$4:$B$24, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="21">
-      <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Project Key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
+    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="67">
+      <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("jira.project.key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="20">
+    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="66">
       <calculatedColumnFormula array="1">IF(
   JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
   "",
@@ -1392,7 +2658,7 @@
   )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="19">
+    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="65">
       <calculatedColumnFormula array="1">IFERROR(
     _xlfn.IFS(
         JiraDataset[[#This Row],[IssueType]] = cfg_type_comment,"SKIP",
@@ -1402,15 +2668,15 @@
     cfg_type_workitem
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="18"/>
+    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="64"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{93F2D14D-2ABD-4171-895D-1041B0893491}" name="CfgComponents" displayName="CfgComponents" ref="I3:I10" totalsRowShown="0">
-  <autoFilter ref="I3:I10" xr:uid="{93F2D14D-2ABD-4171-895D-1041B0893491}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{93F2D14D-2ABD-4171-895D-1041B0893491}" name="CfgComponents" displayName="CfgComponents" ref="I3:I5" totalsRowShown="0">
+  <autoFilter ref="I3:I5" xr:uid="{93F2D14D-2ABD-4171-895D-1041B0893491}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{10F6CCA4-1068-4FC8-AB82-E48B87DB0F71}" name="Component.Name"/>
   </tableColumns>
@@ -1419,8 +2685,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{7007FF9D-9384-422B-8DB3-300D782E5FE6}" name="CfgFixVersions" displayName="CfgFixVersions" ref="G3:G6" totalsRowShown="0">
-  <autoFilter ref="G3:G6" xr:uid="{7007FF9D-9384-422B-8DB3-300D782E5FE6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{7007FF9D-9384-422B-8DB3-300D782E5FE6}" name="CfgFixVersions" displayName="CfgFixVersions" ref="G3:G5" totalsRowShown="0">
+  <autoFilter ref="G3:G5" xr:uid="{7007FF9D-9384-422B-8DB3-300D782E5FE6}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{E20FAA91-E54E-42EA-9BFF-2FDA27CD5D33}" name="FixVersion.Name"/>
   </tableColumns>
@@ -1429,8 +2695,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{6F085B8C-1322-4F43-A516-588923936259}" name="CfgIssueTypes" displayName="CfgIssueTypes" ref="K3:K7" totalsRowShown="0">
-  <autoFilter ref="K3:K7" xr:uid="{6F085B8C-1322-4F43-A516-588923936259}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{6F085B8C-1322-4F43-A516-588923936259}" name="CfgIssueTypes" displayName="CfgIssueTypes" ref="K3:K8" totalsRowShown="0">
+  <autoFilter ref="K3:K8" xr:uid="{6F085B8C-1322-4F43-A516-588923936259}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{A92436BC-3156-493F-B5C6-0BB6B51F89EB}" name="IssueType.Name"/>
   </tableColumns>
@@ -1442,7 +2708,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}" name="CfgPriorities" displayName="CfgPriorities" ref="O3:O9" totalsRowShown="0">
   <autoFilter ref="O3:O9" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="17"/>
+    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="199"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1471,12 +2737,12 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{383560BC-B1F2-44B6-B877-188131EFA163}" name="CfgAutofieldValues" displayName="CfgAutofieldValues" ref="Q3:S6" totalsRowShown="0">
-  <autoFilter ref="Q3:S6" xr:uid="{383560BC-B1F2-44B6-B877-188131EFA163}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{383560BC-B1F2-44B6-B877-188131EFA163}" name="CfgAutofieldValues" displayName="CfgAutofieldValues" ref="Q3:S9" totalsRowShown="0">
+  <autoFilter ref="Q3:S9" xr:uid="{383560BC-B1F2-44B6-B877-188131EFA163}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{D4E1611F-A2CF-465D-A219-1759EA66687D}" name="Name"/>
     <tableColumn id="2" xr3:uid="{174D0D86-B1AA-4BF7-AC91-FCACFC898851}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Remark" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Remark" dataDxfId="198"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1880,7 +3146,7 @@
         <v>10</v>
       </c>
       <c r="L1" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="M1" s="3" t="s">
         <v>11</v>
@@ -1949,7 +3215,7 @@
         <v>32</v>
       </c>
       <c r="AI1" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="AJ1" s="3" t="s">
         <v>33</v>
@@ -1972,7 +3238,7 @@
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
       <c r="J2" s="3" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="K2" s="3">
         <v>1</v>
@@ -2014,7 +3280,7 @@
         <v/>
       </c>
       <c r="AG2" s="3" t="str">
-        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Project Key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
+        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("jira.project.key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
         <v/>
       </c>
       <c r="AH2" s="3" t="str" cm="1">
@@ -2049,33 +3315,31 @@
     </row>
     <row r="3" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>71</v>
+        <v>101</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>58</v>
+        <v>92</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>95</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="J3" s="3"/>
       <c r="K3" s="3">
         <v>2</v>
       </c>
@@ -2105,7 +3369,7 @@
       </c>
       <c r="AD3" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
-        <v>imported</v>
+        <v>jt-imported</v>
       </c>
       <c r="AE3" s="8" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Feature Pod Label", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
@@ -2113,13 +3377,13 @@
       </c>
       <c r="AF3" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], Config!$A$4:$B$24, 2, FALSE), ""))</f>
-        <v/>
+        <v>712020:e4e815aa-df03-418a-9760-3e70901b6ec5</v>
       </c>
       <c r="AG3" s="3" t="str">
-        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Project Key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
-        <v>JITTP2</v>
-      </c>
-      <c r="AH3" s="3" cm="1">
+        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("jira.project.key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
+        <v>PROJECT KEY</v>
+      </c>
+      <c r="AH3" s="3" t="str" cm="1">
         <f t="array" ref="AH3">IF(
   JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
   "",
@@ -2134,7 +3398,7 @@
     IF(_xlpm.seconds=0, "", _xlpm.seconds*60)
   )
 )</f>
-        <v>8640000</v>
+        <v/>
       </c>
       <c r="AI3" s="3" t="str" cm="1">
         <f t="array" ref="AI3">IFERROR(
@@ -2151,7 +3415,7 @@
     </row>
   </sheetData>
   <protectedRanges>
-    <protectedRange sqref="A1:A1048576 D4:N1048576 P4:AD1048576 C1:AB3" name="User Input"/>
+    <protectedRange sqref="D4:N1048576 P4:AD1048576 C1:AB3 A1:A1048576" name="User Input"/>
     <protectedRange algorithmName="SHA-512" hashValue="tpheD+JLADkhiyalt6vInlMwkILPZx4PVQN/k2vmwjOBdYUuHaXCrwtObHeFz5dJh9f853O84pZ1Rn9Ujz33+A==" saltValue="9ir5NB4CJc/69S/Eh84/mA==" spinCount="100000" sqref="AC1:AI3 AE4:AK1048576" name="Computed values"/>
   </protectedRanges>
   <phoneticPr fontId="18" type="noConversion"/>
@@ -2236,7 +3500,7 @@
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="It must be a number (integer). This reference is only used during the import process." sqref="K1" xr:uid="{9C637146-F2E3-4D08-87A8-F70FD358E47E}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Use the Issue ID value to link this work item to an Epic_x000a__x000a_Story Issues are not Child-Issues and should have Epic Link instead. " sqref="M1" xr:uid="{A61138FD-C2B2-49D2-810B-69EAE2230B73}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="This field should be the Issue ID or Issue Key of the child tasks. (upstream linkage is not possible)._x000a__x000a__x000a_To link Epics and Stories, use the Epic Link from the Story Issue." sqref="O1:Q1" xr:uid="{BE6B7503-A11A-4130-9D63-988F0CFED80E}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="AUTOMATIC FIELD" prompt="Do not manually edit these!" sqref="AF2:AH3 AC2:AC3 AF1:AH1" xr:uid="{893DA5FE-9FD0-4D28-BBD0-3D7AEDECEACB}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="AUTOMATIC FIELD" prompt="Do not manually edit these!" sqref="AC2:AC3 AF1:AH3" xr:uid="{893DA5FE-9FD0-4D28-BBD0-3D7AEDECEACB}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="H2:H3" xr:uid="{65EDED96-6789-400B-B504-6BC3F5A79E70}">
       <formula1>INDIRECT("CfgComponents[Component.Name]")</formula1>
     </dataValidation>
@@ -2313,66 +3577,66 @@
   <sheetData>
     <row r="1" spans="1:22" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="11" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="B1" s="11"/>
       <c r="D1" s="11" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="E1" s="11"/>
       <c r="G1" s="6" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="M1" s="6" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="O1" s="6" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="Q1" s="11" t="s">
-        <v>105</v>
+        <v>91</v>
       </c>
       <c r="R1" s="11"/>
       <c r="S1" s="11"/>
       <c r="U1" s="6" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="7"/>
       <c r="D2" s="12" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="E2" s="12"/>
       <c r="F2" s="7"/>
       <c r="G2" s="10" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="H2" s="10"/>
       <c r="I2" s="10" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="J2" s="10"/>
       <c r="K2" s="12" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="L2" s="12"/>
       <c r="M2" s="9" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="N2" s="9"/>
       <c r="O2" s="10" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="P2" s="10"/>
       <c r="Q2" s="12"/>
@@ -2380,69 +3644,69 @@
       <c r="S2" s="9"/>
       <c r="T2" s="7"/>
       <c r="U2" s="9" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="V2" s="9"/>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E3" t="s">
         <v>65</v>
       </c>
-      <c r="B3" t="s">
+      <c r="G3" t="s">
+        <v>69</v>
+      </c>
+      <c r="I3" t="s">
+        <v>68</v>
+      </c>
+      <c r="K3" t="s">
+        <v>67</v>
+      </c>
+      <c r="M3" t="s">
+        <v>72</v>
+      </c>
+      <c r="O3" t="s">
         <v>66</v>
       </c>
-      <c r="D3" t="s">
+      <c r="Q3" t="s">
+        <v>58</v>
+      </c>
+      <c r="R3" t="s">
+        <v>59</v>
+      </c>
+      <c r="S3" t="s">
+        <v>70</v>
+      </c>
+      <c r="U3" s="5" t="s">
         <v>67</v>
-      </c>
-      <c r="E3" t="s">
-        <v>68</v>
-      </c>
-      <c r="G3" t="s">
-        <v>75</v>
-      </c>
-      <c r="I3" t="s">
-        <v>74</v>
-      </c>
-      <c r="K3" t="s">
-        <v>73</v>
-      </c>
-      <c r="M3" t="s">
-        <v>80</v>
-      </c>
-      <c r="O3" t="s">
-        <v>72</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>61</v>
-      </c>
-      <c r="R3" t="s">
-        <v>62</v>
-      </c>
-      <c r="S3" t="s">
-        <v>78</v>
-      </c>
-      <c r="U3" s="5" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="B4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E4">
         <v>1</v>
       </c>
       <c r="G4" t="s">
-        <v>69</v>
+        <v>101</v>
       </c>
       <c r="I4" t="s">
-        <v>76</v>
+        <v>90</v>
       </c>
       <c r="K4" t="s">
         <v>39</v>
@@ -2454,53 +3718,49 @@
         <v>38</v>
       </c>
       <c r="Q4" t="s">
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="R4" t="s">
-        <v>96</v>
-      </c>
-      <c r="S4" s="7"/>
+        <v>103</v>
+      </c>
+      <c r="S4" s="7" t="s">
+        <v>77</v>
+      </c>
       <c r="U4" t="str" cm="1">
-        <f t="array" aca="1" ref="U4:U11" ca="1">_xlfn.UNIQUE((_xlfn.VSTACK(INDIRECT("CfgIssueTypes[IssueType.Name]"),INDIRECT("CfgIgnoreList[IgnoreList.Name]"))))</f>
+        <f t="array" aca="1" ref="U4:U12" ca="1">_xlfn.UNIQUE((_xlfn.VSTACK(INDIRECT("CfgIssueTypes[IssueType.Name]"),INDIRECT("CfgIgnoreList[IgnoreList.Name]"))))</f>
         <v>Story</v>
       </c>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="B5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E5">
         <v>2</v>
       </c>
-      <c r="G5" t="s">
-        <v>70</v>
-      </c>
-      <c r="I5" t="s">
-        <v>77</v>
-      </c>
       <c r="K5" t="s">
         <v>37</v>
       </c>
       <c r="M5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="Q5" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="R5" t="s">
-        <v>40</v>
+        <v>95</v>
       </c>
       <c r="S5" s="7" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="U5" t="str">
         <f ca="1"/>
@@ -2509,35 +3769,24 @@
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>108</v>
+        <v>94</v>
       </c>
       <c r="B6" t="s">
-        <v>52</v>
-      </c>
-      <c r="G6" t="s">
-        <v>71</v>
-      </c>
-      <c r="I6" t="s">
-        <v>100</v>
+        <v>51</v>
       </c>
       <c r="K6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="M6" t="s">
         <v>33</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>54</v>
+        <v>104</v>
       </c>
       <c r="Q6" t="s">
-        <v>49</v>
-      </c>
-      <c r="R6" t="s">
-        <v>109</v>
-      </c>
-      <c r="S6" s="7" t="s">
-        <v>86</v>
-      </c>
+        <v>96</v>
+      </c>
+      <c r="S6" s="7"/>
       <c r="U6" t="str">
         <f ca="1"/>
         <v>Bug</v>
@@ -2546,18 +3795,22 @@
     <row r="7" spans="1:22" x14ac:dyDescent="0.3">
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
-      <c r="I7" t="s">
-        <v>101</v>
-      </c>
       <c r="K7" t="s">
+        <v>41</v>
+      </c>
+      <c r="M7" t="s">
+        <v>45</v>
+      </c>
+      <c r="O7" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="M7" t="s">
-        <v>46</v>
-      </c>
-      <c r="O7" s="1" t="s">
-        <v>43</v>
-      </c>
+      <c r="Q7" t="s">
+        <v>97</v>
+      </c>
+      <c r="R7" t="s">
+        <v>102</v>
+      </c>
+      <c r="S7" s="7"/>
       <c r="U7" t="str">
         <f ca="1"/>
         <v>Epic</v>
@@ -2566,40 +3819,48 @@
     <row r="8" spans="1:22" x14ac:dyDescent="0.3">
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
-      <c r="I8" t="s">
-        <v>102</v>
+      <c r="K8" t="s">
+        <v>105</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>55</v>
-      </c>
+        <v>53</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>98</v>
+      </c>
+      <c r="R8" t="b">
+        <v>1</v>
+      </c>
+      <c r="S8" s="7"/>
       <c r="U8" t="str">
         <f ca="1"/>
-        <v>Comment</v>
+        <v>Sub-Task</v>
       </c>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.3">
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
-      <c r="I9" t="s">
-        <v>103</v>
-      </c>
       <c r="O9" s="1" t="s">
-        <v>56</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>99</v>
+      </c>
+      <c r="R9" t="s">
+        <v>100</v>
+      </c>
+      <c r="S9" s="7"/>
       <c r="U9" t="str">
         <f ca="1"/>
-        <v>Skip</v>
+        <v>Comment</v>
       </c>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.3">
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
-      <c r="I10" t="s">
-        <v>104</v>
-      </c>
       <c r="U10" t="str">
         <f ca="1"/>
-        <v>Note</v>
+        <v>Skip</v>
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.3">
@@ -2607,12 +3868,16 @@
       <c r="E11" s="2"/>
       <c r="U11" t="str">
         <f ca="1"/>
-        <v>WorkItem</v>
+        <v>Note</v>
       </c>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.3">
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
+      <c r="U12" t="str">
+        <f ca="1"/>
+        <v>WorkItem</v>
+      </c>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.3">
       <c r="D13" s="2"/>

</xml_diff>

<commit_message>
JT-139 Fix: ImportTemplate.xlsx FixVersion Excel autofill logic
</commit_message>
<xml_diff>
--- a/resources/templates/ImportTemplate.xlsx
+++ b/resources/templates/ImportTemplate.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workdir\DeerHide\sources\jira-toolkit\resources\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workdir\DeerHide\sources\jira-toolkit\resources\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01FCCE72-DF9E-484F-AFA5-1709264A86F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC11B61B-52F2-4383-A081-3EA527C8CFCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1152" yWindow="1152" windowWidth="34560" windowHeight="18600" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
+    <workbookView xWindow="3156" yWindow="6612" windowWidth="34560" windowHeight="18600" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <definedName name="cfg_labels_ft_label">Config!$R$5</definedName>
     <definedName name="cfg_labels_ft_name">Config!$R$5</definedName>
     <definedName name="cfg_labels_imported">Config!$R$4</definedName>
-    <definedName name="cfg_projectKey">Config!#REF!</definedName>
+    <definedName name="cfg_projectKey">Config!$R$7</definedName>
     <definedName name="cfg_type_comment">Config!$M$4</definedName>
     <definedName name="cfg_type_note">Config!$M$6</definedName>
     <definedName name="cfg_type_skip">Config!$M$5</definedName>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="101">
   <si>
     <t>IssueType</t>
   </si>
@@ -212,21 +212,9 @@
     <t>Sprint 1</t>
   </si>
   <si>
-    <t>Sprint 2</t>
-  </si>
-  <si>
     <t>Feature Pod Label</t>
   </si>
   <si>
-    <t>712020:e4e815aa-df03-418a-9760-3e70901b6ec5</t>
-  </si>
-  <si>
-    <t>712020:69ead6b8-698d-48a8-8abb-b55246f6cb7c</t>
-  </si>
-  <si>
-    <t>712020:63630dfe-2a04-4021-9f7b-53445ba456e7</t>
-  </si>
-  <si>
     <t>Highest</t>
   </si>
   <si>
@@ -347,15 +335,6 @@
     <t>Misc Fields</t>
   </si>
   <si>
-    <t>tom4897</t>
-  </si>
-  <si>
-    <t>Nakool</t>
-  </si>
-  <si>
-    <t>MirageCentury</t>
-  </si>
-  <si>
     <t>pod_test</t>
   </si>
   <si>
@@ -387,6 +366,12 @@
   </si>
   <si>
     <t>Sub-Task</t>
+  </si>
+  <si>
+    <t>AtlassianID (cloud) or Email (DC)</t>
+  </si>
+  <si>
+    <t>4w</t>
   </si>
 </sst>
 </file>
@@ -987,7 +972,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="200">
+  <dxfs count="72">
     <dxf>
       <fill>
         <patternFill patternType="darkUp"/>
@@ -1079,6 +1064,17 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF6699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor auto="1"/>
@@ -1116,17 +1112,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFF99CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6699"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1221,6 +1206,17 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF6699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor auto="1"/>
@@ -1262,301 +1258,6 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="darkUp"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDAF2D0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2CEEF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.89996032593768116"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <strike val="0"/>
-        <color theme="0" tint="-0.34998626667073579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFF9B1AB"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCC99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9999"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF99CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="darkUp"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDAF2D0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2CEEF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.89996032593768116"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <strike val="0"/>
-        <color theme="0" tint="-0.34998626667073579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFF9B1AB"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCC99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9999"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF99CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <alignment vertical="top"/>
     </dxf>
     <dxf>
@@ -1697,858 +1398,6 @@
     </dxf>
     <dxf>
       <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="darkUp"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDAF2D0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2CEEF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.89996032593768116"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <strike val="0"/>
-        <color theme="0" tint="-0.34998626667073579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFF9B1AB"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCC99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9999"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF99CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="darkUp"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDAF2D0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2CEEF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.89996032593768116"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <strike val="0"/>
-        <color theme="0" tint="-0.34998626667073579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFF9B1AB"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCC99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9999"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF99CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="darkUp"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDAF2D0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2CEEF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.89996032593768116"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <strike val="0"/>
-        <color theme="0" tint="-0.34998626667073579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFF9B1AB"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCC99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9999"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF99CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="darkUp"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDAF2D0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2CEEF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.89996032593768116"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <strike val="0"/>
-        <color theme="0" tint="-0.34998626667073579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFF9B1AB"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCC99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9999"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF99CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="darkUp"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDAF2D0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2CEEF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.89996032593768116"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <strike val="0"/>
-        <color theme="0" tint="-0.34998626667073579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFF9B1AB"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCC99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9999"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF99CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="darkUp"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDAF2D0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2CEEF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.89996032593768116"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <strike val="0"/>
-        <color theme="0" tint="-0.34998626667073579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFF9B1AB"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCC99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9999"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF99CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6699"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
@@ -2592,57 +1441,57 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" name="JiraDataset" displayName="JiraDataset" ref="A1:AJ3" totalsRowShown="0" headerRowDxfId="101" dataDxfId="100">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" name="JiraDataset" displayName="JiraDataset" ref="A1:AJ3" totalsRowShown="0" headerRowDxfId="69" dataDxfId="68">
   <autoFilter ref="A1:AJ3" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}"/>
   <tableColumns count="36">
-    <tableColumn id="3" xr3:uid="{AF2EC907-349C-4651-852D-6E39C61E17FF}" name="Priority" dataDxfId="99"/>
-    <tableColumn id="2" xr3:uid="{E90C51F2-4386-421F-A3E4-E2CA9D43D396}" name="IssueType" dataDxfId="98"/>
-    <tableColumn id="1" xr3:uid="{BBAD373B-BA13-47E4-9F74-565F4D9E9680}" name="Summary" dataDxfId="97"/>
-    <tableColumn id="4" xr3:uid="{026E5B97-FAFC-4E46-860E-0B0C976B1148}" name="Issue Key" dataDxfId="96"/>
-    <tableColumn id="5" xr3:uid="{A2C262E8-D544-4669-99F1-151EDE081654}" name="Description" dataDxfId="95"/>
-    <tableColumn id="7" xr3:uid="{0FAD1ACC-432E-462C-8B89-71540710BCB5}" name="FixVersion" dataDxfId="94">
+    <tableColumn id="3" xr3:uid="{AF2EC907-349C-4651-852D-6E39C61E17FF}" name="Priority" dataDxfId="67"/>
+    <tableColumn id="2" xr3:uid="{E90C51F2-4386-421F-A3E4-E2CA9D43D396}" name="IssueType" dataDxfId="66"/>
+    <tableColumn id="1" xr3:uid="{BBAD373B-BA13-47E4-9F74-565F4D9E9680}" name="Summary" dataDxfId="65"/>
+    <tableColumn id="4" xr3:uid="{026E5B97-FAFC-4E46-860E-0B0C976B1148}" name="Issue Key" dataDxfId="64"/>
+    <tableColumn id="5" xr3:uid="{A2C262E8-D544-4669-99F1-151EDE081654}" name="Description" dataDxfId="63"/>
+    <tableColumn id="7" xr3:uid="{0FAD1ACC-432E-462C-8B89-71540710BCB5}" name="FixVersion" dataDxfId="62">
       <calculatedColumnFormula>Config!$G$4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="28" xr3:uid="{07F3030C-7187-4B16-BBDB-798304851975}" name="Assignee.Name" dataDxfId="93"/>
-    <tableColumn id="8" xr3:uid="{8C7FB8DB-A85B-4189-93D8-0F0D4EEEF81B}" name="Component" dataDxfId="92"/>
-    <tableColumn id="9" xr3:uid="{DC5101A8-1204-44D2-BC2C-FEE1A4EFE7C1}" name="Sprint Name" dataDxfId="91"/>
-    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="90"/>
-    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="89"/>
-    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="88"/>
-    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="87"/>
-    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="86">
+    <tableColumn id="28" xr3:uid="{07F3030C-7187-4B16-BBDB-798304851975}" name="Assignee.Name" dataDxfId="61"/>
+    <tableColumn id="8" xr3:uid="{8C7FB8DB-A85B-4189-93D8-0F0D4EEEF81B}" name="Component" dataDxfId="60"/>
+    <tableColumn id="9" xr3:uid="{DC5101A8-1204-44D2-BC2C-FEE1A4EFE7C1}" name="Sprint Name" dataDxfId="59"/>
+    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="58"/>
+    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="57"/>
+    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="56"/>
+    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="55"/>
+    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="54">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[IssueType]]="Epic",JiraDataset[[#This Row],[Summary]],"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="27" xr3:uid="{911C8FDC-5528-43FC-BDF4-D4761F03C0E5}" name="Child-Issue" dataDxfId="85"/>
-    <tableColumn id="41" xr3:uid="{AB248E07-9BFA-42CC-BC41-B4234F677BFB}" name="Child-Issue1" dataDxfId="84"/>
-    <tableColumn id="29" xr3:uid="{89D12135-F3E3-4253-844F-1B9A54169953}" name="Child-Issue2" dataDxfId="83"/>
-    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="82"/>
-    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="81"/>
-    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="80"/>
-    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="79"/>
-    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="78"/>
-    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="77"/>
-    <tableColumn id="18" xr3:uid="{16B98070-7F8A-4FC7-AD99-EA81D0BD26AB}" name="Labels6" dataDxfId="76"/>
-    <tableColumn id="19" xr3:uid="{016EAEF4-8EA9-408B-9F1A-ECFB17E81C77}" name="Labels7" dataDxfId="75"/>
-    <tableColumn id="26" xr3:uid="{8263F9EC-BF0A-46F7-BA83-6083A4262B91}" name="Labels8" dataDxfId="74"/>
-    <tableColumn id="20" xr3:uid="{389B11C5-1B22-48C0-BCA2-72F050425FA1}" name="Labels9" dataDxfId="73"/>
-    <tableColumn id="25" xr3:uid="{AE95F8A2-F7F0-4985-9AE6-4201B9792775}" name="Labels10" dataDxfId="72"/>
-    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="71">
+    <tableColumn id="27" xr3:uid="{911C8FDC-5528-43FC-BDF4-D4761F03C0E5}" name="Child-Issue" dataDxfId="53"/>
+    <tableColumn id="41" xr3:uid="{AB248E07-9BFA-42CC-BC41-B4234F677BFB}" name="Child-Issue1" dataDxfId="52"/>
+    <tableColumn id="29" xr3:uid="{89D12135-F3E3-4253-844F-1B9A54169953}" name="Child-Issue2" dataDxfId="51"/>
+    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="50"/>
+    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="49"/>
+    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="48"/>
+    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="47"/>
+    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="46"/>
+    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="45"/>
+    <tableColumn id="18" xr3:uid="{16B98070-7F8A-4FC7-AD99-EA81D0BD26AB}" name="Labels6" dataDxfId="44"/>
+    <tableColumn id="19" xr3:uid="{016EAEF4-8EA9-408B-9F1A-ECFB17E81C77}" name="Labels7" dataDxfId="43"/>
+    <tableColumn id="26" xr3:uid="{8263F9EC-BF0A-46F7-BA83-6083A4262B91}" name="Labels8" dataDxfId="42"/>
+    <tableColumn id="20" xr3:uid="{389B11C5-1B22-48C0-BCA2-72F050425FA1}" name="Labels9" dataDxfId="41"/>
+    <tableColumn id="25" xr3:uid="{AE95F8A2-F7F0-4985-9AE6-4201B9792775}" name="Labels10" dataDxfId="40"/>
+    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="39">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], Config!$D$4:$E$9, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="70">
+    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="38">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="69">
+    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="37">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Feature Pod Label", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="68">
+    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="36">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], Config!$A$4:$B$24, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="67">
+    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="35">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("jira.project.key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="66">
+    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="34">
       <calculatedColumnFormula array="1">IF(
   JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
   "",
@@ -2658,7 +1507,7 @@
   )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="65">
+    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="33">
       <calculatedColumnFormula array="1">IFERROR(
     _xlfn.IFS(
         JiraDataset[[#This Row],[IssueType]] = cfg_type_comment,"SKIP",
@@ -2668,7 +1517,7 @@
     cfg_type_workitem
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="64"/>
+    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="32"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2708,15 +1557,15 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}" name="CfgPriorities" displayName="CfgPriorities" ref="O3:O9" totalsRowShown="0">
   <autoFilter ref="O3:O9" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="199"/>
+    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="71"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{1EF5833D-4918-4C71-A990-1B275126361D}" name="CfgAssignees" displayName="CfgAssignees" ref="A3:B6" totalsRowShown="0">
-  <autoFilter ref="A3:B6" xr:uid="{1EF5833D-4918-4C71-A990-1B275126361D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{1EF5833D-4918-4C71-A990-1B275126361D}" name="CfgAssignees" displayName="CfgAssignees" ref="A3:B5" totalsRowShown="0">
+  <autoFilter ref="A3:B5" xr:uid="{1EF5833D-4918-4C71-A990-1B275126361D}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{7F7B4E10-E51C-443F-875D-3E6A9FD9994C}" name="Asssignee.Name"/>
     <tableColumn id="2" xr3:uid="{3A4C6F03-89A9-4E38-8288-00D055D51CD3}" name="Assignee.ID"/>
@@ -2742,7 +1591,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{D4E1611F-A2CF-465D-A219-1759EA66687D}" name="Name"/>
     <tableColumn id="2" xr3:uid="{174D0D86-B1AA-4BF7-AC91-FCACFC898851}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Remark" dataDxfId="198"/>
+    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Remark" dataDxfId="70"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3146,7 +1995,7 @@
         <v>10</v>
       </c>
       <c r="L1" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="M1" s="3" t="s">
         <v>11</v>
@@ -3238,7 +2087,7 @@
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
       <c r="J2" s="3" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="K2" s="3">
         <v>1</v>
@@ -3315,31 +2164,33 @@
     </row>
     <row r="3" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>41</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>92</v>
+        <v>54</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="J3" s="3"/>
+      <c r="J3" s="3" t="s">
+        <v>100</v>
+      </c>
       <c r="K3" s="3">
         <v>2</v>
       </c>
@@ -3377,13 +2228,13 @@
       </c>
       <c r="AF3" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], Config!$A$4:$B$24, 2, FALSE), ""))</f>
-        <v>712020:e4e815aa-df03-418a-9760-3e70901b6ec5</v>
+        <v>AtlassianID (cloud) or Email (DC)</v>
       </c>
       <c r="AG3" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("jira.project.key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
         <v>PROJECT KEY</v>
       </c>
-      <c r="AH3" s="3" t="str" cm="1">
+      <c r="AH3" s="3" cm="1">
         <f t="array" ref="AH3">IF(
   JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
   "",
@@ -3398,7 +2249,7 @@
     IF(_xlpm.seconds=0, "", _xlpm.seconds*60)
   )
 )</f>
-        <v/>
+        <v>34560000</v>
       </c>
       <c r="AI3" s="3" t="str" cm="1">
         <f t="array" ref="AI3">IFERROR(
@@ -3420,22 +2271,24 @@
   </protectedRanges>
   <phoneticPr fontId="18" type="noConversion"/>
   <conditionalFormatting sqref="A2:A3 C2:C3">
-    <cfRule type="containsText" dxfId="15" priority="429" operator="containsText" text="blocker">
-      <formula>NOT(ISERROR(SEARCH("blocker",A2)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="430" operator="containsText" text="critical">
+    <cfRule type="containsText" dxfId="15" priority="430" operator="containsText" text="critical">
       <formula>NOT(ISERROR(SEARCH("critical",A2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="13" priority="431" operator="containsText" text="High">
+    <cfRule type="containsText" dxfId="14" priority="431" operator="containsText" text="High">
       <formula>NOT(ISERROR(SEARCH("High",A2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="12" priority="432" operator="containsText" text="Medium">
+    <cfRule type="containsText" dxfId="13" priority="432" operator="containsText" text="Medium">
       <formula>NOT(ISERROR(SEARCH("Medium",A2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:A3">
-    <cfRule type="containsBlanks" dxfId="11" priority="493">
+    <cfRule type="containsBlanks" dxfId="12" priority="493">
       <formula>LEN(TRIM(A2))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:C3">
+    <cfRule type="containsText" dxfId="11" priority="429" operator="containsText" text="blocker">
+      <formula>NOT(ISERROR(SEARCH("blocker",A2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:AJ3">
@@ -3481,7 +2334,7 @@
       <formula>LEN(TRIM(K2))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations xWindow="1573" yWindow="665" count="20">
+  <dataValidations xWindow="1573" yWindow="665" count="21">
     <dataValidation type="whole" allowBlank="1" showErrorMessage="1" prompt="It must be a number (integer). This reference is only used during the import process." sqref="K2:L3" xr:uid="{005E18F2-4447-4781-8F18-5A58920A4F75}">
       <formula1>1</formula1>
       <formula2>1000</formula2>
@@ -3504,7 +2357,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="H2:H3" xr:uid="{65EDED96-6789-400B-B504-6BC3F5A79E70}">
       <formula1>INDIRECT("CfgComponents[Component.Name]")</formula1>
     </dataValidation>
-    <dataValidation type="list" errorStyle="warning" showErrorMessage="1" error="must be a valid fixversion" sqref="G2:G3" xr:uid="{44FDC20A-8BF5-49B5-9D2C-3A1FE5A7D835}">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" error="must be a valid fixversion" sqref="G2:G3" xr:uid="{44FDC20A-8BF5-49B5-9D2C-3A1FE5A7D835}">
       <formula1>INDIRECT("CfgAssignees[Asssignee.Name]")</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="I2:I3" xr:uid="{A898E2E7-BC45-4B88-BA1E-4AAA377361D4}">
@@ -3517,6 +2370,9 @@
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="Creation Marker (Config Sheet)" prompt="Do not manually edit these!" sqref="AD1:AD3" xr:uid="{412C516D-E091-4DDD-9C14-C33AC653C143}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="Feature Pod Label (Config Sheet)" prompt="Do not manually edit these!" sqref="AE1:AE3" xr:uid="{D2234141-379F-4413-AB08-6835BD9FF967}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="AUTOMATIC FIELD" prompt="Do not manually edit these! SKIP types won't be imported into Jira" sqref="AI1:AI3" xr:uid="{5A336857-7D14-4900-8734-BED680BE5154}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" sqref="F2:F3" xr:uid="{7708D6E2-1D6B-41D8-A9EE-0E87219BA8EA}">
+      <formula1>INDIRECT("CfgFixVersions[FixVersion.Name]")</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -3525,7 +2381,7 @@
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xWindow="1573" yWindow="665" count="3">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xWindow="1573" yWindow="665" count="2">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{5EEBB8D5-878D-4D0E-9267-0919B5A1B925}">
           <x14:formula1>
             <xm:f>Config!$O$4:$O$10</xm:f>
@@ -3537,12 +2393,6 @@
             <xm:f>Config!$U$4:$U$33</xm:f>
           </x14:formula1>
           <xm:sqref>B2:B3</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" xr:uid="{7708D6E2-1D6B-41D8-A9EE-0E87219BA8EA}">
-          <x14:formula1>
-            <xm:f>Config!$G$4:$G$8</xm:f>
-          </x14:formula1>
-          <xm:sqref>F2:F3</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -3577,66 +2427,66 @@
   <sheetData>
     <row r="1" spans="1:22" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="11" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B1" s="11"/>
       <c r="D1" s="11" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E1" s="11"/>
       <c r="G1" s="6" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="M1" s="6" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="O1" s="6" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="Q1" s="11" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="R1" s="11"/>
       <c r="S1" s="11"/>
       <c r="U1" s="6" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="7"/>
       <c r="D2" s="12" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="E2" s="12"/>
       <c r="F2" s="7"/>
       <c r="G2" s="10" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="H2" s="10"/>
       <c r="I2" s="10" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="J2" s="10"/>
       <c r="K2" s="12" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="L2" s="12"/>
       <c r="M2" s="9" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="N2" s="9"/>
       <c r="O2" s="10" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="P2" s="10"/>
       <c r="Q2" s="12"/>
@@ -3644,57 +2494,57 @@
       <c r="S2" s="9"/>
       <c r="T2" s="7"/>
       <c r="U2" s="9" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="V2" s="9"/>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D3" t="s">
+        <v>60</v>
+      </c>
+      <c r="E3" t="s">
+        <v>61</v>
+      </c>
+      <c r="G3" t="s">
+        <v>65</v>
+      </c>
+      <c r="I3" t="s">
+        <v>64</v>
+      </c>
+      <c r="K3" t="s">
+        <v>63</v>
+      </c>
+      <c r="M3" t="s">
+        <v>68</v>
+      </c>
+      <c r="O3" t="s">
         <v>62</v>
       </c>
-      <c r="B3" t="s">
+      <c r="Q3" t="s">
+        <v>54</v>
+      </c>
+      <c r="R3" t="s">
+        <v>55</v>
+      </c>
+      <c r="S3" t="s">
+        <v>66</v>
+      </c>
+      <c r="U3" s="5" t="s">
         <v>63</v>
-      </c>
-      <c r="D3" t="s">
-        <v>64</v>
-      </c>
-      <c r="E3" t="s">
-        <v>65</v>
-      </c>
-      <c r="G3" t="s">
-        <v>69</v>
-      </c>
-      <c r="I3" t="s">
-        <v>68</v>
-      </c>
-      <c r="K3" t="s">
-        <v>67</v>
-      </c>
-      <c r="M3" t="s">
-        <v>72</v>
-      </c>
-      <c r="O3" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>58</v>
-      </c>
-      <c r="R3" t="s">
-        <v>59</v>
-      </c>
-      <c r="S3" t="s">
-        <v>70</v>
-      </c>
-      <c r="U3" s="5" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>92</v>
+        <v>54</v>
       </c>
       <c r="B4" t="s">
-        <v>49</v>
+        <v>99</v>
       </c>
       <c r="D4" t="s">
         <v>46</v>
@@ -3703,10 +2553,10 @@
         <v>1</v>
       </c>
       <c r="G4" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="I4" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="K4" t="s">
         <v>39</v>
@@ -3718,13 +2568,13 @@
         <v>38</v>
       </c>
       <c r="Q4" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="R4" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="S4" s="7" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="U4" t="str" cm="1">
         <f t="array" aca="1" ref="U4:U12" ca="1">_xlfn.UNIQUE((_xlfn.VSTACK(INDIRECT("CfgIssueTypes[IssueType.Name]"),INDIRECT("CfgIgnoreList[IgnoreList.Name]"))))</f>
@@ -3732,18 +2582,6 @@
       </c>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B5" t="s">
-        <v>50</v>
-      </c>
-      <c r="D5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E5">
-        <v>2</v>
-      </c>
       <c r="K5" t="s">
         <v>37</v>
       </c>
@@ -3751,16 +2589,16 @@
         <v>44</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="Q5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="R5" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="S5" s="7" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="U5" t="str">
         <f ca="1"/>
@@ -3768,12 +2606,6 @@
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>94</v>
-      </c>
-      <c r="B6" t="s">
-        <v>51</v>
-      </c>
       <c r="K6" t="s">
         <v>40</v>
       </c>
@@ -3781,10 +2613,10 @@
         <v>33</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="Q6" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="S6" s="7"/>
       <c r="U6" t="str">
@@ -3805,10 +2637,10 @@
         <v>42</v>
       </c>
       <c r="Q7" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="R7" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="S7" s="7"/>
       <c r="U7" t="str">
@@ -3820,13 +2652,13 @@
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="K8" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="Q8" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="R8" t="b">
         <v>1</v>
@@ -3841,13 +2673,13 @@
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="O9" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="Q9" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="R9" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="S9" s="7"/>
       <c r="U9" t="str">

</xml_diff>

<commit_message>
JT-232 Update sample datasets and enhance custom field configurations
- Add new custom field definitions to config_importer_full.json, full_dataset_sample.xlsx, and ImportTemplate.xlsx to support number, text, select, and date types
</commit_message>
<xml_diff>
--- a/resources/templates/ImportTemplate.xlsx
+++ b/resources/templates/ImportTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workdir\DeerHide\sources\jira-toolkit\resources\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC11B61B-52F2-4383-A081-3EA527C8CFCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6BCD59E-577E-4328-B7B7-C716757B942C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3156" yWindow="6612" windowWidth="34560" windowHeight="18600" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
+    <workbookView xWindow="14685" yWindow="5445" windowWidth="33090" windowHeight="19545" activeTab="1" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset" sheetId="1" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="117">
   <si>
     <t>IssueType</t>
   </si>
@@ -332,9 +332,6 @@
     <t>Development</t>
   </si>
   <si>
-    <t>Misc Fields</t>
-  </si>
-  <si>
     <t>pod_test</t>
   </si>
   <si>
@@ -372,6 +369,57 @@
   </si>
   <si>
     <t>4w</t>
+  </si>
+  <si>
+    <t>Configuration</t>
+  </si>
+  <si>
+    <t>Custom Fields</t>
+  </si>
+  <si>
+    <t>Id</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Format</t>
+  </si>
+  <si>
+    <t>CF Number</t>
+  </si>
+  <si>
+    <t>customfield_10125</t>
+  </si>
+  <si>
+    <t>number</t>
+  </si>
+  <si>
+    <t>CF Plain Text</t>
+  </si>
+  <si>
+    <t>customfield_10124</t>
+  </si>
+  <si>
+    <t>text</t>
+  </si>
+  <si>
+    <t>CF Select</t>
+  </si>
+  <si>
+    <t>customfield_10126</t>
+  </si>
+  <si>
+    <t>select</t>
+  </si>
+  <si>
+    <t>CF Date</t>
+  </si>
+  <si>
+    <t>customfield_10123</t>
+  </si>
+  <si>
+    <t>date</t>
   </si>
 </sst>
 </file>
@@ -972,7 +1020,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="72">
+  <dxfs count="56">
     <dxf>
       <fill>
         <patternFill patternType="darkUp"/>
@@ -1116,146 +1164,10 @@
       </fill>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="darkUp"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDAF2D0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2CEEF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.89996032593768116"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <strike val="0"/>
-        <color theme="0" tint="-0.34998626667073579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor auto="1"/>
-          <bgColor rgb="FFF9B1AB"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCC99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9999"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF99CC"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
       <alignment vertical="top"/>
@@ -1398,12 +1310,6 @@
     </dxf>
     <dxf>
       <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1441,57 +1347,55 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" name="JiraDataset" displayName="JiraDataset" ref="A1:AJ3" totalsRowShown="0" headerRowDxfId="69" dataDxfId="68">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" name="JiraDataset" displayName="JiraDataset" ref="A1:AJ3" totalsRowShown="0" headerRowDxfId="55" dataDxfId="54">
   <autoFilter ref="A1:AJ3" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}"/>
   <tableColumns count="36">
-    <tableColumn id="3" xr3:uid="{AF2EC907-349C-4651-852D-6E39C61E17FF}" name="Priority" dataDxfId="67"/>
-    <tableColumn id="2" xr3:uid="{E90C51F2-4386-421F-A3E4-E2CA9D43D396}" name="IssueType" dataDxfId="66"/>
-    <tableColumn id="1" xr3:uid="{BBAD373B-BA13-47E4-9F74-565F4D9E9680}" name="Summary" dataDxfId="65"/>
-    <tableColumn id="4" xr3:uid="{026E5B97-FAFC-4E46-860E-0B0C976B1148}" name="Issue Key" dataDxfId="64"/>
-    <tableColumn id="5" xr3:uid="{A2C262E8-D544-4669-99F1-151EDE081654}" name="Description" dataDxfId="63"/>
-    <tableColumn id="7" xr3:uid="{0FAD1ACC-432E-462C-8B89-71540710BCB5}" name="FixVersion" dataDxfId="62">
-      <calculatedColumnFormula>Config!$G$4</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="28" xr3:uid="{07F3030C-7187-4B16-BBDB-798304851975}" name="Assignee.Name" dataDxfId="61"/>
-    <tableColumn id="8" xr3:uid="{8C7FB8DB-A85B-4189-93D8-0F0D4EEEF81B}" name="Component" dataDxfId="60"/>
-    <tableColumn id="9" xr3:uid="{DC5101A8-1204-44D2-BC2C-FEE1A4EFE7C1}" name="Sprint Name" dataDxfId="59"/>
-    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="58"/>
-    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="57"/>
-    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="56"/>
-    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="55"/>
-    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="54">
+    <tableColumn id="3" xr3:uid="{AF2EC907-349C-4651-852D-6E39C61E17FF}" name="Priority" dataDxfId="53"/>
+    <tableColumn id="2" xr3:uid="{E90C51F2-4386-421F-A3E4-E2CA9D43D396}" name="IssueType" dataDxfId="52"/>
+    <tableColumn id="1" xr3:uid="{BBAD373B-BA13-47E4-9F74-565F4D9E9680}" name="Summary" dataDxfId="51"/>
+    <tableColumn id="4" xr3:uid="{026E5B97-FAFC-4E46-860E-0B0C976B1148}" name="Issue Key" dataDxfId="50"/>
+    <tableColumn id="5" xr3:uid="{A2C262E8-D544-4669-99F1-151EDE081654}" name="Description" dataDxfId="49"/>
+    <tableColumn id="7" xr3:uid="{0FAD1ACC-432E-462C-8B89-71540710BCB5}" name="FixVersion" dataDxfId="48"/>
+    <tableColumn id="28" xr3:uid="{07F3030C-7187-4B16-BBDB-798304851975}" name="Assignee.Name" dataDxfId="47"/>
+    <tableColumn id="8" xr3:uid="{8C7FB8DB-A85B-4189-93D8-0F0D4EEEF81B}" name="Component" dataDxfId="46"/>
+    <tableColumn id="9" xr3:uid="{DC5101A8-1204-44D2-BC2C-FEE1A4EFE7C1}" name="Sprint Name" dataDxfId="45"/>
+    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="44"/>
+    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="43"/>
+    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="42"/>
+    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="41"/>
+    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="40">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[IssueType]]="Epic",JiraDataset[[#This Row],[Summary]],"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="27" xr3:uid="{911C8FDC-5528-43FC-BDF4-D4761F03C0E5}" name="Child-Issue" dataDxfId="53"/>
-    <tableColumn id="41" xr3:uid="{AB248E07-9BFA-42CC-BC41-B4234F677BFB}" name="Child-Issue1" dataDxfId="52"/>
-    <tableColumn id="29" xr3:uid="{89D12135-F3E3-4253-844F-1B9A54169953}" name="Child-Issue2" dataDxfId="51"/>
-    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="50"/>
-    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="49"/>
-    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="48"/>
-    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="47"/>
-    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="46"/>
-    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="45"/>
-    <tableColumn id="18" xr3:uid="{16B98070-7F8A-4FC7-AD99-EA81D0BD26AB}" name="Labels6" dataDxfId="44"/>
-    <tableColumn id="19" xr3:uid="{016EAEF4-8EA9-408B-9F1A-ECFB17E81C77}" name="Labels7" dataDxfId="43"/>
-    <tableColumn id="26" xr3:uid="{8263F9EC-BF0A-46F7-BA83-6083A4262B91}" name="Labels8" dataDxfId="42"/>
-    <tableColumn id="20" xr3:uid="{389B11C5-1B22-48C0-BCA2-72F050425FA1}" name="Labels9" dataDxfId="41"/>
-    <tableColumn id="25" xr3:uid="{AE95F8A2-F7F0-4985-9AE6-4201B9792775}" name="Labels10" dataDxfId="40"/>
-    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="39">
+    <tableColumn id="27" xr3:uid="{911C8FDC-5528-43FC-BDF4-D4761F03C0E5}" name="Child-Issue" dataDxfId="39"/>
+    <tableColumn id="41" xr3:uid="{AB248E07-9BFA-42CC-BC41-B4234F677BFB}" name="Child-Issue1" dataDxfId="38"/>
+    <tableColumn id="29" xr3:uid="{89D12135-F3E3-4253-844F-1B9A54169953}" name="Child-Issue2" dataDxfId="37"/>
+    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="36"/>
+    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="35"/>
+    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="34"/>
+    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="33"/>
+    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="32"/>
+    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="31"/>
+    <tableColumn id="18" xr3:uid="{16B98070-7F8A-4FC7-AD99-EA81D0BD26AB}" name="Labels6" dataDxfId="30"/>
+    <tableColumn id="19" xr3:uid="{016EAEF4-8EA9-408B-9F1A-ECFB17E81C77}" name="Labels7" dataDxfId="29"/>
+    <tableColumn id="26" xr3:uid="{8263F9EC-BF0A-46F7-BA83-6083A4262B91}" name="Labels8" dataDxfId="28"/>
+    <tableColumn id="20" xr3:uid="{389B11C5-1B22-48C0-BCA2-72F050425FA1}" name="Labels9" dataDxfId="27"/>
+    <tableColumn id="25" xr3:uid="{AE95F8A2-F7F0-4985-9AE6-4201B9792775}" name="Labels10" dataDxfId="26"/>
+    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="25">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], Config!$D$4:$E$9, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="38">
+    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="24">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="37">
+    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="23">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Feature Pod Label", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="36">
+    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="22">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], Config!$A$4:$B$24, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="35">
+    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="21">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("jira.project.key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="34">
+    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="20">
       <calculatedColumnFormula array="1">IF(
   JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
   "",
@@ -1507,7 +1411,7 @@
   )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="33">
+    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="19">
       <calculatedColumnFormula array="1">IFERROR(
     _xlfn.IFS(
         JiraDataset[[#This Row],[IssueType]] = cfg_type_comment,"SKIP",
@@ -1517,9 +1421,22 @@
     cfg_type_workitem
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="32"/>
+    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3EF499BE-ED9A-4C28-BC5A-BCDEF51C613F}" name="CfgCustomFields" displayName="CfgCustomFields" ref="U3:X7" totalsRowShown="0">
+  <autoFilter ref="U3:X7" xr:uid="{3EF499BE-ED9A-4C28-BC5A-BCDEF51C613F}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{44010E5A-E449-477A-BFB0-2ECA215E3FEB}" name="Name"/>
+    <tableColumn id="2" xr3:uid="{0E558995-744D-4813-9A4E-F64FFF5047AE}" name="Id"/>
+    <tableColumn id="3" xr3:uid="{8D81F1E3-8799-4AE9-BACA-610A64846357}" name="Type"/>
+    <tableColumn id="4" xr3:uid="{BEA106CA-BE66-4629-B856-FE53C841A6BA}" name="Format"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -1557,7 +1474,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}" name="CfgPriorities" displayName="CfgPriorities" ref="O3:O9" totalsRowShown="0">
   <autoFilter ref="O3:O9" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="71"/>
+    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1591,7 +1508,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{D4E1611F-A2CF-465D-A219-1759EA66687D}" name="Name"/>
     <tableColumn id="2" xr3:uid="{174D0D86-B1AA-4BF7-AC91-FCACFC898851}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Remark" dataDxfId="70"/>
+    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Remark" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1925,42 +1842,42 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F73058B-F76D-4AAE-8108-6C4469E9D8B5}">
   <dimension ref="A1:AK3"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelCol="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.6640625" customWidth="1"/>
-    <col min="4" max="4" width="11.88671875" hidden="1" customWidth="1"/>
+    <col min="1" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.7109375" customWidth="1"/>
+    <col min="4" max="4" width="11.85546875" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="33" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="46.33203125" customWidth="1"/>
-    <col min="7" max="7" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.5546875" customWidth="1"/>
+    <col min="6" max="6" width="46.28515625" customWidth="1"/>
+    <col min="7" max="7" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.5703125" customWidth="1"/>
     <col min="9" max="9" width="14" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.33203125" customWidth="1"/>
-    <col min="13" max="13" width="14.44140625" customWidth="1"/>
-    <col min="14" max="14" width="14.33203125" customWidth="1"/>
+    <col min="10" max="11" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.28515625" customWidth="1"/>
+    <col min="13" max="13" width="14.42578125" customWidth="1"/>
+    <col min="14" max="14" width="14.28515625" customWidth="1"/>
     <col min="15" max="15" width="0" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="22.33203125" hidden="1" customWidth="1"/>
-    <col min="17" max="17" width="12.88671875" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="12.44140625" customWidth="1"/>
-    <col min="19" max="19" width="15.5546875" customWidth="1"/>
-    <col min="20" max="20" width="12.88671875" customWidth="1"/>
+    <col min="16" max="16" width="22.28515625" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="12.85546875" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="12.42578125" customWidth="1"/>
+    <col min="19" max="19" width="15.5703125" customWidth="1"/>
+    <col min="20" max="20" width="12.85546875" customWidth="1"/>
     <col min="21" max="21" width="10" customWidth="1"/>
     <col min="22" max="22" width="10" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="10" customWidth="1"/>
-    <col min="24" max="24" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="10" customWidth="1" outlineLevel="1"/>
     <col min="31" max="31" width="10" customWidth="1"/>
-    <col min="32" max="32" width="8.6640625" customWidth="1" outlineLevel="1"/>
-    <col min="33" max="34" width="13.109375" customWidth="1" outlineLevel="1"/>
-    <col min="35" max="35" width="11.44140625" customWidth="1" outlineLevel="1"/>
-    <col min="36" max="37" width="13.6640625" customWidth="1" outlineLevel="1"/>
-    <col min="38" max="38" width="36.5546875" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="18.6640625" customWidth="1"/>
-    <col min="41" max="41" width="87.33203125" customWidth="1"/>
+    <col min="32" max="32" width="8.7109375" customWidth="1" outlineLevel="1"/>
+    <col min="33" max="34" width="13.140625" customWidth="1" outlineLevel="1"/>
+    <col min="35" max="35" width="11.42578125" customWidth="1" outlineLevel="1"/>
+    <col min="36" max="37" width="13.7109375" customWidth="1" outlineLevel="1"/>
+    <col min="38" max="38" width="36.5703125" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="18.7109375" customWidth="1"/>
+    <col min="41" max="41" width="87.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>1</v>
       </c>
@@ -2070,7 +1987,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
         <v>33</v>
@@ -2162,7 +2079,7 @@
       </c>
       <c r="AJ2" s="3"/>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>48</v>
       </c>
@@ -2177,7 +2094,7 @@
         <v>84</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>54</v>
@@ -2189,7 +2106,7 @@
         <v>46</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K3" s="3">
         <v>2</v>
@@ -2390,7 +2307,7 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Issue Type" xr:uid="{28BF52BF-C0B0-4D22-B02F-F1408D5A055B}">
           <x14:formula1>
-            <xm:f>Config!$U$4:$U$33</xm:f>
+            <xm:f>Config!$Z$4:$Z$33</xm:f>
           </x14:formula1>
           <xm:sqref>B2:B3</xm:sqref>
         </x14:dataValidation>
@@ -2402,30 +2319,30 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2D54512-1380-4F02-BB23-352387C91232}">
-  <dimension ref="A1:V21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:AA21"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.6640625" customWidth="1"/>
+    <col min="1" max="1" width="29.7109375" customWidth="1"/>
     <col min="2" max="2" width="49" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.33203125" customWidth="1"/>
-    <col min="4" max="5" width="18.6640625" customWidth="1"/>
-    <col min="6" max="6" width="4.33203125" customWidth="1"/>
-    <col min="7" max="7" width="18.5546875" customWidth="1"/>
-    <col min="8" max="8" width="4.33203125" customWidth="1"/>
-    <col min="9" max="9" width="19.109375" customWidth="1"/>
-    <col min="10" max="10" width="4.33203125" customWidth="1"/>
-    <col min="11" max="11" width="18.5546875" customWidth="1"/>
-    <col min="12" max="12" width="4.33203125" customWidth="1"/>
-    <col min="13" max="13" width="17.5546875" customWidth="1"/>
-    <col min="14" max="14" width="4.33203125" customWidth="1"/>
-    <col min="15" max="15" width="18.6640625" customWidth="1"/>
-    <col min="16" max="16" width="4.33203125" customWidth="1"/>
-    <col min="17" max="18" width="18.6640625" customWidth="1"/>
+    <col min="3" max="3" width="4.28515625" customWidth="1"/>
+    <col min="4" max="5" width="18.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.28515625" customWidth="1"/>
+    <col min="7" max="7" width="18.5703125" customWidth="1"/>
+    <col min="8" max="8" width="4.28515625" customWidth="1"/>
+    <col min="9" max="9" width="19.140625" customWidth="1"/>
+    <col min="10" max="10" width="4.28515625" customWidth="1"/>
+    <col min="11" max="11" width="18.5703125" customWidth="1"/>
+    <col min="12" max="12" width="4.28515625" customWidth="1"/>
+    <col min="13" max="13" width="17.5703125" customWidth="1"/>
+    <col min="14" max="14" width="4.28515625" customWidth="1"/>
+    <col min="15" max="15" width="18.7109375" customWidth="1"/>
+    <col min="16" max="16" width="4.28515625" customWidth="1"/>
+    <col min="17" max="18" width="18.7109375" customWidth="1"/>
     <col min="19" max="19" width="35" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="22.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:27" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
         <v>69</v>
       </c>
@@ -2450,15 +2367,21 @@
         <v>53</v>
       </c>
       <c r="Q1" s="11" t="s">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="R1" s="11"/>
       <c r="S1" s="11"/>
-      <c r="U1" s="6" t="s">
+      <c r="U1" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="V1" s="11"/>
+      <c r="W1" s="11"/>
+      <c r="X1" s="11"/>
+      <c r="Z1" s="6" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
         <v>75</v>
       </c>
@@ -2493,12 +2416,17 @@
       <c r="R2" s="12"/>
       <c r="S2" s="9"/>
       <c r="T2" s="7"/>
-      <c r="U2" s="9" t="s">
+      <c r="U2" s="7"/>
+      <c r="V2" s="7"/>
+      <c r="W2" s="7"/>
+      <c r="X2" s="7"/>
+      <c r="Y2" s="7"/>
+      <c r="Z2" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="V2" s="9"/>
+      <c r="AA2" s="9"/>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>58</v>
       </c>
@@ -2535,16 +2463,28 @@
       <c r="S3" t="s">
         <v>66</v>
       </c>
-      <c r="U3" s="5" t="s">
+      <c r="U3" t="s">
+        <v>54</v>
+      </c>
+      <c r="V3" t="s">
+        <v>102</v>
+      </c>
+      <c r="W3" t="s">
+        <v>103</v>
+      </c>
+      <c r="X3" t="s">
+        <v>104</v>
+      </c>
+      <c r="Z3" s="5" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>54</v>
       </c>
       <c r="B4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D4" t="s">
         <v>46</v>
@@ -2553,7 +2493,7 @@
         <v>1</v>
       </c>
       <c r="G4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I4" t="s">
         <v>86</v>
@@ -2571,17 +2511,26 @@
         <v>51</v>
       </c>
       <c r="R4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="S4" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="U4" t="str" cm="1">
-        <f t="array" aca="1" ref="U4:U12" ca="1">_xlfn.UNIQUE((_xlfn.VSTACK(INDIRECT("CfgIssueTypes[IssueType.Name]"),INDIRECT("CfgIgnoreList[IgnoreList.Name]"))))</f>
+      <c r="U4" t="s">
+        <v>105</v>
+      </c>
+      <c r="V4" t="s">
+        <v>106</v>
+      </c>
+      <c r="W4" t="s">
+        <v>107</v>
+      </c>
+      <c r="Z4" t="str" cm="1">
+        <f t="array" aca="1" ref="Z4:Z12" ca="1">_xlfn.UNIQUE((_xlfn.VSTACK(INDIRECT("CfgIssueTypes[IssueType.Name]"),INDIRECT("CfgIgnoreList[IgnoreList.Name]"))))</f>
         <v>Story</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="K5" t="s">
         <v>37</v>
       </c>
@@ -2595,17 +2544,26 @@
         <v>47</v>
       </c>
       <c r="R5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="S5" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="U5" t="str">
+      <c r="U5" t="s">
+        <v>108</v>
+      </c>
+      <c r="V5" t="s">
+        <v>109</v>
+      </c>
+      <c r="W5" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z5" t="str">
         <f ca="1"/>
         <v>Task</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="K6" t="s">
         <v>40</v>
       </c>
@@ -2613,18 +2571,27 @@
         <v>33</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="Q6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="S6" s="7"/>
-      <c r="U6" t="str">
+      <c r="U6" t="s">
+        <v>111</v>
+      </c>
+      <c r="V6" t="s">
+        <v>112</v>
+      </c>
+      <c r="W6" t="s">
+        <v>113</v>
+      </c>
+      <c r="Z6" t="str">
         <f ca="1"/>
         <v>Bug</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="K7" t="s">
@@ -2637,118 +2604,128 @@
         <v>42</v>
       </c>
       <c r="Q7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="R7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="S7" s="7"/>
-      <c r="U7" t="str">
+      <c r="U7" t="s">
+        <v>114</v>
+      </c>
+      <c r="V7" t="s">
+        <v>115</v>
+      </c>
+      <c r="W7" t="s">
+        <v>116</v>
+      </c>
+      <c r="Z7" t="str">
         <f ca="1"/>
         <v>Epic</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="K8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="O8" s="1" t="s">
         <v>49</v>
       </c>
       <c r="Q8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="R8" t="b">
         <v>1</v>
       </c>
       <c r="S8" s="7"/>
-      <c r="U8" t="str">
+      <c r="Z8" t="str">
         <f ca="1"/>
         <v>Sub-Task</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="O9" s="1" t="s">
         <v>50</v>
       </c>
       <c r="Q9" t="s">
+        <v>91</v>
+      </c>
+      <c r="R9" t="s">
         <v>92</v>
       </c>
-      <c r="R9" t="s">
-        <v>93</v>
-      </c>
       <c r="S9" s="7"/>
-      <c r="U9" t="str">
+      <c r="Z9" t="str">
         <f ca="1"/>
         <v>Comment</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
-      <c r="U10" t="str">
+      <c r="Z10" t="str">
         <f ca="1"/>
         <v>Skip</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
-      <c r="U11" t="str">
+      <c r="Z11" t="str">
         <f ca="1"/>
         <v>Note</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
-      <c r="U12" t="str">
+      <c r="Z12" t="str">
         <f ca="1"/>
         <v>WorkItem</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="4:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="4:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
     </row>
-    <row r="19" spans="4:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
     </row>
-    <row r="20" spans="4:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
     </row>
-    <row r="21" spans="4:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
+    <mergeCell ref="U1:X1"/>
     <mergeCell ref="Q1:S1"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="A1:B1"/>
@@ -2760,7 +2737,7 @@
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
-  <tableParts count="8">
+  <tableParts count="9">
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>
@@ -2769,11 +2746,32 @@
     <tablePart r:id="rId7"/>
     <tablePart r:id="rId8"/>
     <tablePart r:id="rId9"/>
+    <tablePart r:id="rId10"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FB038601AF41D04A88A4BD446922F1A8" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e8d32171d27ae41230d53456f24efae5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c471fd26-9765-4fbe-b6fd-c17c1e55c974" xmlns:ns3="9df69692-83aa-4c55-88c1-62abad05f4fe" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f2fb84de5621acf32f385a2ba90fb29" ns2:_="" ns3:_="">
     <xsd:import namespace="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
@@ -3002,27 +3000,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FFE630F-6530-4863-AB67-8477539A0000}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
+    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2C983B91-58B3-4C2C-AC55-FFEC9F0DB5F6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3039,23 +3036,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FFE630F-6530-4863-AB67-8477539A0000}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
-    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
JT-232 Add support for 'any' custom field type
</commit_message>
<xml_diff>
--- a/resources/templates/ImportTemplate.xlsx
+++ b/resources/templates/ImportTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workdir\DeerHide\sources\jira-toolkit\resources\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6BCD59E-577E-4328-B7B7-C716757B942C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F55D66A0-1E6F-4D7B-9000-CD63805D1508}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14685" yWindow="5445" windowWidth="33090" windowHeight="19545" activeTab="1" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
+    <workbookView xWindow="9060" yWindow="7155" windowWidth="33090" windowHeight="19545" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset" sheetId="1" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="120">
   <si>
     <t>IssueType</t>
   </si>
@@ -420,6 +420,15 @@
   </si>
   <si>
     <t>date</t>
+  </si>
+  <si>
+    <t>CF Field</t>
+  </si>
+  <si>
+    <t>any</t>
+  </si>
+  <si>
+    <t>customfield_10128</t>
   </si>
 </sst>
 </file>
@@ -1428,8 +1437,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3EF499BE-ED9A-4C28-BC5A-BCDEF51C613F}" name="CfgCustomFields" displayName="CfgCustomFields" ref="U3:X7" totalsRowShown="0">
-  <autoFilter ref="U3:X7" xr:uid="{3EF499BE-ED9A-4C28-BC5A-BCDEF51C613F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3EF499BE-ED9A-4C28-BC5A-BCDEF51C613F}" name="CfgCustomFields" displayName="CfgCustomFields" ref="U3:X8" totalsRowShown="0">
+  <autoFilter ref="U3:X8" xr:uid="{3EF499BE-ED9A-4C28-BC5A-BCDEF51C613F}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{44010E5A-E449-477A-BFB0-2ECA215E3FEB}" name="Name"/>
     <tableColumn id="2" xr3:uid="{0E558995-744D-4813-9A4E-F64FFF5047AE}" name="Id"/>
@@ -2640,6 +2649,15 @@
         <v>1</v>
       </c>
       <c r="S8" s="7"/>
+      <c r="U8" t="s">
+        <v>117</v>
+      </c>
+      <c r="V8" t="s">
+        <v>119</v>
+      </c>
+      <c r="W8" t="s">
+        <v>118</v>
+      </c>
       <c r="Z8" t="str">
         <f ca="1"/>
         <v>Sub-Task</v>
@@ -2752,26 +2770,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FB038601AF41D04A88A4BD446922F1A8" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e8d32171d27ae41230d53456f24efae5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c471fd26-9765-4fbe-b6fd-c17c1e55c974" xmlns:ns3="9df69692-83aa-4c55-88c1-62abad05f4fe" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f2fb84de5621acf32f385a2ba90fb29" ns2:_="" ns3:_="">
     <xsd:import namespace="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
@@ -3000,26 +2998,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FFE630F-6530-4863-AB67-8477539A0000}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
-    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2C983B91-58B3-4C2C-AC55-FFEC9F0DB5F6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3036,4 +3035,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FFE630F-6530-4863-AB67-8477539A0000}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
+    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update ImportTemplate.xlsx to reflect recent changes (configuration)
</commit_message>
<xml_diff>
--- a/resources/templates/ImportTemplate.xlsx
+++ b/resources/templates/ImportTemplate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workdir\DeerHide\sources\jira-toolkit\resources\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F55D66A0-1E6F-4D7B-9000-CD63805D1508}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09FDBF7F-D200-4D23-A13C-FBD71614ACEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9060" yWindow="7155" windowWidth="33090" windowHeight="19545" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
+    <workbookView xWindow="675" yWindow="4890" windowWidth="25740" windowHeight="15045" activeTab="1" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset" sheetId="1" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="121">
   <si>
     <t>IssueType</t>
   </si>
@@ -341,9 +341,6 @@
     <t>jira.project.key</t>
   </si>
   <si>
-    <t>validation.skip_rowtype</t>
-  </si>
-  <si>
     <t>validation.skip_issuetypes</t>
   </si>
   <si>
@@ -429,6 +426,12 @@
   </si>
   <si>
     <t>customfield_10128</t>
+  </si>
+  <si>
+    <t>app.import.auto_open_page</t>
+  </si>
+  <si>
+    <t>no</t>
   </si>
 </sst>
 </file>
@@ -1512,8 +1515,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{383560BC-B1F2-44B6-B877-188131EFA163}" name="CfgAutofieldValues" displayName="CfgAutofieldValues" ref="Q3:S9" totalsRowShown="0">
-  <autoFilter ref="Q3:S9" xr:uid="{383560BC-B1F2-44B6-B877-188131EFA163}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{383560BC-B1F2-44B6-B877-188131EFA163}" name="CfgAutofieldValues" displayName="CfgAutofieldValues" ref="Q3:S10" totalsRowShown="0">
+  <autoFilter ref="Q3:S10" xr:uid="{383560BC-B1F2-44B6-B877-188131EFA163}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{D4E1611F-A2CF-465D-A219-1759EA66687D}" name="Name"/>
     <tableColumn id="2" xr3:uid="{174D0D86-B1AA-4BF7-AC91-FCACFC898851}" name="Value"/>
@@ -1999,7 +2002,7 @@
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>35</v>
@@ -2103,7 +2106,7 @@
         <v>84</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>54</v>
@@ -2115,7 +2118,7 @@
         <v>46</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K3" s="3">
         <v>2</v>
@@ -2376,12 +2379,12 @@
         <v>53</v>
       </c>
       <c r="Q1" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="R1" s="11"/>
       <c r="S1" s="11"/>
       <c r="U1" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="V1" s="11"/>
       <c r="W1" s="11"/>
@@ -2476,13 +2479,13 @@
         <v>54</v>
       </c>
       <c r="V3" t="s">
+        <v>101</v>
+      </c>
+      <c r="W3" t="s">
         <v>102</v>
       </c>
-      <c r="W3" t="s">
+      <c r="X3" t="s">
         <v>103</v>
-      </c>
-      <c r="X3" t="s">
-        <v>104</v>
       </c>
       <c r="Z3" s="5" t="s">
         <v>63</v>
@@ -2493,7 +2496,7 @@
         <v>54</v>
       </c>
       <c r="B4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D4" t="s">
         <v>46</v>
@@ -2502,7 +2505,7 @@
         <v>1</v>
       </c>
       <c r="G4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="I4" t="s">
         <v>86</v>
@@ -2520,19 +2523,19 @@
         <v>51</v>
       </c>
       <c r="R4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="S4" s="7" t="s">
         <v>73</v>
       </c>
       <c r="U4" t="s">
+        <v>104</v>
+      </c>
+      <c r="V4" t="s">
         <v>105</v>
       </c>
-      <c r="V4" t="s">
+      <c r="W4" t="s">
         <v>106</v>
-      </c>
-      <c r="W4" t="s">
-        <v>107</v>
       </c>
       <c r="Z4" t="str" cm="1">
         <f t="array" aca="1" ref="Z4:Z12" ca="1">_xlfn.UNIQUE((_xlfn.VSTACK(INDIRECT("CfgIssueTypes[IssueType.Name]"),INDIRECT("CfgIgnoreList[IgnoreList.Name]"))))</f>
@@ -2559,13 +2562,13 @@
         <v>74</v>
       </c>
       <c r="U5" t="s">
+        <v>107</v>
+      </c>
+      <c r="V5" t="s">
         <v>108</v>
       </c>
-      <c r="V5" t="s">
+      <c r="W5" t="s">
         <v>109</v>
-      </c>
-      <c r="W5" t="s">
-        <v>110</v>
       </c>
       <c r="Z5" t="str">
         <f ca="1"/>
@@ -2580,20 +2583,20 @@
         <v>33</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="Q6" t="s">
         <v>88</v>
       </c>
       <c r="S6" s="7"/>
       <c r="U6" t="s">
+        <v>110</v>
+      </c>
+      <c r="V6" t="s">
         <v>111</v>
       </c>
-      <c r="V6" t="s">
+      <c r="W6" t="s">
         <v>112</v>
-      </c>
-      <c r="W6" t="s">
-        <v>113</v>
       </c>
       <c r="Z6" t="str">
         <f ca="1"/>
@@ -2616,17 +2619,17 @@
         <v>89</v>
       </c>
       <c r="R7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="S7" s="7"/>
       <c r="U7" t="s">
+        <v>113</v>
+      </c>
+      <c r="V7" t="s">
         <v>114</v>
       </c>
-      <c r="V7" t="s">
+      <c r="W7" t="s">
         <v>115</v>
-      </c>
-      <c r="W7" t="s">
-        <v>116</v>
       </c>
       <c r="Z7" t="str">
         <f ca="1"/>
@@ -2637,26 +2640,20 @@
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="K8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="O8" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="Q8" t="s">
-        <v>90</v>
-      </c>
-      <c r="R8" t="b">
-        <v>1</v>
-      </c>
       <c r="S8" s="7"/>
       <c r="U8" t="s">
+        <v>116</v>
+      </c>
+      <c r="V8" t="s">
+        <v>118</v>
+      </c>
+      <c r="W8" t="s">
         <v>117</v>
-      </c>
-      <c r="V8" t="s">
-        <v>119</v>
-      </c>
-      <c r="W8" t="s">
-        <v>118</v>
       </c>
       <c r="Z8" t="str">
         <f ca="1"/>
@@ -2670,10 +2667,10 @@
         <v>50</v>
       </c>
       <c r="Q9" t="s">
+        <v>90</v>
+      </c>
+      <c r="R9" t="s">
         <v>91</v>
-      </c>
-      <c r="R9" t="s">
-        <v>92</v>
       </c>
       <c r="S9" s="7"/>
       <c r="Z9" t="str">
@@ -2684,6 +2681,13 @@
     <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
+      <c r="Q10" t="s">
+        <v>119</v>
+      </c>
+      <c r="R10" t="s">
+        <v>120</v>
+      </c>
+      <c r="S10" s="7"/>
       <c r="Z10" t="str">
         <f ca="1"/>
         <v>Skip</v>

</xml_diff>

<commit_message>
JT-312 refactor(config): simplify starter Excel template config for first-time setup
Keep the Excel config focused on practical defaults by removing non-essential sections while preserving commonly customized fields and root-level validation skips. Reintroduce metadata.version.
</commit_message>
<xml_diff>
--- a/resources/templates/ImportTemplate.xlsx
+++ b/resources/templates/ImportTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workdir\DeerHide\sources\jira-toolkit\resources\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{003E1DC9-7C6D-4031-B67D-8F83CD74C94E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19EF8646-AAC6-4786-B8CE-C82C9A8B8D04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10215" yWindow="9390" windowWidth="31710" windowHeight="20325" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
+    <workbookView xWindow="15060" yWindow="5175" windowWidth="43200" windowHeight="23445" activeTab="1" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="105">
   <si>
     <t>IssueType</t>
   </si>
@@ -206,9 +206,6 @@
     <t>Skip</t>
   </si>
   <si>
-    <t>WorkItem</t>
-  </si>
-  <si>
     <t>Sprint 1</t>
   </si>
   <si>
@@ -347,9 +344,6 @@
     <t>Version_Tag</t>
   </si>
   <si>
-    <t>PROJECT KEY</t>
-  </si>
-  <si>
     <t>jt-imported</t>
   </si>
   <si>
@@ -380,61 +374,16 @@
     <t>Format</t>
   </si>
   <si>
-    <t>CF Number</t>
-  </si>
-  <si>
-    <t>customfield_10125</t>
-  </si>
-  <si>
-    <t>number</t>
-  </si>
-  <si>
-    <t>CF Plain Text</t>
-  </si>
-  <si>
-    <t>customfield_10124</t>
-  </si>
-  <si>
-    <t>text</t>
-  </si>
-  <si>
-    <t>CF Select</t>
-  </si>
-  <si>
-    <t>customfield_10126</t>
-  </si>
-  <si>
-    <t>select</t>
-  </si>
-  <si>
-    <t>CF Date</t>
-  </si>
-  <si>
-    <t>customfield_10123</t>
-  </si>
-  <si>
-    <t>date</t>
-  </si>
-  <si>
-    <t>CF Field</t>
-  </si>
-  <si>
-    <t>any</t>
-  </si>
-  <si>
-    <t>customfield_10128</t>
-  </si>
-  <si>
-    <t>app.import.auto_open_page</t>
-  </si>
-  <si>
-    <t>no</t>
-  </si>
-  <si>
-    <t>jira.components_source</t>
-  </si>
-  <si>
-    <t>jira</t>
+    <t>Initiative</t>
+  </si>
+  <si>
+    <t>https://your-instance.atlassian.net</t>
+  </si>
+  <si>
+    <t>metadata.version</t>
+  </si>
+  <si>
+    <t>PROJECT-KEY</t>
   </si>
 </sst>
 </file>
@@ -1443,8 +1392,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3EF499BE-ED9A-4C28-BC5A-BCDEF51C613F}" name="CfgCustomFields" displayName="CfgCustomFields" ref="U3:X8" totalsRowShown="0">
-  <autoFilter ref="U3:X8" xr:uid="{3EF499BE-ED9A-4C28-BC5A-BCDEF51C613F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3EF499BE-ED9A-4C28-BC5A-BCDEF51C613F}" name="CfgCustomFields" displayName="CfgCustomFields" ref="U3:X4" insertRow="1" totalsRowShown="0">
+  <autoFilter ref="U3:X4" xr:uid="{3EF499BE-ED9A-4C28-BC5A-BCDEF51C613F}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{44010E5A-E449-477A-BFB0-2ECA215E3FEB}" name="Name"/>
     <tableColumn id="2" xr3:uid="{0E558995-744D-4813-9A4E-F64FFF5047AE}" name="Id"/>
@@ -1476,8 +1425,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{6F085B8C-1322-4F43-A516-588923936259}" name="CfgIssueTypes" displayName="CfgIssueTypes" ref="K3:K8" totalsRowShown="0">
-  <autoFilter ref="K3:K8" xr:uid="{6F085B8C-1322-4F43-A516-588923936259}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{6F085B8C-1322-4F43-A516-588923936259}" name="CfgIssueTypes" displayName="CfgIssueTypes" ref="K3:K9" totalsRowShown="0">
+  <autoFilter ref="K3:K9" xr:uid="{6F085B8C-1322-4F43-A516-588923936259}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{A92436BC-3156-493F-B5C6-0BB6B51F89EB}" name="IssueType.Name"/>
   </tableColumns>
@@ -1518,8 +1467,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{383560BC-B1F2-44B6-B877-188131EFA163}" name="CfgAutofieldValues" displayName="CfgAutofieldValues" ref="Q3:S11" totalsRowShown="0">
-  <autoFilter ref="Q3:S11" xr:uid="{383560BC-B1F2-44B6-B877-188131EFA163}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{383560BC-B1F2-44B6-B877-188131EFA163}" name="CfgAutofieldValues" displayName="CfgAutofieldValues" ref="Q3:S9" totalsRowShown="0">
+  <autoFilter ref="Q3:S9" xr:uid="{383560BC-B1F2-44B6-B877-188131EFA163}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{D4E1611F-A2CF-465D-A219-1759EA66687D}" name="Name"/>
     <tableColumn id="2" xr3:uid="{174D0D86-B1AA-4BF7-AC91-FCACFC898851}" name="Value"/>
@@ -1530,8 +1479,8 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{0ABE2B38-573A-4A51-8D54-C217B9D7D54F}" name="CfgIgnoreList" displayName="CfgIgnoreList" ref="M3:M7" totalsRowShown="0">
-  <autoFilter ref="M3:M7" xr:uid="{0ABE2B38-573A-4A51-8D54-C217B9D7D54F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{0ABE2B38-573A-4A51-8D54-C217B9D7D54F}" name="CfgIgnoreList" displayName="CfgIgnoreList" ref="M3:M6" totalsRowShown="0">
+  <autoFilter ref="M3:M6" xr:uid="{0ABE2B38-573A-4A51-8D54-C217B9D7D54F}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{1396737E-05D6-4D62-AF56-4B039C3A3607}" name="IgnoreList.Name"/>
   </tableColumns>
@@ -1927,7 +1876,7 @@
         <v>10</v>
       </c>
       <c r="L1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="M1" s="3" t="s">
         <v>11</v>
@@ -2019,7 +1968,7 @@
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
       <c r="J2" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="K2" s="3">
         <v>1</v>
@@ -2096,32 +2045,32 @@
     </row>
     <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>41</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="K3" s="3">
         <v>2</v>
@@ -2164,7 +2113,7 @@
       </c>
       <c r="AG3" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("jira.project.key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
-        <v>PROJECT KEY</v>
+        <v>PROJECT-KEY</v>
       </c>
       <c r="AH3" s="3" cm="1">
         <f t="array" ref="AH3">IF(
@@ -2183,7 +2132,7 @@
 )</f>
         <v>34560000</v>
       </c>
-      <c r="AI3" s="3" t="str" cm="1">
+      <c r="AI3" s="3" cm="1">
         <f t="array" ref="AI3">IFERROR(
     _xlfn.IFS(
         JiraDataset[[#This Row],[IssueType]] = cfg_type_comment,"SKIP",
@@ -2192,7 +2141,7 @@
     ),
     cfg_type_workitem
 )</f>
-        <v>WorkItem</v>
+        <v>0</v>
       </c>
       <c r="AJ3" s="3"/>
     </row>
@@ -2359,72 +2308,72 @@
   <sheetData>
     <row r="1" spans="1:27" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B1" s="11"/>
       <c r="D1" s="11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E1" s="11"/>
       <c r="G1" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="K1" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="M1" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="O1" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="M1" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="O1" s="6" t="s">
-        <v>53</v>
-      </c>
       <c r="Q1" s="11" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="R1" s="11"/>
       <c r="S1" s="11"/>
       <c r="U1" s="11" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="V1" s="11"/>
       <c r="W1" s="11"/>
       <c r="X1" s="11"/>
       <c r="Z1" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="7"/>
       <c r="D2" s="12" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E2" s="12"/>
       <c r="F2" s="7"/>
       <c r="G2" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H2" s="10"/>
       <c r="I2" s="10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="J2" s="10"/>
       <c r="K2" s="12" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="L2" s="12"/>
       <c r="M2" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="N2" s="9"/>
       <c r="O2" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="P2" s="10"/>
       <c r="Q2" s="12"/>
@@ -2437,7 +2386,7 @@
       <c r="X2" s="7"/>
       <c r="Y2" s="7"/>
       <c r="Z2" s="9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AA2" s="9"/>
     </row>
@@ -2446,72 +2395,72 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D3" t="s">
         <v>58</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>59</v>
       </c>
-      <c r="E3" t="s">
+      <c r="G3" t="s">
+        <v>63</v>
+      </c>
+      <c r="I3" t="s">
+        <v>62</v>
+      </c>
+      <c r="K3" t="s">
+        <v>61</v>
+      </c>
+      <c r="M3" t="s">
+        <v>66</v>
+      </c>
+      <c r="O3" t="s">
         <v>60</v>
       </c>
-      <c r="G3" t="s">
+      <c r="Q3" t="s">
+        <v>53</v>
+      </c>
+      <c r="R3" t="s">
+        <v>54</v>
+      </c>
+      <c r="S3" t="s">
         <v>64</v>
       </c>
-      <c r="I3" t="s">
-        <v>63</v>
-      </c>
-      <c r="K3" t="s">
-        <v>62</v>
-      </c>
-      <c r="M3" t="s">
-        <v>67</v>
-      </c>
-      <c r="O3" t="s">
+      <c r="U3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V3" t="s">
+        <v>98</v>
+      </c>
+      <c r="W3" t="s">
+        <v>99</v>
+      </c>
+      <c r="X3" t="s">
+        <v>100</v>
+      </c>
+      <c r="Z3" s="5" t="s">
         <v>61</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>54</v>
-      </c>
-      <c r="R3" t="s">
-        <v>55</v>
-      </c>
-      <c r="S3" t="s">
-        <v>65</v>
-      </c>
-      <c r="U3" t="s">
-        <v>54</v>
-      </c>
-      <c r="V3" t="s">
-        <v>100</v>
-      </c>
-      <c r="W3" t="s">
-        <v>101</v>
-      </c>
-      <c r="X3" t="s">
-        <v>102</v>
-      </c>
-      <c r="Z3" s="5" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E4">
         <v>1</v>
       </c>
       <c r="G4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="K4" t="s">
         <v>39</v>
@@ -2523,22 +2472,13 @@
         <v>38</v>
       </c>
       <c r="Q4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="R4" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="S4" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="U4" t="s">
-        <v>103</v>
-      </c>
-      <c r="V4" t="s">
-        <v>104</v>
-      </c>
-      <c r="W4" t="s">
-        <v>105</v>
+        <v>71</v>
       </c>
       <c r="Z4" t="str" cm="1">
         <f t="array" aca="1" ref="Z4:Z12" ca="1">_xlfn.UNIQUE((_xlfn.VSTACK(INDIRECT("CfgIssueTypes[IssueType.Name]"),INDIRECT("CfgIgnoreList[IgnoreList.Name]"))))</f>
@@ -2553,25 +2493,16 @@
         <v>44</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="Q5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="R5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="S5" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="U5" t="s">
-        <v>106</v>
-      </c>
-      <c r="V5" t="s">
-        <v>107</v>
-      </c>
-      <c r="W5" t="s">
-        <v>108</v>
+        <v>72</v>
       </c>
       <c r="Z5" t="str">
         <f ca="1"/>
@@ -2586,21 +2517,15 @@
         <v>33</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="Q6" t="s">
-        <v>87</v>
+        <v>86</v>
+      </c>
+      <c r="R6" t="s">
+        <v>102</v>
       </c>
       <c r="S6" s="7"/>
-      <c r="U6" t="s">
-        <v>109</v>
-      </c>
-      <c r="V6" t="s">
-        <v>110</v>
-      </c>
-      <c r="W6" t="s">
-        <v>111</v>
-      </c>
       <c r="Z6" t="str">
         <f ca="1"/>
         <v>Bug</v>
@@ -2612,28 +2537,16 @@
       <c r="K7" t="s">
         <v>41</v>
       </c>
-      <c r="M7" t="s">
-        <v>45</v>
-      </c>
       <c r="O7" s="1" t="s">
         <v>42</v>
       </c>
       <c r="Q7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="R7" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="S7" s="7"/>
-      <c r="U7" t="s">
-        <v>112</v>
-      </c>
-      <c r="V7" t="s">
-        <v>113</v>
-      </c>
-      <c r="W7" t="s">
-        <v>114</v>
-      </c>
       <c r="Z7" t="str">
         <f ca="1"/>
         <v>Epic</v>
@@ -2643,21 +2556,18 @@
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="K8" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>103</v>
+      </c>
+      <c r="R8">
+        <v>7</v>
       </c>
       <c r="S8" s="7"/>
-      <c r="U8" t="s">
-        <v>115</v>
-      </c>
-      <c r="V8" t="s">
-        <v>117</v>
-      </c>
-      <c r="W8" t="s">
-        <v>116</v>
-      </c>
       <c r="Z8" t="str">
         <f ca="1"/>
         <v>Sub-Task</v>
@@ -2666,49 +2576,40 @@
     <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
+      <c r="K9" t="s">
+        <v>101</v>
+      </c>
       <c r="O9" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="Q9" t="s">
+        <v>88</v>
+      </c>
+      <c r="R9" t="s">
         <v>89</v>
-      </c>
-      <c r="R9" t="s">
-        <v>90</v>
       </c>
       <c r="S9" s="7"/>
       <c r="Z9" t="str">
         <f ca="1"/>
-        <v>Comment</v>
+        <v>Initiative</v>
       </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
-      <c r="Q10" t="s">
-        <v>118</v>
-      </c>
-      <c r="R10" t="s">
-        <v>119</v>
-      </c>
       <c r="S10" s="7"/>
       <c r="Z10" t="str">
         <f ca="1"/>
-        <v>Skip</v>
+        <v>Comment</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
-      <c r="Q11" t="s">
-        <v>120</v>
-      </c>
-      <c r="R11" t="s">
-        <v>121</v>
-      </c>
       <c r="S11" s="7"/>
       <c r="Z11" t="str">
         <f ca="1"/>
-        <v>Note</v>
+        <v>Skip</v>
       </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.25">
@@ -2716,7 +2617,7 @@
       <c r="E12" s="2"/>
       <c r="Z12" t="str">
         <f ca="1"/>
-        <v>WorkItem</v>
+        <v>Note</v>
       </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.25">
@@ -2784,26 +2685,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FB038601AF41D04A88A4BD446922F1A8" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e8d32171d27ae41230d53456f24efae5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c471fd26-9765-4fbe-b6fd-c17c1e55c974" xmlns:ns3="9df69692-83aa-4c55-88c1-62abad05f4fe" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f2fb84de5621acf32f385a2ba90fb29" ns2:_="" ns3:_="">
     <xsd:import namespace="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
@@ -3032,10 +2913,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2C983B91-58B3-4C2C-AC55-FFEC9F0DB5F6}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
+    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3052,20 +2964,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2C983B91-58B3-4C2C-AC55-FFEC9F0DB5F6}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
-    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
JT-306 chore: layout of the import template files
</commit_message>
<xml_diff>
--- a/resources/templates/ImportTemplate.xlsx
+++ b/resources/templates/ImportTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workdir\DeerHide\sources\jira-toolkit\resources\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19EF8646-AAC6-4786-B8CE-C82C9A8B8D04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{110EB2ED-6994-4498-ACC7-09390093827A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15060" yWindow="5175" windowWidth="43200" windowHeight="23445" activeTab="1" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
+    <workbookView xWindow="8085" yWindow="4980" windowWidth="43200" windowHeight="23445" activeTab="1" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset" sheetId="1" r:id="rId1"/>
@@ -1128,12 +1128,6 @@
       </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
       <alignment vertical="top"/>
     </dxf>
     <dxf>
@@ -1274,6 +1268,12 @@
     </dxf>
     <dxf>
       <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1311,55 +1311,55 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" name="JiraDataset" displayName="JiraDataset" ref="A1:AJ3" totalsRowShown="0" headerRowDxfId="55" dataDxfId="54">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" name="JiraDataset" displayName="JiraDataset" ref="A1:AJ3" totalsRowShown="0" headerRowDxfId="53" dataDxfId="52">
   <autoFilter ref="A1:AJ3" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}"/>
   <tableColumns count="36">
-    <tableColumn id="3" xr3:uid="{AF2EC907-349C-4651-852D-6E39C61E17FF}" name="Priority" dataDxfId="53"/>
-    <tableColumn id="2" xr3:uid="{E90C51F2-4386-421F-A3E4-E2CA9D43D396}" name="IssueType" dataDxfId="52"/>
-    <tableColumn id="1" xr3:uid="{BBAD373B-BA13-47E4-9F74-565F4D9E9680}" name="Summary" dataDxfId="51"/>
-    <tableColumn id="4" xr3:uid="{026E5B97-FAFC-4E46-860E-0B0C976B1148}" name="Issue Key" dataDxfId="50"/>
-    <tableColumn id="5" xr3:uid="{A2C262E8-D544-4669-99F1-151EDE081654}" name="Description" dataDxfId="49"/>
-    <tableColumn id="7" xr3:uid="{0FAD1ACC-432E-462C-8B89-71540710BCB5}" name="FixVersion" dataDxfId="48"/>
-    <tableColumn id="28" xr3:uid="{07F3030C-7187-4B16-BBDB-798304851975}" name="Assignee.Name" dataDxfId="47"/>
-    <tableColumn id="8" xr3:uid="{8C7FB8DB-A85B-4189-93D8-0F0D4EEEF81B}" name="Component" dataDxfId="46"/>
-    <tableColumn id="9" xr3:uid="{DC5101A8-1204-44D2-BC2C-FEE1A4EFE7C1}" name="Sprint Name" dataDxfId="45"/>
-    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="44"/>
-    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="43"/>
-    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="42"/>
-    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="41"/>
-    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="40">
+    <tableColumn id="3" xr3:uid="{AF2EC907-349C-4651-852D-6E39C61E17FF}" name="Priority" dataDxfId="51"/>
+    <tableColumn id="2" xr3:uid="{E90C51F2-4386-421F-A3E4-E2CA9D43D396}" name="IssueType" dataDxfId="50"/>
+    <tableColumn id="1" xr3:uid="{BBAD373B-BA13-47E4-9F74-565F4D9E9680}" name="Summary" dataDxfId="49"/>
+    <tableColumn id="4" xr3:uid="{026E5B97-FAFC-4E46-860E-0B0C976B1148}" name="Issue Key" dataDxfId="48"/>
+    <tableColumn id="5" xr3:uid="{A2C262E8-D544-4669-99F1-151EDE081654}" name="Description" dataDxfId="47"/>
+    <tableColumn id="7" xr3:uid="{0FAD1ACC-432E-462C-8B89-71540710BCB5}" name="FixVersion" dataDxfId="46"/>
+    <tableColumn id="28" xr3:uid="{07F3030C-7187-4B16-BBDB-798304851975}" name="Assignee.Name" dataDxfId="45"/>
+    <tableColumn id="8" xr3:uid="{8C7FB8DB-A85B-4189-93D8-0F0D4EEEF81B}" name="Component" dataDxfId="44"/>
+    <tableColumn id="9" xr3:uid="{DC5101A8-1204-44D2-BC2C-FEE1A4EFE7C1}" name="Sprint Name" dataDxfId="43"/>
+    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="42"/>
+    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="41"/>
+    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="40"/>
+    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="39"/>
+    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="38">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[IssueType]]="Epic",JiraDataset[[#This Row],[Summary]],"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="27" xr3:uid="{911C8FDC-5528-43FC-BDF4-D4761F03C0E5}" name="Child-Issue" dataDxfId="39"/>
-    <tableColumn id="41" xr3:uid="{AB248E07-9BFA-42CC-BC41-B4234F677BFB}" name="Child-Issue1" dataDxfId="38"/>
-    <tableColumn id="29" xr3:uid="{89D12135-F3E3-4253-844F-1B9A54169953}" name="Child-Issue2" dataDxfId="37"/>
-    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="36"/>
-    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="35"/>
-    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="34"/>
-    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="33"/>
-    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="32"/>
-    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="31"/>
-    <tableColumn id="18" xr3:uid="{16B98070-7F8A-4FC7-AD99-EA81D0BD26AB}" name="Labels6" dataDxfId="30"/>
-    <tableColumn id="19" xr3:uid="{016EAEF4-8EA9-408B-9F1A-ECFB17E81C77}" name="Labels7" dataDxfId="29"/>
-    <tableColumn id="26" xr3:uid="{8263F9EC-BF0A-46F7-BA83-6083A4262B91}" name="Labels8" dataDxfId="28"/>
-    <tableColumn id="20" xr3:uid="{389B11C5-1B22-48C0-BCA2-72F050425FA1}" name="Labels9" dataDxfId="27"/>
-    <tableColumn id="25" xr3:uid="{AE95F8A2-F7F0-4985-9AE6-4201B9792775}" name="Labels10" dataDxfId="26"/>
-    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="25">
+    <tableColumn id="27" xr3:uid="{911C8FDC-5528-43FC-BDF4-D4761F03C0E5}" name="Child-Issue" dataDxfId="37"/>
+    <tableColumn id="41" xr3:uid="{AB248E07-9BFA-42CC-BC41-B4234F677BFB}" name="Child-Issue1" dataDxfId="36"/>
+    <tableColumn id="29" xr3:uid="{89D12135-F3E3-4253-844F-1B9A54169953}" name="Child-Issue2" dataDxfId="35"/>
+    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="34"/>
+    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="33"/>
+    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="32"/>
+    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="31"/>
+    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="30"/>
+    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="29"/>
+    <tableColumn id="18" xr3:uid="{16B98070-7F8A-4FC7-AD99-EA81D0BD26AB}" name="Labels6" dataDxfId="28"/>
+    <tableColumn id="19" xr3:uid="{016EAEF4-8EA9-408B-9F1A-ECFB17E81C77}" name="Labels7" dataDxfId="27"/>
+    <tableColumn id="26" xr3:uid="{8263F9EC-BF0A-46F7-BA83-6083A4262B91}" name="Labels8" dataDxfId="26"/>
+    <tableColumn id="20" xr3:uid="{389B11C5-1B22-48C0-BCA2-72F050425FA1}" name="Labels9" dataDxfId="25"/>
+    <tableColumn id="25" xr3:uid="{AE95F8A2-F7F0-4985-9AE6-4201B9792775}" name="Labels10" dataDxfId="24"/>
+    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="23">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], Config!$D$4:$E$9, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="24">
+    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="22">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="23">
+    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="21">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Feature Pod Label", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="22">
+    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="20">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], Config!$A$4:$B$24, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="21">
+    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="19">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("jira.project.key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="20">
+    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="18">
       <calculatedColumnFormula array="1">IF(
   JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
   "",
@@ -1375,7 +1375,7 @@
   )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="19">
+    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="17">
       <calculatedColumnFormula array="1">IFERROR(
     _xlfn.IFS(
         JiraDataset[[#This Row],[IssueType]] = cfg_type_comment,"SKIP",
@@ -1385,7 +1385,7 @@
     cfg_type_workitem
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="18"/>
+    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1438,7 +1438,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}" name="CfgPriorities" displayName="CfgPriorities" ref="O3:O9" totalsRowShown="0">
   <autoFilter ref="O3:O9" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="17"/>
+    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="55"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1472,7 +1472,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{D4E1611F-A2CF-465D-A219-1759EA66687D}" name="Name"/>
     <tableColumn id="2" xr3:uid="{174D0D86-B1AA-4BF7-AC91-FCACFC898851}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Remark" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Remark" dataDxfId="54"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1809,10 +1809,10 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.7109375" customWidth="1"/>
+    <col min="3" max="3" width="41.140625" customWidth="1"/>
     <col min="4" max="4" width="11.85546875" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="33" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="46.28515625" customWidth="1"/>
+    <col min="5" max="5" width="71.28515625" customWidth="1"/>
+    <col min="6" max="6" width="20.85546875" customWidth="1"/>
     <col min="7" max="7" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22.5703125" customWidth="1"/>
     <col min="9" max="9" width="14" bestFit="1" customWidth="1"/>
@@ -2685,6 +2685,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FB038601AF41D04A88A4BD446922F1A8" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e8d32171d27ae41230d53456f24efae5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c471fd26-9765-4fbe-b6fd-c17c1e55c974" xmlns:ns3="9df69692-83aa-4c55-88c1-62abad05f4fe" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f2fb84de5621acf32f385a2ba90fb29" ns2:_="" ns3:_="">
     <xsd:import namespace="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
@@ -2913,27 +2933,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FFE630F-6530-4863-AB67-8477539A0000}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
+    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2C983B91-58B3-4C2C-AC55-FFEC9F0DB5F6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2950,23 +2969,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FFE630F-6530-4863-AB67-8477539A0000}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
-    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
JT-85 Update ImportTemplate.xlsx to support CfgTeams tables
</commit_message>
<xml_diff>
--- a/resources/templates/ImportTemplate.xlsx
+++ b/resources/templates/ImportTemplate.xlsx
@@ -8,23 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workdir\DeerHide\sources\jira-toolkit\resources\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{110EB2ED-6994-4498-ACC7-09390093827A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4062769F-6A46-4AC5-A90C-0B6BE8F81ED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8085" yWindow="4980" windowWidth="43200" windowHeight="23445" activeTab="1" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
+    <workbookView xWindow="3900" yWindow="5655" windowWidth="43200" windowHeight="23445" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset" sheetId="1" r:id="rId1"/>
     <sheet name="Config" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="cfg_labels_ft_label">Config!$R$5</definedName>
-    <definedName name="cfg_labels_ft_name">Config!$R$5</definedName>
-    <definedName name="cfg_labels_imported">Config!$R$4</definedName>
-    <definedName name="cfg_projectKey">Config!$R$7</definedName>
-    <definedName name="cfg_type_comment">Config!$M$4</definedName>
-    <definedName name="cfg_type_note">Config!$M$6</definedName>
-    <definedName name="cfg_type_skip">Config!$M$5</definedName>
-    <definedName name="cfg_type_workitem">Config!$M$7</definedName>
+    <definedName name="cfg_labels_ft_label">Config!$U$5</definedName>
+    <definedName name="cfg_labels_ft_name">Config!$U$5</definedName>
+    <definedName name="cfg_labels_imported">Config!$U$4</definedName>
+    <definedName name="cfg_projectKey">Config!$U$7</definedName>
+    <definedName name="cfg_type_comment">Config!$P$4</definedName>
+    <definedName name="cfg_type_note">Config!$P$6</definedName>
+    <definedName name="cfg_type_skip">Config!$P$5</definedName>
+    <definedName name="cfg_type_workitem">Config!$P$7</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="110">
   <si>
     <t>IssueType</t>
   </si>
@@ -384,6 +384,21 @@
   </si>
   <si>
     <t>PROJECT-KEY</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>Teams</t>
+  </si>
+  <si>
+    <t>Team.Name</t>
+  </si>
+  <si>
+    <t>Team.ID</t>
+  </si>
+  <si>
+    <t>Team ID</t>
   </si>
 </sst>
 </file>
@@ -984,7 +999,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="56">
+  <dxfs count="57">
     <dxf>
       <fill>
         <patternFill patternType="darkUp"/>
@@ -1126,6 +1141,9 @@
           <bgColor rgb="FFFF99CC"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment vertical="top"/>
@@ -1305,61 +1323,62 @@
 <file path=xl/namedSheetViews/namedSheetView1.xml><?xml version="1.0" encoding="utf-8"?>
 <namedSheetViews xmlns="http://schemas.microsoft.com/office/spreadsheetml/2019/namedsheetviews" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <namedSheetView name="View1" id="{77233F75-225A-4D7F-8A86-543E0A8C6E58}">
-    <nsvFilter filterId="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" ref="A1:AJ3" tableId="1"/>
+    <nsvFilter filterId="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" ref="A1:AK3" tableId="1"/>
   </namedSheetView>
 </namedSheetViews>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" name="JiraDataset" displayName="JiraDataset" ref="A1:AJ3" totalsRowShown="0" headerRowDxfId="53" dataDxfId="52">
-  <autoFilter ref="A1:AJ3" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}"/>
-  <tableColumns count="36">
-    <tableColumn id="3" xr3:uid="{AF2EC907-349C-4651-852D-6E39C61E17FF}" name="Priority" dataDxfId="51"/>
-    <tableColumn id="2" xr3:uid="{E90C51F2-4386-421F-A3E4-E2CA9D43D396}" name="IssueType" dataDxfId="50"/>
-    <tableColumn id="1" xr3:uid="{BBAD373B-BA13-47E4-9F74-565F4D9E9680}" name="Summary" dataDxfId="49"/>
-    <tableColumn id="4" xr3:uid="{026E5B97-FAFC-4E46-860E-0B0C976B1148}" name="Issue Key" dataDxfId="48"/>
-    <tableColumn id="5" xr3:uid="{A2C262E8-D544-4669-99F1-151EDE081654}" name="Description" dataDxfId="47"/>
-    <tableColumn id="7" xr3:uid="{0FAD1ACC-432E-462C-8B89-71540710BCB5}" name="FixVersion" dataDxfId="46"/>
-    <tableColumn id="28" xr3:uid="{07F3030C-7187-4B16-BBDB-798304851975}" name="Assignee.Name" dataDxfId="45"/>
-    <tableColumn id="8" xr3:uid="{8C7FB8DB-A85B-4189-93D8-0F0D4EEEF81B}" name="Component" dataDxfId="44"/>
-    <tableColumn id="9" xr3:uid="{DC5101A8-1204-44D2-BC2C-FEE1A4EFE7C1}" name="Sprint Name" dataDxfId="43"/>
-    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="42"/>
-    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="41"/>
-    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="40"/>
-    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="39"/>
-    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="38">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" name="JiraDataset" displayName="JiraDataset" ref="A1:AK3" totalsRowShown="0" headerRowDxfId="54" dataDxfId="53">
+  <autoFilter ref="A1:AK3" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}"/>
+  <tableColumns count="37">
+    <tableColumn id="3" xr3:uid="{AF2EC907-349C-4651-852D-6E39C61E17FF}" name="Priority" dataDxfId="52"/>
+    <tableColumn id="2" xr3:uid="{E90C51F2-4386-421F-A3E4-E2CA9D43D396}" name="IssueType" dataDxfId="51"/>
+    <tableColumn id="1" xr3:uid="{BBAD373B-BA13-47E4-9F74-565F4D9E9680}" name="Summary" dataDxfId="50"/>
+    <tableColumn id="4" xr3:uid="{026E5B97-FAFC-4E46-860E-0B0C976B1148}" name="Issue Key" dataDxfId="49"/>
+    <tableColumn id="5" xr3:uid="{A2C262E8-D544-4669-99F1-151EDE081654}" name="Description" dataDxfId="48"/>
+    <tableColumn id="7" xr3:uid="{0FAD1ACC-432E-462C-8B89-71540710BCB5}" name="FixVersion" dataDxfId="47"/>
+    <tableColumn id="28" xr3:uid="{07F3030C-7187-4B16-BBDB-798304851975}" name="Assignee.Name" dataDxfId="46"/>
+    <tableColumn id="8" xr3:uid="{8C7FB8DB-A85B-4189-93D8-0F0D4EEEF81B}" name="Component" dataDxfId="45"/>
+    <tableColumn id="31" xr3:uid="{28FC7838-B632-4214-BEDE-FDACBD086707}" name="Team" dataDxfId="16"/>
+    <tableColumn id="9" xr3:uid="{DC5101A8-1204-44D2-BC2C-FEE1A4EFE7C1}" name="Sprint Name" dataDxfId="44"/>
+    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="43"/>
+    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="42"/>
+    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="41"/>
+    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="40"/>
+    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="39">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[IssueType]]="Epic",JiraDataset[[#This Row],[Summary]],"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="27" xr3:uid="{911C8FDC-5528-43FC-BDF4-D4761F03C0E5}" name="Child-Issue" dataDxfId="37"/>
-    <tableColumn id="41" xr3:uid="{AB248E07-9BFA-42CC-BC41-B4234F677BFB}" name="Child-Issue1" dataDxfId="36"/>
-    <tableColumn id="29" xr3:uid="{89D12135-F3E3-4253-844F-1B9A54169953}" name="Child-Issue2" dataDxfId="35"/>
-    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="34"/>
-    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="33"/>
-    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="32"/>
-    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="31"/>
-    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="30"/>
-    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="29"/>
-    <tableColumn id="18" xr3:uid="{16B98070-7F8A-4FC7-AD99-EA81D0BD26AB}" name="Labels6" dataDxfId="28"/>
-    <tableColumn id="19" xr3:uid="{016EAEF4-8EA9-408B-9F1A-ECFB17E81C77}" name="Labels7" dataDxfId="27"/>
-    <tableColumn id="26" xr3:uid="{8263F9EC-BF0A-46F7-BA83-6083A4262B91}" name="Labels8" dataDxfId="26"/>
-    <tableColumn id="20" xr3:uid="{389B11C5-1B22-48C0-BCA2-72F050425FA1}" name="Labels9" dataDxfId="25"/>
-    <tableColumn id="25" xr3:uid="{AE95F8A2-F7F0-4985-9AE6-4201B9792775}" name="Labels10" dataDxfId="24"/>
-    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="23">
-      <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], Config!$D$4:$E$9, 2, FALSE), ""))</calculatedColumnFormula>
+    <tableColumn id="27" xr3:uid="{911C8FDC-5528-43FC-BDF4-D4761F03C0E5}" name="Child-Issue" dataDxfId="38"/>
+    <tableColumn id="41" xr3:uid="{AB248E07-9BFA-42CC-BC41-B4234F677BFB}" name="Child-Issue1" dataDxfId="37"/>
+    <tableColumn id="29" xr3:uid="{89D12135-F3E3-4253-844F-1B9A54169953}" name="Child-Issue2" dataDxfId="36"/>
+    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="35"/>
+    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="34"/>
+    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="33"/>
+    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="32"/>
+    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="31"/>
+    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="30"/>
+    <tableColumn id="18" xr3:uid="{16B98070-7F8A-4FC7-AD99-EA81D0BD26AB}" name="Labels6" dataDxfId="29"/>
+    <tableColumn id="19" xr3:uid="{016EAEF4-8EA9-408B-9F1A-ECFB17E81C77}" name="Labels7" dataDxfId="28"/>
+    <tableColumn id="26" xr3:uid="{8263F9EC-BF0A-46F7-BA83-6083A4262B91}" name="Labels8" dataDxfId="27"/>
+    <tableColumn id="20" xr3:uid="{389B11C5-1B22-48C0-BCA2-72F050425FA1}" name="Labels9" dataDxfId="26"/>
+    <tableColumn id="25" xr3:uid="{AE95F8A2-F7F0-4985-9AE6-4201B9792775}" name="Labels10" dataDxfId="25"/>
+    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="24">
+      <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], Config!$G$4:$H$9, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="22">
+    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="23">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="21">
+    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="22">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Feature Pod Label", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="20">
+    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="21">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], Config!$A$4:$B$24, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="19">
+    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="20">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("jira.project.key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="18">
+    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="19">
       <calculatedColumnFormula array="1">IF(
   JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
   "",
@@ -1375,7 +1394,7 @@
   )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="17">
+    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="18">
       <calculatedColumnFormula array="1">IFERROR(
     _xlfn.IFS(
         JiraDataset[[#This Row],[IssueType]] = cfg_type_comment,"SKIP",
@@ -1385,15 +1404,15 @@
     cfg_type_workitem
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="16"/>
+    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3EF499BE-ED9A-4C28-BC5A-BCDEF51C613F}" name="CfgCustomFields" displayName="CfgCustomFields" ref="U3:X4" insertRow="1" totalsRowShown="0">
-  <autoFilter ref="U3:X4" xr:uid="{3EF499BE-ED9A-4C28-BC5A-BCDEF51C613F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3EF499BE-ED9A-4C28-BC5A-BCDEF51C613F}" name="CfgCustomFields" displayName="CfgCustomFields" ref="X3:AA4" insertRow="1" totalsRowShown="0">
+  <autoFilter ref="X3:AA4" xr:uid="{3EF499BE-ED9A-4C28-BC5A-BCDEF51C613F}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{44010E5A-E449-477A-BFB0-2ECA215E3FEB}" name="Name"/>
     <tableColumn id="2" xr3:uid="{0E558995-744D-4813-9A4E-F64FFF5047AE}" name="Id"/>
@@ -1404,9 +1423,20 @@
 </table>
 </file>
 
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{9BDE4941-2A84-46A5-8151-88377A8724D2}" name="CfgTeams" displayName="CfgTeams" ref="D3:E4" totalsRowShown="0">
+  <autoFilter ref="D3:E4" xr:uid="{9BDE4941-2A84-46A5-8151-88377A8724D2}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{00649780-E35F-4B89-8C72-05E0797C267E}" name="Team.Name"/>
+    <tableColumn id="2" xr3:uid="{AE7CB114-5EE3-4BFF-9E4E-5034242719C9}" name="Team.ID"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{93F2D14D-2ABD-4171-895D-1041B0893491}" name="CfgComponents" displayName="CfgComponents" ref="I3:I5" totalsRowShown="0">
-  <autoFilter ref="I3:I5" xr:uid="{93F2D14D-2ABD-4171-895D-1041B0893491}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{93F2D14D-2ABD-4171-895D-1041B0893491}" name="CfgComponents" displayName="CfgComponents" ref="L3:L5" totalsRowShown="0">
+  <autoFilter ref="L3:L5" xr:uid="{93F2D14D-2ABD-4171-895D-1041B0893491}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{10F6CCA4-1068-4FC8-AB82-E48B87DB0F71}" name="Component.Name"/>
   </tableColumns>
@@ -1415,8 +1445,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{7007FF9D-9384-422B-8DB3-300D782E5FE6}" name="CfgFixVersions" displayName="CfgFixVersions" ref="G3:G5" totalsRowShown="0">
-  <autoFilter ref="G3:G5" xr:uid="{7007FF9D-9384-422B-8DB3-300D782E5FE6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{7007FF9D-9384-422B-8DB3-300D782E5FE6}" name="CfgFixVersions" displayName="CfgFixVersions" ref="J3:J5" totalsRowShown="0">
+  <autoFilter ref="J3:J5" xr:uid="{7007FF9D-9384-422B-8DB3-300D782E5FE6}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{E20FAA91-E54E-42EA-9BFF-2FDA27CD5D33}" name="FixVersion.Name"/>
   </tableColumns>
@@ -1425,8 +1455,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{6F085B8C-1322-4F43-A516-588923936259}" name="CfgIssueTypes" displayName="CfgIssueTypes" ref="K3:K9" totalsRowShown="0">
-  <autoFilter ref="K3:K9" xr:uid="{6F085B8C-1322-4F43-A516-588923936259}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{6F085B8C-1322-4F43-A516-588923936259}" name="CfgIssueTypes" displayName="CfgIssueTypes" ref="N3:N9" totalsRowShown="0">
+  <autoFilter ref="N3:N9" xr:uid="{6F085B8C-1322-4F43-A516-588923936259}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{A92436BC-3156-493F-B5C6-0BB6B51F89EB}" name="IssueType.Name"/>
   </tableColumns>
@@ -1435,10 +1465,10 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}" name="CfgPriorities" displayName="CfgPriorities" ref="O3:O9" totalsRowShown="0">
-  <autoFilter ref="O3:O9" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}" name="CfgPriorities" displayName="CfgPriorities" ref="R3:R9" totalsRowShown="0">
+  <autoFilter ref="R3:R9" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="55"/>
+    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="56"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1456,8 +1486,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{72674B63-54C8-47AC-9FF0-4034C2D499BA}" name="CfgSprints" displayName="CfgSprints" ref="D3:E5" totalsRowShown="0">
-  <autoFilter ref="D3:E5" xr:uid="{72674B63-54C8-47AC-9FF0-4034C2D499BA}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{72674B63-54C8-47AC-9FF0-4034C2D499BA}" name="CfgSprints" displayName="CfgSprints" ref="G3:H5" totalsRowShown="0">
+  <autoFilter ref="G3:H5" xr:uid="{72674B63-54C8-47AC-9FF0-4034C2D499BA}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{397B719B-4CC6-4F47-8F3C-168F13ED56DA}" name="Sprint.Name"/>
     <tableColumn id="2" xr3:uid="{2FD208E7-540E-4D07-9144-6E9F3065D9DE}" name="Sprint.ID"/>
@@ -1467,20 +1497,20 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{383560BC-B1F2-44B6-B877-188131EFA163}" name="CfgAutofieldValues" displayName="CfgAutofieldValues" ref="Q3:S9" totalsRowShown="0">
-  <autoFilter ref="Q3:S9" xr:uid="{383560BC-B1F2-44B6-B877-188131EFA163}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{383560BC-B1F2-44B6-B877-188131EFA163}" name="CfgAutofieldValues" displayName="CfgAutofieldValues" ref="T3:V9" totalsRowShown="0">
+  <autoFilter ref="T3:V9" xr:uid="{383560BC-B1F2-44B6-B877-188131EFA163}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{D4E1611F-A2CF-465D-A219-1759EA66687D}" name="Name"/>
     <tableColumn id="2" xr3:uid="{174D0D86-B1AA-4BF7-AC91-FCACFC898851}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Remark" dataDxfId="54"/>
+    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Remark" dataDxfId="55"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{0ABE2B38-573A-4A51-8D54-C217B9D7D54F}" name="CfgIgnoreList" displayName="CfgIgnoreList" ref="M3:M6" totalsRowShown="0">
-  <autoFilter ref="M3:M6" xr:uid="{0ABE2B38-573A-4A51-8D54-C217B9D7D54F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{0ABE2B38-573A-4A51-8D54-C217B9D7D54F}" name="CfgIgnoreList" displayName="CfgIgnoreList" ref="P3:P6" totalsRowShown="0">
+  <autoFilter ref="P3:P6" xr:uid="{0ABE2B38-573A-4A51-8D54-C217B9D7D54F}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{1396737E-05D6-4D62-AF56-4B039C3A3607}" name="IgnoreList.Name"/>
   </tableColumns>
@@ -1805,43 +1835,37 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F73058B-F76D-4AAE-8108-6C4469E9D8B5}">
-  <dimension ref="A1:AK3"/>
+  <dimension ref="A1:AL3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.140625" customWidth="1"/>
-    <col min="4" max="4" width="11.85546875" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="71.28515625" customWidth="1"/>
+    <col min="3" max="3" width="50" customWidth="1"/>
+    <col min="4" max="4" width="50" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="50" customWidth="1"/>
     <col min="6" max="6" width="20.85546875" customWidth="1"/>
-    <col min="7" max="7" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.5703125" customWidth="1"/>
-    <col min="9" max="9" width="14" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.28515625" customWidth="1"/>
-    <col min="13" max="13" width="14.42578125" customWidth="1"/>
-    <col min="14" max="14" width="14.28515625" customWidth="1"/>
-    <col min="15" max="15" width="0" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="22.28515625" hidden="1" customWidth="1"/>
-    <col min="17" max="17" width="12.85546875" hidden="1" customWidth="1"/>
-    <col min="18" max="18" width="12.42578125" customWidth="1"/>
-    <col min="19" max="19" width="15.5703125" customWidth="1"/>
-    <col min="20" max="20" width="12.85546875" customWidth="1"/>
-    <col min="21" max="21" width="10" customWidth="1"/>
-    <col min="22" max="22" width="10" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="10" customWidth="1"/>
-    <col min="24" max="24" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10" customWidth="1" outlineLevel="1"/>
-    <col min="31" max="31" width="10" customWidth="1"/>
-    <col min="32" max="32" width="8.7109375" customWidth="1" outlineLevel="1"/>
-    <col min="33" max="34" width="13.140625" customWidth="1" outlineLevel="1"/>
-    <col min="35" max="35" width="11.42578125" customWidth="1" outlineLevel="1"/>
-    <col min="36" max="37" width="13.7109375" customWidth="1" outlineLevel="1"/>
-    <col min="38" max="38" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="18.7109375" customWidth="1"/>
-    <col min="41" max="41" width="87.28515625" customWidth="1"/>
+    <col min="7" max="10" width="14.28515625" customWidth="1"/>
+    <col min="11" max="11" width="11.42578125" customWidth="1"/>
+    <col min="12" max="12" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.28515625" customWidth="1"/>
+    <col min="14" max="14" width="14.42578125" customWidth="1"/>
+    <col min="15" max="15" width="14.28515625" customWidth="1"/>
+    <col min="16" max="16" width="0" hidden="1" customWidth="1"/>
+    <col min="17" max="17" width="22.28515625" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="9.85546875" hidden="1" customWidth="1"/>
+    <col min="19" max="25" width="11.42578125" customWidth="1"/>
+    <col min="26" max="29" width="11.42578125" customWidth="1" outlineLevel="1"/>
+    <col min="30" max="31" width="10" customWidth="1" outlineLevel="1"/>
+    <col min="32" max="32" width="10" customWidth="1"/>
+    <col min="33" max="33" width="8.7109375" customWidth="1" outlineLevel="1"/>
+    <col min="34" max="35" width="13.140625" customWidth="1" outlineLevel="1"/>
+    <col min="36" max="36" width="11.42578125" customWidth="1" outlineLevel="1"/>
+    <col min="37" max="38" width="13.7109375" customWidth="1" outlineLevel="1"/>
+    <col min="39" max="39" width="36.5703125" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="18.7109375" customWidth="1"/>
+    <col min="42" max="42" width="87.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>1</v>
       </c>
@@ -1867,91 +1891,94 @@
         <v>7</v>
       </c>
       <c r="I1" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="J1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>83</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="U1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="V1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="W1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="X1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="X1" s="3" t="s">
+      <c r="Y1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="Y1" s="3" t="s">
+      <c r="Z1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="AA1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="AA1" s="3" t="s">
+      <c r="AB1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="AB1" s="3" t="s">
+      <c r="AC1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="AC1" s="3" t="s">
+      <c r="AD1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="AD1" s="3" t="s">
+      <c r="AE1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="AE1" s="3" t="s">
+      <c r="AF1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="AF1" s="3" t="s">
+      <c r="AG1" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="AG1" s="3" t="s">
+      <c r="AH1" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="AH1" s="4" t="s">
+      <c r="AI1" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="AI1" s="4" t="s">
+      <c r="AJ1" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="AJ1" s="3" t="s">
+      <c r="AK1" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
         <v>34</v>
@@ -1967,19 +1994,19 @@
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="3"/>
+      <c r="K2" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="K2" s="3">
+      <c r="L2" s="3">
         <v>1</v>
       </c>
-      <c r="L2" s="3"/>
       <c r="M2" s="3"/>
-      <c r="N2" s="3" t="str">
+      <c r="N2" s="3"/>
+      <c r="O2" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[IssueType]]="Epic",JiraDataset[[#This Row],[Summary]],"")</f>
         <v/>
       </c>
-      <c r="O2" s="3"/>
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
       <c r="R2" s="3"/>
@@ -1993,28 +2020,29 @@
       <c r="Z2" s="3"/>
       <c r="AA2" s="3"/>
       <c r="AB2" s="3"/>
-      <c r="AC2" s="3" t="str">
-        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], Config!$D$4:$E$9, 2, FALSE), ""))</f>
+      <c r="AC2" s="3"/>
+      <c r="AD2" s="3" t="str">
+        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], Config!$G$4:$H$9, 2, FALSE), ""))</f>
         <v/>
       </c>
-      <c r="AD2" s="3" t="str">
+      <c r="AE2" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
         <v/>
       </c>
-      <c r="AE2" s="8" t="str">
+      <c r="AF2" s="8" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Feature Pod Label", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
         <v/>
       </c>
-      <c r="AF2" s="3" t="str">
+      <c r="AG2" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], Config!$A$4:$B$24, 2, FALSE), ""))</f>
         <v/>
       </c>
-      <c r="AG2" s="3" t="str">
+      <c r="AH2" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("jira.project.key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
         <v/>
       </c>
-      <c r="AH2" s="3" t="str" cm="1">
-        <f t="array" ref="AH2">IF(
+      <c r="AI2" s="3" t="str" cm="1">
+        <f t="array" ref="AI2">IF(
   JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
   "",
   _xlfn.LET(
@@ -2030,8 +2058,8 @@
 )</f>
         <v/>
       </c>
-      <c r="AI2" s="3" t="str" cm="1">
-        <f t="array" ref="AI2">IFERROR(
+      <c r="AJ2" s="3" t="str" cm="1">
+        <f t="array" ref="AJ2">IFERROR(
     _xlfn.IFS(
         JiraDataset[[#This Row],[IssueType]] = cfg_type_comment,"SKIP",
         JiraDataset[[#This Row],[IssueType]] = cfg_type_skip,"SKIP",
@@ -2041,9 +2069,9 @@
 )</f>
         <v>SKIP</v>
       </c>
-      <c r="AJ2" s="3"/>
+      <c r="AK2" s="3"/>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>47</v>
       </c>
@@ -2066,22 +2094,22 @@
       <c r="H3" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="3"/>
+      <c r="J3" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="K3" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="K3" s="3">
+      <c r="L3" s="3">
         <v>2</v>
       </c>
-      <c r="L3" s="3"/>
       <c r="M3" s="3"/>
-      <c r="N3" s="3" t="str">
+      <c r="N3" s="3"/>
+      <c r="O3" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[IssueType]]="Epic",JiraDataset[[#This Row],[Summary]],"")</f>
         <v>Test, Epic</v>
       </c>
-      <c r="O3" s="3"/>
       <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
       <c r="R3" s="3"/>
@@ -2095,28 +2123,29 @@
       <c r="Z3" s="3"/>
       <c r="AA3" s="3"/>
       <c r="AB3" s="3"/>
-      <c r="AC3" s="3">
-        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], Config!$D$4:$E$9, 2, FALSE), ""))</f>
+      <c r="AC3" s="3"/>
+      <c r="AD3" s="3">
+        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], Config!$G$4:$H$9, 2, FALSE), ""))</f>
         <v>1</v>
       </c>
-      <c r="AD3" s="3" t="str">
+      <c r="AE3" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
         <v>jt-imported</v>
       </c>
-      <c r="AE3" s="8" t="str">
+      <c r="AF3" s="8" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Feature Pod Label", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
         <v>pod_test</v>
       </c>
-      <c r="AF3" s="3" t="str">
+      <c r="AG3" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], Config!$A$4:$B$24, 2, FALSE), ""))</f>
         <v>AtlassianID (cloud) or Email (DC)</v>
       </c>
-      <c r="AG3" s="3" t="str">
+      <c r="AH3" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("jira.project.key", CfgAutofieldValues[Name], CfgAutofieldValues[Value]))</f>
         <v>PROJECT-KEY</v>
       </c>
-      <c r="AH3" s="3" cm="1">
-        <f t="array" ref="AH3">IF(
+      <c r="AI3" s="3" cm="1">
+        <f t="array" ref="AI3">IF(
   JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
   "",
   _xlfn.LET(
@@ -2132,8 +2161,8 @@
 )</f>
         <v>34560000</v>
       </c>
-      <c r="AI3" s="3" cm="1">
-        <f t="array" ref="AI3">IFERROR(
+      <c r="AJ3" s="3" cm="1">
+        <f t="array" ref="AJ3">IFERROR(
     _xlfn.IFS(
         JiraDataset[[#This Row],[IssueType]] = cfg_type_comment,"SKIP",
         JiraDataset[[#This Row],[IssueType]] = cfg_type_skip,"SKIP",
@@ -2143,12 +2172,12 @@
 )</f>
         <v>0</v>
       </c>
-      <c r="AJ3" s="3"/>
+      <c r="AK3" s="3"/>
     </row>
   </sheetData>
   <protectedRanges>
-    <protectedRange sqref="D4:N1048576 P4:AD1048576 C1:AB3 A1:A1048576" name="User Input"/>
-    <protectedRange algorithmName="SHA-512" hashValue="tpheD+JLADkhiyalt6vInlMwkILPZx4PVQN/k2vmwjOBdYUuHaXCrwtObHeFz5dJh9f853O84pZ1Rn9Ujz33+A==" saltValue="9ir5NB4CJc/69S/Eh84/mA==" spinCount="100000" sqref="AC1:AI3 AE4:AK1048576" name="Computed values"/>
+    <protectedRange sqref="D4:O1048576 Q4:AE1048576 C1:AC3 A1:A1048576" name="User Input"/>
+    <protectedRange algorithmName="SHA-512" hashValue="tpheD+JLADkhiyalt6vInlMwkILPZx4PVQN/k2vmwjOBdYUuHaXCrwtObHeFz5dJh9f853O84pZ1Rn9Ujz33+A==" saltValue="9ir5NB4CJc/69S/Eh84/mA==" spinCount="100000" sqref="AD1:AJ3 AF4:AL1048576" name="Computed values"/>
   </protectedRanges>
   <phoneticPr fontId="18" type="noConversion"/>
   <conditionalFormatting sqref="A2:A3 C2:C3">
@@ -2172,7 +2201,7 @@
       <formula>NOT(ISERROR(SEARCH("blocker",A2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:AJ3">
+  <conditionalFormatting sqref="A2:AK3">
     <cfRule type="expression" dxfId="10" priority="409" stopIfTrue="1">
       <formula>$B2=cfg_type_comment</formula>
     </cfRule>
@@ -2197,7 +2226,7 @@
       <formula>LEN(TRIM(B2))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2:AJ3">
+  <conditionalFormatting sqref="B2:AK3">
     <cfRule type="expression" dxfId="3" priority="1">
       <formula>$B2="Epic"</formula>
     </cfRule>
@@ -2210,49 +2239,52 @@
       <formula>LEN(TRIM(C2))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:L3">
+  <conditionalFormatting sqref="L2:M3">
     <cfRule type="containsBlanks" dxfId="0" priority="412">
-      <formula>LEN(TRIM(K2))=0</formula>
+      <formula>LEN(TRIM(L2))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations xWindow="1573" yWindow="665" count="21">
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" prompt="It must be a number (integer). This reference is only used during the import process." sqref="K2:L3" xr:uid="{005E18F2-4447-4781-8F18-5A58920A4F75}">
+  <dataValidations xWindow="1573" yWindow="665" count="22">
+    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" prompt="It must be a number (integer). This reference is only used during the import process." sqref="L2:M3" xr:uid="{005E18F2-4447-4781-8F18-5A58920A4F75}">
       <formula1>1</formula1>
       <formula2>1000</formula2>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="J2:J3" xr:uid="{386E3B68-2486-4DDE-BEB1-45F897521149}"/>
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" promptTitle="Warning" prompt="This field should be the Issue ID or Issue Key of the child tasks. (upstream linkage is not possible)._x000a__x000a__x000a_To link Epics and Stories, use the Epic Link from the Story Issue." sqref="O2:Q3" xr:uid="{D7BD960D-9CEA-4120-B2E3-2AE0D4661093}">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="K2:K3" xr:uid="{386E3B68-2486-4DDE-BEB1-45F897521149}"/>
+    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" promptTitle="Warning" prompt="This field should be the Issue ID or Issue Key of the child tasks. (upstream linkage is not possible)._x000a__x000a__x000a_To link Epics and Stories, use the Epic Link from the Story Issue." sqref="P2:R3" xr:uid="{D7BD960D-9CEA-4120-B2E3-2AE0D4661093}">
       <formula1>1</formula1>
       <formula2>1000</formula2>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Note" prompt="The content of this column will be ignored during the Jira import." sqref="AJ2:AJ3" xr:uid="{2DA3EDB6-7635-4349-8860-B614B5B71275}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Note" prompt="The content of this column will be ignored during the Jira import." sqref="AK2:AK3" xr:uid="{2DA3EDB6-7635-4349-8860-B614B5B71275}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Permissions" prompt="Updating Existing Issues requires global admin permissions" sqref="D2:D3" xr:uid="{D5E4A4BB-53C8-42DF-9B52-F5E00AC6407B}"/>
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" promptTitle="Warning" prompt="Use the Issue ID value to link this work item to an Epic_x000a__x000a_Story Issues are not Child-Issues and should have Epic Link instead. " sqref="M2:M3" xr:uid="{16C14239-D6AA-4935-8809-57760481D8F1}">
+    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" promptTitle="Warning" prompt="Use the Issue ID value to link this work item to an Epic_x000a__x000a_Story Issues are not Child-Issues and should have Epic Link instead. " sqref="N2:N3" xr:uid="{16C14239-D6AA-4935-8809-57760481D8F1}">
       <formula1>1</formula1>
       <formula2>1000</formula2>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="It must be a number (integer). This reference is only used during the import process." sqref="K1" xr:uid="{9C637146-F2E3-4D08-87A8-F70FD358E47E}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Use the Issue ID value to link this work item to an Epic_x000a__x000a_Story Issues are not Child-Issues and should have Epic Link instead. " sqref="M1" xr:uid="{A61138FD-C2B2-49D2-810B-69EAE2230B73}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="This field should be the Issue ID or Issue Key of the child tasks. (upstream linkage is not possible)._x000a__x000a__x000a_To link Epics and Stories, use the Epic Link from the Story Issue." sqref="O1:Q1" xr:uid="{BE6B7503-A11A-4130-9D63-988F0CFED80E}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="AUTOMATIC FIELD" prompt="Do not manually edit these!" sqref="AC2:AC3 AF1:AH3" xr:uid="{893DA5FE-9FD0-4D28-BBD0-3D7AEDECEACB}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="It must be a number (integer). This reference is only used during the import process." sqref="L1" xr:uid="{9C637146-F2E3-4D08-87A8-F70FD358E47E}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Use the Issue ID value to link this work item to an Epic_x000a__x000a_Story Issues are not Child-Issues and should have Epic Link instead. " sqref="N1" xr:uid="{A61138FD-C2B2-49D2-810B-69EAE2230B73}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="This field should be the Issue ID or Issue Key of the child tasks. (upstream linkage is not possible)._x000a__x000a__x000a_To link Epics and Stories, use the Epic Link from the Story Issue." sqref="P1:R1" xr:uid="{BE6B7503-A11A-4130-9D63-988F0CFED80E}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="AUTOMATIC FIELD" prompt="Do not manually edit these!" sqref="AD2:AD3 AG1:AI3" xr:uid="{893DA5FE-9FD0-4D28-BBD0-3D7AEDECEACB}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="H2:H3" xr:uid="{65EDED96-6789-400B-B504-6BC3F5A79E70}">
       <formula1>INDIRECT("CfgComponents[Component.Name]")</formula1>
     </dataValidation>
     <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" error="must be a valid fixversion" sqref="G2:G3" xr:uid="{44FDC20A-8BF5-49B5-9D2C-3A1FE5A7D835}">
       <formula1>INDIRECT("CfgAssignees[Assignee.Name]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="I2:I3" xr:uid="{A898E2E7-BC45-4B88-BA1E-4AAA377361D4}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="J2:J3" xr:uid="{A898E2E7-BC45-4B88-BA1E-4AAA377361D4}">
       <formula1>INDIRECT("CfgSprints[Sprint.Name]")</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showErrorMessage="1" promptTitle="Warning" prompt="Field only used for Epic Issues, so they can be referenced in Story Issues via the Epic Link field.," sqref="N2:N3 L2:L3" xr:uid="{541AD292-0123-4B65-9663-081991FDF0C1}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Field only used for Epic Issues, so they can be referenced in Story Issues via the Epic Link field.," sqref="L1" xr:uid="{64C73155-DEE7-497D-8A98-01E54655ACA8}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="It must be a number (integer) or the Work Item key. This reference is only used during the import process to set the parent." sqref="L1" xr:uid="{8A2BE248-5762-43AD-9C47-C5A92A2E2357}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Field only used for Epic work item, so they can be referenced in Story work items via the Epic Link field. _x000a_DC Only" sqref="N1" xr:uid="{E8F6E005-1F9B-40F3-B24C-E2A3D286C532}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="Creation Marker (Config Sheet)" prompt="Do not manually edit these!" sqref="AD1:AD3" xr:uid="{412C516D-E091-4DDD-9C14-C33AC653C143}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="Feature Pod Label (Config Sheet)" prompt="Do not manually edit these!" sqref="AE1:AE3" xr:uid="{D2234141-379F-4413-AB08-6835BD9FF967}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="AUTOMATIC FIELD" prompt="Do not manually edit these! SKIP types won't be imported into Jira" sqref="AI1:AI3" xr:uid="{5A336857-7D14-4900-8734-BED680BE5154}"/>
+    <dataValidation allowBlank="1" showErrorMessage="1" promptTitle="Warning" prompt="Field only used for Epic Issues, so they can be referenced in Story Issues via the Epic Link field.," sqref="O2:O3 M2:M3" xr:uid="{541AD292-0123-4B65-9663-081991FDF0C1}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Field only used for Epic Issues, so they can be referenced in Story Issues via the Epic Link field.," sqref="M1" xr:uid="{64C73155-DEE7-497D-8A98-01E54655ACA8}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="It must be a number (integer) or the Work Item key. This reference is only used during the import process to set the parent." sqref="M1" xr:uid="{8A2BE248-5762-43AD-9C47-C5A92A2E2357}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Field only used for Epic work item, so they can be referenced in Story work items via the Epic Link field. _x000a_DC Only" sqref="O1" xr:uid="{E8F6E005-1F9B-40F3-B24C-E2A3D286C532}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="Creation Marker (Config Sheet)" prompt="Do not manually edit these!" sqref="AE1:AE3" xr:uid="{412C516D-E091-4DDD-9C14-C33AC653C143}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="Feature Pod Label (Config Sheet)" prompt="Do not manually edit these!" sqref="AF1:AF3" xr:uid="{D2234141-379F-4413-AB08-6835BD9FF967}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="AUTOMATIC FIELD" prompt="Do not manually edit these! SKIP types won't be imported into Jira" sqref="AJ1:AJ3" xr:uid="{5A336857-7D14-4900-8734-BED680BE5154}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" sqref="F2:F3" xr:uid="{7708D6E2-1D6B-41D8-A9EE-0E87219BA8EA}">
       <formula1>INDIRECT("CfgFixVersions[FixVersion.Name]")</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="I2:I3" xr:uid="{ED307577-9088-47BA-9824-74F4BBFC13C9}">
+      <formula1>INDIRECT("CfgTeams[Team.Name]")</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2265,13 +2297,13 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xWindow="1573" yWindow="665" count="2">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{5EEBB8D5-878D-4D0E-9267-0919B5A1B925}">
           <x14:formula1>
-            <xm:f>Config!$O$4:$O$10</xm:f>
+            <xm:f>Config!$R$4:$R$10</xm:f>
           </x14:formula1>
           <xm:sqref>A2:A3</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Issue Type" xr:uid="{28BF52BF-C0B0-4D22-B02F-F1408D5A055B}">
           <x14:formula1>
-            <xm:f>Config!$Z$4:$Z$33</xm:f>
+            <xm:f>Config!$AC$4:$AC$33</xm:f>
           </x14:formula1>
           <xm:sqref>B2:B3</xm:sqref>
         </x14:dataValidation>
@@ -2283,114 +2315,123 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2D54512-1380-4F02-BB23-352387C91232}">
-  <dimension ref="A1:AA21"/>
+  <dimension ref="A1:AD21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.7109375" customWidth="1"/>
     <col min="2" max="2" width="49" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="4.28515625" customWidth="1"/>
-    <col min="4" max="5" width="18.7109375" customWidth="1"/>
+    <col min="4" max="5" width="49" customWidth="1"/>
     <col min="6" max="6" width="4.28515625" customWidth="1"/>
-    <col min="7" max="7" width="18.5703125" customWidth="1"/>
-    <col min="8" max="8" width="4.28515625" customWidth="1"/>
-    <col min="9" max="9" width="19.140625" customWidth="1"/>
-    <col min="10" max="10" width="4.28515625" customWidth="1"/>
-    <col min="11" max="11" width="18.5703125" customWidth="1"/>
-    <col min="12" max="12" width="4.28515625" customWidth="1"/>
-    <col min="13" max="13" width="17.5703125" customWidth="1"/>
-    <col min="14" max="14" width="4.28515625" customWidth="1"/>
-    <col min="15" max="15" width="18.7109375" customWidth="1"/>
-    <col min="16" max="16" width="4.28515625" customWidth="1"/>
-    <col min="17" max="18" width="18.7109375" customWidth="1"/>
-    <col min="19" max="19" width="35" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="18.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.28515625" customWidth="1"/>
+    <col min="10" max="10" width="18.5703125" customWidth="1"/>
+    <col min="11" max="11" width="4.28515625" customWidth="1"/>
+    <col min="12" max="12" width="19.140625" customWidth="1"/>
+    <col min="13" max="13" width="4.28515625" customWidth="1"/>
+    <col min="14" max="14" width="18.5703125" customWidth="1"/>
+    <col min="15" max="15" width="4.28515625" customWidth="1"/>
+    <col min="16" max="16" width="17.5703125" customWidth="1"/>
+    <col min="17" max="17" width="4.28515625" customWidth="1"/>
+    <col min="18" max="18" width="18.7109375" customWidth="1"/>
+    <col min="19" max="19" width="4.28515625" customWidth="1"/>
+    <col min="20" max="21" width="18.7109375" customWidth="1"/>
+    <col min="22" max="22" width="35" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="22.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:30" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
         <v>67</v>
       </c>
       <c r="B1" s="11"/>
       <c r="D1" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="E1" s="11"/>
+      <c r="G1" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="E1" s="11"/>
-      <c r="G1" s="6" t="s">
+      <c r="H1" s="11"/>
+      <c r="J1" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="L1" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="N1" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="P1" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="R1" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="Q1" s="11" t="s">
+      <c r="T1" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="R1" s="11"/>
-      <c r="S1" s="11"/>
-      <c r="U1" s="11" t="s">
+      <c r="U1" s="11"/>
+      <c r="V1" s="11"/>
+      <c r="X1" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="V1" s="11"/>
-      <c r="W1" s="11"/>
-      <c r="X1" s="11"/>
-      <c r="Z1" s="6" t="s">
+      <c r="Y1" s="11"/>
+      <c r="Z1" s="11"/>
+      <c r="AA1" s="11"/>
+      <c r="AC1" s="6" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
         <v>73</v>
       </c>
       <c r="B2" s="12"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="12" t="s">
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="E2" s="12"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="10" t="s">
+      <c r="H2" s="12"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10" t="s">
+      <c r="K2" s="10"/>
+      <c r="L2" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="J2" s="10"/>
-      <c r="K2" s="12" t="s">
+      <c r="M2" s="10"/>
+      <c r="N2" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="L2" s="12"/>
-      <c r="M2" s="9" t="s">
+      <c r="O2" s="12"/>
+      <c r="P2" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="N2" s="9"/>
-      <c r="O2" s="10" t="s">
+      <c r="Q2" s="9"/>
+      <c r="R2" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="P2" s="10"/>
-      <c r="Q2" s="12"/>
-      <c r="R2" s="12"/>
-      <c r="S2" s="9"/>
-      <c r="T2" s="7"/>
-      <c r="U2" s="7"/>
-      <c r="V2" s="7"/>
+      <c r="S2" s="10"/>
+      <c r="T2" s="12"/>
+      <c r="U2" s="12"/>
+      <c r="V2" s="9"/>
       <c r="W2" s="7"/>
       <c r="X2" s="7"/>
       <c r="Y2" s="7"/>
-      <c r="Z2" s="9" t="s">
+      <c r="Z2" s="7"/>
+      <c r="AA2" s="7"/>
+      <c r="AB2" s="7"/>
+      <c r="AC2" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="AA2" s="9"/>
+      <c r="AD2" s="9"/>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -2398,52 +2439,58 @@
         <v>57</v>
       </c>
       <c r="D3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E3" t="s">
+        <v>108</v>
+      </c>
+      <c r="G3" t="s">
         <v>58</v>
       </c>
-      <c r="E3" t="s">
+      <c r="H3" t="s">
         <v>59</v>
       </c>
-      <c r="G3" t="s">
+      <c r="J3" t="s">
         <v>63</v>
       </c>
-      <c r="I3" t="s">
+      <c r="L3" t="s">
         <v>62</v>
       </c>
-      <c r="K3" t="s">
+      <c r="N3" t="s">
         <v>61</v>
       </c>
-      <c r="M3" t="s">
+      <c r="P3" t="s">
         <v>66</v>
       </c>
-      <c r="O3" t="s">
+      <c r="R3" t="s">
         <v>60</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="T3" t="s">
         <v>53</v>
       </c>
-      <c r="R3" t="s">
+      <c r="U3" t="s">
         <v>54</v>
       </c>
-      <c r="S3" t="s">
+      <c r="V3" t="s">
         <v>64</v>
       </c>
-      <c r="U3" t="s">
+      <c r="X3" t="s">
         <v>53</v>
       </c>
-      <c r="V3" t="s">
+      <c r="Y3" t="s">
         <v>98</v>
       </c>
-      <c r="W3" t="s">
+      <c r="Z3" t="s">
         <v>99</v>
       </c>
-      <c r="X3" t="s">
+      <c r="AA3" t="s">
         <v>100</v>
       </c>
-      <c r="Z3" s="5" t="s">
+      <c r="AC3" s="5" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>53</v>
       </c>
@@ -2451,226 +2498,233 @@
         <v>94</v>
       </c>
       <c r="D4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E4" t="s">
+        <v>109</v>
+      </c>
+      <c r="G4" t="s">
         <v>45</v>
       </c>
-      <c r="E4">
+      <c r="H4">
         <v>1</v>
       </c>
-      <c r="G4" t="s">
+      <c r="J4" t="s">
         <v>90</v>
       </c>
-      <c r="I4" t="s">
+      <c r="L4" t="s">
         <v>84</v>
       </c>
-      <c r="K4" t="s">
+      <c r="N4" t="s">
         <v>39</v>
       </c>
-      <c r="M4" t="s">
+      <c r="P4" t="s">
         <v>34</v>
       </c>
-      <c r="O4" s="1" t="s">
+      <c r="R4" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="T4" t="s">
         <v>50</v>
       </c>
-      <c r="R4" t="s">
+      <c r="U4" t="s">
         <v>91</v>
       </c>
-      <c r="S4" s="7" t="s">
+      <c r="V4" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="Z4" t="str" cm="1">
-        <f t="array" aca="1" ref="Z4:Z12" ca="1">_xlfn.UNIQUE((_xlfn.VSTACK(INDIRECT("CfgIssueTypes[IssueType.Name]"),INDIRECT("CfgIgnoreList[IgnoreList.Name]"))))</f>
+      <c r="AC4" t="str" cm="1">
+        <f t="array" aca="1" ref="AC4:AC12" ca="1">_xlfn.UNIQUE((_xlfn.VSTACK(INDIRECT("CfgIssueTypes[IssueType.Name]"),INDIRECT("CfgIgnoreList[IgnoreList.Name]"))))</f>
         <v>Story</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="K5" t="s">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="N5" t="s">
         <v>37</v>
       </c>
-      <c r="M5" t="s">
+      <c r="P5" t="s">
         <v>44</v>
       </c>
-      <c r="O5" s="1" t="s">
+      <c r="R5" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="Q5" t="s">
+      <c r="T5" t="s">
         <v>46</v>
       </c>
-      <c r="R5" t="s">
+      <c r="U5" t="s">
         <v>85</v>
       </c>
-      <c r="S5" s="7" t="s">
+      <c r="V5" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="Z5" t="str">
+      <c r="AC5" t="str">
         <f ca="1"/>
         <v>Task</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="K6" t="s">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="N6" t="s">
         <v>40</v>
       </c>
-      <c r="M6" t="s">
+      <c r="P6" t="s">
         <v>33</v>
       </c>
-      <c r="O6" s="1" t="s">
+      <c r="R6" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="Q6" t="s">
+      <c r="T6" t="s">
         <v>86</v>
       </c>
-      <c r="R6" t="s">
+      <c r="U6" t="s">
         <v>102</v>
       </c>
-      <c r="S6" s="7"/>
-      <c r="Z6" t="str">
+      <c r="V6" s="7"/>
+      <c r="AC6" t="str">
         <f ca="1"/>
         <v>Bug</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="K7" t="s">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="N7" t="s">
         <v>41</v>
       </c>
-      <c r="O7" s="1" t="s">
+      <c r="R7" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="Q7" t="s">
+      <c r="T7" t="s">
         <v>87</v>
       </c>
-      <c r="R7" t="s">
+      <c r="U7" t="s">
         <v>104</v>
       </c>
-      <c r="S7" s="7"/>
-      <c r="Z7" t="str">
+      <c r="V7" s="7"/>
+      <c r="AC7" t="str">
         <f ca="1"/>
         <v>Epic</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="K8" t="s">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="N8" t="s">
         <v>93</v>
       </c>
-      <c r="O8" s="1" t="s">
+      <c r="R8" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="Q8" t="s">
+      <c r="T8" t="s">
         <v>103</v>
       </c>
-      <c r="R8">
+      <c r="U8">
         <v>7</v>
       </c>
-      <c r="S8" s="7"/>
-      <c r="Z8" t="str">
+      <c r="V8" s="7"/>
+      <c r="AC8" t="str">
         <f ca="1"/>
         <v>Sub-Task</v>
       </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="K9" t="s">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="N9" t="s">
         <v>101</v>
       </c>
-      <c r="O9" s="1" t="s">
+      <c r="R9" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="Q9" t="s">
+      <c r="T9" t="s">
         <v>88</v>
       </c>
-      <c r="R9" t="s">
+      <c r="U9" t="s">
         <v>89</v>
       </c>
-      <c r="S9" s="7"/>
-      <c r="Z9" t="str">
+      <c r="V9" s="7"/>
+      <c r="AC9" t="str">
         <f ca="1"/>
         <v>Initiative</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="S10" s="7"/>
-      <c r="Z10" t="str">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="V10" s="7"/>
+      <c r="AC10" t="str">
         <f ca="1"/>
         <v>Comment</v>
       </c>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="S11" s="7"/>
-      <c r="Z11" t="str">
+    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="V11" s="7"/>
+      <c r="AC11" t="str">
         <f ca="1"/>
         <v>Skip</v>
       </c>
     </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="Z12" t="str">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="AC12" t="str">
         <f ca="1"/>
         <v>Note</v>
       </c>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
+    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
+    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
+    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
+    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
     </row>
-    <row r="17" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
+    <row r="17" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
     </row>
-    <row r="18" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
+    <row r="18" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
     </row>
-    <row r="19" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
+    <row r="19" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
     </row>
-    <row r="20" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
+    <row r="20" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
     </row>
-    <row r="21" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
+    <row r="21" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="U1:X1"/>
-    <mergeCell ref="Q1:S1"/>
-    <mergeCell ref="D1:E1"/>
+  <mergeCells count="9">
+    <mergeCell ref="X1:AA1"/>
+    <mergeCell ref="T1:V1"/>
+    <mergeCell ref="G1:H1"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="Q2:R2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="T2:U2"/>
+    <mergeCell ref="D1:E1"/>
   </mergeCells>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
-  <tableParts count="9">
+  <tableParts count="10">
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>
@@ -2680,31 +2734,12 @@
     <tablePart r:id="rId8"/>
     <tablePart r:id="rId9"/>
     <tablePart r:id="rId10"/>
+    <tablePart r:id="rId11"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FB038601AF41D04A88A4BD446922F1A8" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e8d32171d27ae41230d53456f24efae5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c471fd26-9765-4fbe-b6fd-c17c1e55c974" xmlns:ns3="9df69692-83aa-4c55-88c1-62abad05f4fe" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f2fb84de5621acf32f385a2ba90fb29" ns2:_="" ns3:_="">
     <xsd:import namespace="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
@@ -2933,10 +2968,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2C983B91-58B3-4C2C-AC55-FFEC9F0DB5F6}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
+    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2953,20 +3019,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2C983B91-58B3-4C2C-AC55-FFEC9F0DB5F6}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
-    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
JT-143 Fix: update ImportTemplate.xlsx with the correct default issuetype levels (1 to 4).
</commit_message>
<xml_diff>
--- a/resources/templates/ImportTemplate.xlsx
+++ b/resources/templates/ImportTemplate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workdir\DeerHide\sources\jira-toolkit\resources\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4BC4158-D472-4903-A82C-8B483D399CF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5D59A5B-E3CC-4BE2-8CC3-FDE61B5D10DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1485" yWindow="6135" windowWidth="29685" windowHeight="23445" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
+    <workbookView xWindow="735" yWindow="735" windowWidth="29685" windowHeight="23445" activeTab="4" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="7" r:id="rId10"/>
+    <pivotCache cacheId="9" r:id="rId10"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -83,7 +83,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Issue type (Epic, Story, Task…). Skip types like comment/note are ignored.</t>
         </r>
@@ -819,7 +819,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -982,12 +982,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="9"/>
@@ -1357,7 +1351,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1407,7 +1401,6 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="16" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1598,35 +1591,35 @@
       </fill>
     </dxf>
     <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <alignment vertical="top"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -2006,7 +1999,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9326BD75-A09D-4578-BB55-882D1F75C66E}" name="PT_Issues" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9326BD75-A09D-4578-BB55-882D1F75C66E}" name="PT_Issues" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A5:B12" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="36">
     <pivotField showAll="0"/>
@@ -2114,7 +2107,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A931C4D6-0F40-4FC0-8FE0-7829E37288EB}" name="PT_Assignees" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A931C4D6-0F40-4FC0-8FE0-7829E37288EB}" name="PT_Assignees" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="D5:E10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="36">
     <pivotField showAll="0"/>
@@ -2297,19 +2290,19 @@
     <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="27">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], 'Config - Mappings'!$G$4:$H$8, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="16">
+    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="26">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgMisc[Name], CfgMisc[Value],"",1))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="17">
+    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="25">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Work Group", CfgMisc[Name], CfgMisc[Value],"",1))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="26">
+    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="24">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], 'Config - Mappings'!$A$4:$B$26, 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="25">
+    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="23">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("jira.project.key", CfgBasic[Name], CfgBasic[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="24">
+    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="22">
       <calculatedColumnFormula array="1">IF(
   JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
   "",
@@ -2325,7 +2318,7 @@
   )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="23">
+    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="21">
       <calculatedColumnFormula array="1">IFERROR(
     _xlfn.IFS(
         JiraDataset[[#This Row],[IssueType]] = cfg_type_comment,"SKIP",
@@ -2335,7 +2328,7 @@
     cfg_type_workitem
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="22"/>
+    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2345,7 +2338,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}" name="CfgPriorities" displayName="CfgPriorities" ref="L22:L28" totalsRowShown="0">
   <autoFilter ref="L22:L28" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2381,7 +2374,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{724752C0-2EB0-4307-9766-E95D142383BC}" name="Name"/>
     <tableColumn id="2" xr3:uid="{1B4D7FE1-60C9-4319-8B9F-E66C19764AEE}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{F0634D25-384E-480B-B675-9F8463C0D844}" name="Note" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{F0634D25-384E-480B-B675-9F8463C0D844}" name="Note" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2437,7 +2430,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{D4E1611F-A2CF-465D-A219-1759EA66687D}" name="Name"/>
     <tableColumn id="2" xr3:uid="{174D0D86-B1AA-4BF7-AC91-FCACFC898851}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Note" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Note" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3340,13 +3333,13 @@
       <c r="A6" s="14" t="s">
         <v>149</v>
       </c>
-      <c r="B6" s="21">
+      <c r="B6">
         <v>1</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="E6" s="21">
+      <c r="E6">
         <v>1</v>
       </c>
     </row>
@@ -3354,13 +3347,13 @@
       <c r="A7" s="15" t="s">
         <v>149</v>
       </c>
-      <c r="B7" s="21">
+      <c r="B7">
         <v>1</v>
       </c>
       <c r="D7" s="15" t="s">
         <v>155</v>
       </c>
-      <c r="E7" s="21">
+      <c r="E7">
         <v>1</v>
       </c>
     </row>
@@ -3368,13 +3361,13 @@
       <c r="A8" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="B8" s="21">
+      <c r="B8">
         <v>1</v>
       </c>
       <c r="D8" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="E8" s="21">
+      <c r="E8">
         <v>1</v>
       </c>
     </row>
@@ -3382,13 +3375,13 @@
       <c r="A9" s="14" t="s">
         <v>165</v>
       </c>
-      <c r="B9" s="21">
+      <c r="B9">
         <v>1</v>
       </c>
       <c r="D9" s="15" t="s">
         <v>149</v>
       </c>
-      <c r="E9" s="21">
+      <c r="E9">
         <v>1</v>
       </c>
     </row>
@@ -3396,13 +3389,13 @@
       <c r="A10" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="B10" s="21">
+      <c r="B10">
         <v>1</v>
       </c>
       <c r="D10" s="14" t="s">
         <v>148</v>
       </c>
-      <c r="E10" s="21">
+      <c r="E10">
         <v>2</v>
       </c>
     </row>
@@ -3410,7 +3403,7 @@
       <c r="A11" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="B11" s="21">
+      <c r="B11">
         <v>1</v>
       </c>
     </row>
@@ -3418,7 +3411,7 @@
       <c r="A12" s="14" t="s">
         <v>148</v>
       </c>
-      <c r="B12" s="21">
+      <c r="B12">
         <v>2</v>
       </c>
     </row>
@@ -4042,7 +4035,7 @@
         <v>38</v>
       </c>
       <c r="M4">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -4062,7 +4055,7 @@
         <v>36</v>
       </c>
       <c r="M5">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
@@ -4084,7 +4077,7 @@
         <v>40</v>
       </c>
       <c r="M6">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -4106,7 +4099,7 @@
         <v>41</v>
       </c>
       <c r="M7">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
@@ -4128,7 +4121,7 @@
         <v>89</v>
       </c>
       <c r="M8">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
@@ -4674,6 +4667,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FB038601AF41D04A88A4BD446922F1A8" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e8d32171d27ae41230d53456f24efae5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c471fd26-9765-4fbe-b6fd-c17c1e55c974" xmlns:ns3="9df69692-83aa-4c55-88c1-62abad05f4fe" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f2fb84de5621acf32f385a2ba90fb29" ns2:_="" ns3:_="">
     <xsd:import namespace="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
@@ -4902,15 +4904,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -4923,6 +4916,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2C983B91-58B3-4C2C-AC55-FFEC9F0DB5F6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4941,14 +4942,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FFE630F-6530-4863-AB67-8477539A0000}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
JT-143 chore: update ImportTemplate.xlsx for recent data import changes
Fix references that pointed to individual cells instead of indirect tables.
Reduce the number of label fields from 10 to 5, since multiple labels are now supported in a single cell (`label; label; ...`).
Reorder columns to make the template more logical to fill out and review.
</commit_message>
<xml_diff>
--- a/resources/templates/ImportTemplate.xlsx
+++ b/resources/templates/ImportTemplate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workdir\DeerHide\sources\jira-toolkit\resources\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5D59A5B-E3CC-4BE2-8CC3-FDE61B5D10DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12369D8C-D85F-47D4-A1D7-BC151129C134}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="735" yWindow="735" windowWidth="29685" windowHeight="23445" activeTab="4" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
+    <workbookView xWindow="1845" yWindow="4695" windowWidth="33615" windowHeight="23445" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="9" r:id="rId10"/>
+    <pivotCache cacheId="0" r:id="rId10"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -115,7 +115,59 @@
         </r>
       </text>
     </comment>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{9C29F0D9-EEC2-4CD5-94B3-E79BFBEEBA7A}">
+    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{D37165B4-6A0B-4DE1-BBC9-E2B87095C67A}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Assignee name from CfgAssignees (mapped to account ID).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{BF9D9590-454C-4556-A96A-8432D26EB0AA}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Component name from CfgComponents. One per cell.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{098743DC-80FD-4D99-8C10-F8768C499BB1}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Effort estimate. Blank if unknown. Format 1w 2d 4h (week=5days, day=8h)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0" xr:uid="{E0BF772F-400D-4779-B463-DF3B16DC24EF}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Sprint name from CfgSprints. Blank if unplanned.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0" xr:uid="{9C29F0D9-EEC2-4CD5-94B3-E79BFBEEBA7A}">
       <text>
         <r>
           <rPr>
@@ -128,7 +180,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{D37165B4-6A0B-4DE1-BBC9-E2B87095C67A}">
+    <comment ref="L1" authorId="0" shapeId="0" xr:uid="{E6A239CC-FBE8-42B6-BE3E-9D37323CB14A}">
       <text>
         <r>
           <rPr>
@@ -137,63 +189,12 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Assignee name from CfgAssignees (mapped to account ID).</t>
+          <t>Unique local ID in this file (not a Jira key). Used for links.
+Empty row can be generated using -af/--auto-fix</t>
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{BF9D9590-454C-4556-A96A-8432D26EB0AA}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Component name from CfgComponents. One per cell.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{E0BF772F-400D-4779-B463-DF3B16DC24EF}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Sprint name from CfgSprints. Blank if unplanned.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0" shapeId="0" xr:uid="{098743DC-80FD-4D99-8C10-F8768C499BB1}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Effort estimate. Blank if unknown. Format 1w 2d 4h (week=5days, day=8h)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0" shapeId="0" xr:uid="{E6A239CC-FBE8-42B6-BE3E-9D37323CB14A}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Unique local ID in this file (not a Jira key). Used for links.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="L1" authorId="0" shapeId="0" xr:uid="{B1D0971D-6639-458E-AEB8-E00BC927C14D}">
+    <comment ref="M1" authorId="0" shapeId="0" xr:uid="{B1D0971D-6639-458E-AEB8-E00BC927C14D}">
       <text>
         <r>
           <rPr>
@@ -206,7 +207,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R1" authorId="0" shapeId="0" xr:uid="{FD454FB1-970A-43A3-8724-BF23CA54530B}">
+    <comment ref="P1" authorId="0" shapeId="0" xr:uid="{FD454FB1-970A-43A3-8724-BF23CA54530B}">
       <text>
         <r>
           <rPr>
@@ -246,7 +247,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="200">
   <si>
     <t>IssueType</t>
   </si>
@@ -287,15 +288,6 @@
     <t>Epic Name</t>
   </si>
   <si>
-    <t>Child-Issue</t>
-  </si>
-  <si>
-    <t>Child-Issue1</t>
-  </si>
-  <si>
-    <t>Child-Issue2</t>
-  </si>
-  <si>
     <t>Labels</t>
   </si>
   <si>
@@ -314,21 +306,6 @@
     <t>Labels5</t>
   </si>
   <si>
-    <t>Labels6</t>
-  </si>
-  <si>
-    <t>Labels7</t>
-  </si>
-  <si>
-    <t>Labels8</t>
-  </si>
-  <si>
-    <t>Labels9</t>
-  </si>
-  <si>
-    <t>Labels10</t>
-  </si>
-  <si>
     <t>Sprint</t>
   </si>
   <si>
@@ -473,9 +450,6 @@
     <t>List of Components</t>
   </si>
   <si>
-    <t>Accepted User Types</t>
-  </si>
-  <si>
     <t>Issue Types that won't be imported</t>
   </si>
   <si>
@@ -813,6 +787,66 @@
   </si>
   <si>
     <t>This sheet is ignored by the importer, it can contain anything</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>QA Team</t>
+  </si>
+  <si>
+    <t>PM Team</t>
+  </si>
+  <si>
+    <t>Design Team</t>
+  </si>
+  <si>
+    <t>Dev Team</t>
+  </si>
+  <si>
+    <t>Accepted IssueType and Levels</t>
+  </si>
+  <si>
+    <t>CF Number01</t>
+  </si>
+  <si>
+    <t>customfield_10125</t>
+  </si>
+  <si>
+    <t>number</t>
+  </si>
+  <si>
+    <t>CF Plain Text</t>
+  </si>
+  <si>
+    <t>customfield_10124</t>
+  </si>
+  <si>
+    <t>text</t>
+  </si>
+  <si>
+    <t>CF Date</t>
+  </si>
+  <si>
+    <t>customfield_10123</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>CF List</t>
+  </si>
+  <si>
+    <t>customfield_10126</t>
+  </si>
+  <si>
+    <t>any</t>
+  </si>
+  <si>
+    <t>The names need to match a column in the dataset (first sheet)</t>
+  </si>
+  <si>
+    <t>This is the description of the work item</t>
   </si>
 </sst>
 </file>
@@ -1351,7 +1385,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1401,6 +1435,9 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="16" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" shrinkToFit="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1447,7 +1484,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="58">
+  <dxfs count="52">
     <dxf>
       <fill>
         <patternFill patternType="darkUp"/>
@@ -1591,121 +1628,101 @@
       </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
       <font>
         <b val="0"/>
       </font>
       <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
       <alignment vertical="top"/>
     </dxf>
     <dxf>
@@ -1743,6 +1760,9 @@
     </dxf>
     <dxf>
       <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1774,7 +1794,7 @@
 <file path=xl/namedSheetViews/namedSheetView1.xml><?xml version="1.0" encoding="utf-8"?>
 <namedSheetViews xmlns="http://schemas.microsoft.com/office/spreadsheetml/2019/namedsheetviews" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <namedSheetView name="View1" id="{77233F75-225A-4D7F-8A86-543E0A8C6E58}">
-    <nsvFilter filterId="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" ref="A1:AJ3" tableId="1"/>
+    <nsvFilter filterId="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" ref="A1:AD3" tableId="1"/>
   </namedSheetView>
 </namedSheetViews>
 </file>
@@ -1999,7 +2019,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9326BD75-A09D-4578-BB55-882D1F75C66E}" name="PT_Issues" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9326BD75-A09D-4578-BB55-882D1F75C66E}" name="PT_Issues" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A5:B12" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="36">
     <pivotField showAll="0"/>
@@ -2107,7 +2127,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A931C4D6-0F40-4FC0-8FE0-7829E37288EB}" name="PT_Assignees" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A931C4D6-0F40-4FC0-8FE0-7829E37288EB}" name="PT_Assignees" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="D5:E10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="36">
     <pivotField showAll="0"/>
@@ -2252,57 +2272,53 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" name="JiraDataset" displayName="JiraDataset" ref="A1:AJ3" totalsRowShown="0" headerRowDxfId="57" dataDxfId="56">
-  <autoFilter ref="A1:AJ3" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}"/>
-  <tableColumns count="36">
-    <tableColumn id="3" xr3:uid="{AF2EC907-349C-4651-852D-6E39C61E17FF}" name="Priority" dataDxfId="55"/>
-    <tableColumn id="2" xr3:uid="{E90C51F2-4386-421F-A3E4-E2CA9D43D396}" name="IssueType" dataDxfId="54"/>
-    <tableColumn id="1" xr3:uid="{BBAD373B-BA13-47E4-9F74-565F4D9E9680}" name="Summary" dataDxfId="53"/>
-    <tableColumn id="4" xr3:uid="{026E5B97-FAFC-4E46-860E-0B0C976B1148}" name="Issue Key" dataDxfId="52"/>
-    <tableColumn id="5" xr3:uid="{A2C262E8-D544-4669-99F1-151EDE081654}" name="Description" dataDxfId="51"/>
-    <tableColumn id="7" xr3:uid="{0FAD1ACC-432E-462C-8B89-71540710BCB5}" name="FixVersion" dataDxfId="50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" name="JiraDataset" displayName="JiraDataset" ref="A1:AD3" totalsRowShown="0" headerRowDxfId="50" dataDxfId="49">
+  <autoFilter ref="A1:AD3" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}"/>
+  <tableColumns count="30">
+    <tableColumn id="3" xr3:uid="{AF2EC907-349C-4651-852D-6E39C61E17FF}" name="Priority" dataDxfId="48"/>
+    <tableColumn id="2" xr3:uid="{E90C51F2-4386-421F-A3E4-E2CA9D43D396}" name="IssueType" dataDxfId="47"/>
+    <tableColumn id="1" xr3:uid="{BBAD373B-BA13-47E4-9F74-565F4D9E9680}" name="Summary" dataDxfId="46"/>
+    <tableColumn id="4" xr3:uid="{026E5B97-FAFC-4E46-860E-0B0C976B1148}" name="Issue Key" dataDxfId="45"/>
+    <tableColumn id="5" xr3:uid="{A2C262E8-D544-4669-99F1-151EDE081654}" name="Description" dataDxfId="44"/>
+    <tableColumn id="28" xr3:uid="{07F3030C-7187-4B16-BBDB-798304851975}" name="Assignee.Name" dataDxfId="43"/>
+    <tableColumn id="8" xr3:uid="{8C7FB8DB-A85B-4189-93D8-0F0D4EEEF81B}" name="Component" dataDxfId="42"/>
+    <tableColumn id="31" xr3:uid="{BB70BDE8-70CB-404D-896E-075FB6ED93B1}" name="Team.Name" dataDxfId="20"/>
+    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="17"/>
+    <tableColumn id="9" xr3:uid="{DC5101A8-1204-44D2-BC2C-FEE1A4EFE7C1}" name="Sprint Name" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{0FAD1ACC-432E-462C-8B89-71540710BCB5}" name="FixVersion" dataDxfId="16">
       <calculatedColumnFormula>'Config - Mappings'!$J$4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="28" xr3:uid="{07F3030C-7187-4B16-BBDB-798304851975}" name="Assignee.Name" dataDxfId="49"/>
-    <tableColumn id="8" xr3:uid="{8C7FB8DB-A85B-4189-93D8-0F0D4EEEF81B}" name="Component" dataDxfId="48"/>
-    <tableColumn id="9" xr3:uid="{DC5101A8-1204-44D2-BC2C-FEE1A4EFE7C1}" name="Sprint Name" dataDxfId="47"/>
-    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="46"/>
-    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="45"/>
-    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="44"/>
-    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="43"/>
-    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="42">
+    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="41"/>
+    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="40"/>
+    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="39"/>
+    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="38">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[IssueType]]="Epic",JiraDataset[[#This Row],[Summary]],"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="27" xr3:uid="{911C8FDC-5528-43FC-BDF4-D4761F03C0E5}" name="Child-Issue" dataDxfId="41"/>
-    <tableColumn id="41" xr3:uid="{AB248E07-9BFA-42CC-BC41-B4234F677BFB}" name="Child-Issue1" dataDxfId="40"/>
-    <tableColumn id="29" xr3:uid="{89D12135-F3E3-4253-844F-1B9A54169953}" name="Child-Issue2" dataDxfId="39"/>
-    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="38"/>
-    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="37"/>
-    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="36"/>
-    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="35"/>
-    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="34"/>
-    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="33"/>
-    <tableColumn id="18" xr3:uid="{16B98070-7F8A-4FC7-AD99-EA81D0BD26AB}" name="Labels6" dataDxfId="32"/>
-    <tableColumn id="19" xr3:uid="{016EAEF4-8EA9-408B-9F1A-ECFB17E81C77}" name="Labels7" dataDxfId="31"/>
-    <tableColumn id="26" xr3:uid="{8263F9EC-BF0A-46F7-BA83-6083A4262B91}" name="Labels8" dataDxfId="30"/>
-    <tableColumn id="20" xr3:uid="{389B11C5-1B22-48C0-BCA2-72F050425FA1}" name="Labels9" dataDxfId="29"/>
-    <tableColumn id="25" xr3:uid="{AE95F8A2-F7F0-4985-9AE6-4201B9792775}" name="Labels10" dataDxfId="28"/>
-    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="27">
-      <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], 'Config - Mappings'!$G$4:$H$8, 2, FALSE), ""))</calculatedColumnFormula>
+    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="37"/>
+    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="36"/>
+    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="35"/>
+    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="34"/>
+    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="33"/>
+    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="32"/>
+    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="22">
+      <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], CfgSprints[], 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="26">
+    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="31">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgMisc[Name], CfgMisc[Value],"",1))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="25">
+    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="30">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Work Group", CfgMisc[Name], CfgMisc[Value],"",1))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="24">
-      <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], 'Config - Mappings'!$A$4:$B$26, 2, FALSE), ""))</calculatedColumnFormula>
+    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="21">
+      <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], CfgAssignees[], 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="23">
+    <tableColumn id="32" xr3:uid="{B9236297-6F08-4471-BC00-A337F6321979}" name="Team" dataDxfId="19">
+      <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Team.Name]], CfgTeams[], 2, FALSE), ""))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="29">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("jira.project.key", CfgBasic[Name], CfgBasic[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="22">
+    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="28">
       <calculatedColumnFormula array="1">IF(
   JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
   "",
@@ -2318,7 +2334,7 @@
   )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="21">
+    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="27">
       <calculatedColumnFormula array="1">IFERROR(
     _xlfn.IFS(
         JiraDataset[[#This Row],[IssueType]] = cfg_type_comment,"SKIP",
@@ -2328,7 +2344,7 @@
     cfg_type_workitem
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="20"/>
+    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2338,15 +2354,15 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}" name="CfgPriorities" displayName="CfgPriorities" ref="L22:L28" totalsRowShown="0">
   <autoFilter ref="L22:L28" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="17"/>
+    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="51"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{DE352608-207B-4EFC-9BD3-2BD6976D373F}" name="CfgTeams" displayName="CfgTeams" ref="D3:E9" totalsRowShown="0">
-  <autoFilter ref="D3:E9" xr:uid="{DE352608-207B-4EFC-9BD3-2BD6976D373F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{DE352608-207B-4EFC-9BD3-2BD6976D373F}" name="CfgTeams" displayName="CfgTeams" ref="D3:E8" totalsRowShown="0">
+  <autoFilter ref="D3:E8" xr:uid="{DE352608-207B-4EFC-9BD3-2BD6976D373F}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{59E7B951-2640-4BEF-926D-11574E54F447}" name="Team.Name"/>
     <tableColumn id="2" xr3:uid="{1C40E406-7D3C-45A3-AAA3-B5BBB7E9C3AA}" name="Team.ID"/>
@@ -2356,8 +2372,8 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{71F57F46-4709-4A78-8D88-CD75C743FE14}" name="CfgCustomFields" displayName="CfgCustomFields" ref="E3:H4" insertRow="1" totalsRowShown="0">
-  <autoFilter ref="E3:H4" xr:uid="{71F57F46-4709-4A78-8D88-CD75C743FE14}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{71F57F46-4709-4A78-8D88-CD75C743FE14}" name="CfgCustomFields" displayName="CfgCustomFields" ref="E3:H7" totalsRowShown="0">
+  <autoFilter ref="E3:H7" xr:uid="{71F57F46-4709-4A78-8D88-CD75C743FE14}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{4E62A8D1-901A-4C3B-920B-726A6F2C172C}" name="Name"/>
     <tableColumn id="2" xr3:uid="{F3AA6FE2-2D0B-4D90-9B62-6DA6E107F572}" name="Id"/>
@@ -2374,7 +2390,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{724752C0-2EB0-4307-9766-E95D142383BC}" name="Name"/>
     <tableColumn id="2" xr3:uid="{1B4D7FE1-60C9-4319-8B9F-E66C19764AEE}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{F0634D25-384E-480B-B675-9F8463C0D844}" name="Note" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{F0634D25-384E-480B-B675-9F8463C0D844}" name="Note" dataDxfId="23"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2430,7 +2446,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{D4E1611F-A2CF-465D-A219-1759EA66687D}" name="Name"/>
     <tableColumn id="2" xr3:uid="{174D0D86-B1AA-4BF7-AC91-FCACFC898851}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Note" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Note" dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2442,7 +2458,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{19232286-858A-4316-B524-2259E904D535}" name="Name"/>
     <tableColumn id="2" xr3:uid="{E6137B31-22A5-4579-8A81-0FBB4015A668}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{03DA91C8-48E1-4BFC-B993-8C1071BAA534}" name="Note" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{03DA91C8-48E1-4BFC-B993-8C1071BAA534}" name="Note" dataDxfId="24"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2821,39 +2837,38 @@
   <sheetPr>
     <tabColor theme="4"/>
   </sheetPr>
-  <dimension ref="A1:AL3"/>
+  <dimension ref="A1:AP3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="31.7109375" customWidth="1"/>
     <col min="4" max="4" width="26.42578125" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="39.42578125" customWidth="1"/>
-    <col min="6" max="6" width="14.28515625" customWidth="1"/>
-    <col min="7" max="7" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.5703125" customWidth="1"/>
-    <col min="9" max="9" width="16.42578125" customWidth="1"/>
-    <col min="10" max="11" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="20" customWidth="1"/>
+    <col min="9" max="9" width="22.5703125" customWidth="1"/>
+    <col min="10" max="10" width="16.42578125" customWidth="1"/>
+    <col min="11" max="11" width="14.42578125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="14.28515625" customWidth="1"/>
-    <col min="13" max="13" width="14.42578125" customWidth="1"/>
-    <col min="14" max="14" width="14.28515625" customWidth="1"/>
-    <col min="15" max="15" width="0" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="22.28515625" hidden="1" customWidth="1"/>
-    <col min="17" max="17" width="12.85546875" hidden="1" customWidth="1"/>
-    <col min="18" max="24" width="14.28515625" customWidth="1"/>
-    <col min="25" max="28" width="14.28515625" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="29" max="30" width="10" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="31" max="31" width="10" customWidth="1" collapsed="1"/>
-    <col min="32" max="32" width="28.140625" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="33" max="33" width="15.85546875" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="34" max="34" width="14" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="35" max="35" width="12.5703125" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="36" max="37" width="13.7109375" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="38" max="38" width="36.5703125" bestFit="1" customWidth="1" collapsed="1"/>
-    <col min="40" max="40" width="18.7109375" customWidth="1"/>
-    <col min="41" max="41" width="87.28515625" customWidth="1"/>
+    <col min="13" max="13" width="13.140625" customWidth="1"/>
+    <col min="14" max="14" width="13.140625" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="15" max="15" width="14.42578125" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="16" max="16" width="14.28515625" customWidth="1" collapsed="1"/>
+    <col min="17" max="21" width="14.28515625" customWidth="1"/>
+    <col min="22" max="22" width="14.28515625" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="23" max="24" width="13.140625" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="25" max="26" width="28.140625" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="27" max="27" width="13.42578125" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="28" max="29" width="28.140625" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="30" max="30" width="21.140625" customWidth="1" collapsed="1"/>
+    <col min="31" max="31" width="14" customWidth="1"/>
+    <col min="32" max="32" width="12.5703125" customWidth="1"/>
+    <col min="33" max="34" width="13.7109375" customWidth="1"/>
+    <col min="35" max="35" width="36.5703125" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="18.7109375" customWidth="1"/>
+    <col min="38" max="38" width="87.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>1</v>
       </c>
@@ -2870,110 +2885,92 @@
         <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
-        <v>80</v>
-      </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" t="s">
+        <v>71</v>
+      </c>
+      <c r="N1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="U1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="V1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="W1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="X1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="X1" s="3" t="s">
+      <c r="Y1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="Y1" s="3" t="s">
+      <c r="Z1" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="AA1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="AB1" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="AA1" s="3" t="s">
+      <c r="AC1" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="AD1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="AB1" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="AC1" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="AD1" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="AE1" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="AF1" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="AG1" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="AH1" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="AI1" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="AJ1" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
@@ -2983,46 +2980,43 @@
       <c r="K2" s="3"/>
       <c r="L2" s="3"/>
       <c r="M2" s="3"/>
-      <c r="N2" s="3" t="str">
+      <c r="N2" s="3"/>
+      <c r="O2" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[IssueType]]="Epic",JiraDataset[[#This Row],[Summary]],"")</f>
         <v/>
       </c>
-      <c r="O2" s="3"/>
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
       <c r="R2" s="3"/>
       <c r="S2" s="3"/>
       <c r="T2" s="3"/>
       <c r="U2" s="3"/>
-      <c r="V2" s="3"/>
-      <c r="W2" s="3"/>
-      <c r="X2" s="3"/>
-      <c r="Y2" s="3"/>
-      <c r="Z2" s="3"/>
-      <c r="AA2" s="3"/>
-      <c r="AB2" s="3"/>
-      <c r="AC2" s="3" t="str">
-        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], 'Config - Mappings'!$G$4:$H$8, 2, FALSE), ""))</f>
+      <c r="V2" s="3" t="str">
+        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], CfgSprints[], 2, FALSE), ""))</f>
         <v/>
       </c>
-      <c r="AD2" s="3" t="str">
+      <c r="W2" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgMisc[Name], CfgMisc[Value],"",1))</f>
         <v/>
       </c>
-      <c r="AE2" s="3" t="str">
+      <c r="X2" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Work Group", CfgMisc[Name], CfgMisc[Value],"",1))</f>
         <v/>
       </c>
-      <c r="AF2" s="3" t="str">
-        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], 'Config - Mappings'!$A$4:$B$26, 2, FALSE), ""))</f>
+      <c r="Y2" s="3" t="str">
+        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], CfgAssignees[], 2, FALSE), ""))</f>
         <v/>
       </c>
-      <c r="AG2" s="3" t="str">
+      <c r="Z2" s="3" t="str">
+        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Team.Name]], CfgTeams[], 2, FALSE), ""))</f>
+        <v/>
+      </c>
+      <c r="AA2" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("jira.project.key", CfgBasic[Name], CfgBasic[Value]))</f>
         <v/>
       </c>
-      <c r="AH2" s="3" t="str" cm="1">
-        <f t="array" ref="AH2">IF(
+      <c r="AB2" s="3" t="str" cm="1">
+        <f t="array" ref="AB2">IF(
   JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
   "",
   _xlfn.LET(
@@ -3038,8 +3032,8 @@
 )</f>
         <v/>
       </c>
-      <c r="AI2" s="3" t="str" cm="1">
-        <f t="array" ref="AI2">IFERROR(
+      <c r="AC2" s="3" t="str" cm="1">
+        <f t="array" ref="AC2">IFERROR(
     _xlfn.IFS(
         JiraDataset[[#This Row],[IssueType]] = cfg_type_comment,"SKIP",
         JiraDataset[[#This Row],[IssueType]] = cfg_type_skip,"SKIP",
@@ -3049,85 +3043,86 @@
 )</f>
         <v>SKIP</v>
       </c>
-      <c r="AJ2" s="3"/>
-    </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AD2" s="3"/>
+    </row>
+    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3" t="str">
+      <c r="E3" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="K3" s="3" t="str">
         <f>'Config - Mappings'!$J$4</f>
         <v>JITTP Version 1</v>
       </c>
-      <c r="G3" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="K3" s="3"/>
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>
-      <c r="N3" s="3" t="str">
+      <c r="N3" s="3"/>
+      <c r="O3" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[IssueType]]="Epic",JiraDataset[[#This Row],[Summary]],"")</f>
         <v>First Work Item</v>
       </c>
-      <c r="O3" s="3"/>
-      <c r="P3" s="3"/>
-      <c r="Q3" s="3"/>
+      <c r="P3" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="Q3" s="3" t="s">
+        <v>161</v>
+      </c>
       <c r="R3" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="S3" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="T3" s="3" t="s">
-        <v>171</v>
-      </c>
+        <v>162</v>
+      </c>
+      <c r="S3" s="3"/>
+      <c r="T3" s="3"/>
       <c r="U3" s="3"/>
-      <c r="V3" s="3"/>
-      <c r="W3" s="3"/>
-      <c r="X3" s="3"/>
-      <c r="Y3" s="3"/>
-      <c r="Z3" s="3"/>
-      <c r="AA3" s="3"/>
-      <c r="AB3" s="3"/>
-      <c r="AC3" s="3">
-        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], 'Config - Mappings'!$G$4:$H$8, 2, FALSE), ""))</f>
+      <c r="V3" s="3">
+        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], CfgSprints[], 2, FALSE), ""))</f>
         <v>97</v>
       </c>
-      <c r="AD3" s="3" t="str">
+      <c r="W3" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgMisc[Name], CfgMisc[Value],"",1))</f>
         <v>imported</v>
       </c>
-      <c r="AE3" s="3" t="str">
+      <c r="X3" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Work Group", CfgMisc[Name], CfgMisc[Value],"",1))</f>
         <v>pod_test</v>
       </c>
-      <c r="AF3" s="3" t="str">
-        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], 'Config - Mappings'!$A$4:$B$26, 2, FALSE), ""))</f>
+      <c r="Y3" s="3" t="str">
+        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], CfgAssignees[], 2, FALSE), ""))</f>
         <v>712020:09876543212345678901</v>
       </c>
-      <c r="AG3" s="3" t="str">
+      <c r="Z3" s="3" t="str">
+        <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Team.Name]], CfgTeams[], 2, FALSE), ""))</f>
+        <v>712020:09876543212345678902</v>
+      </c>
+      <c r="AA3" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("jira.project.key", CfgBasic[Name], CfgBasic[Value]))</f>
         <v>JITTP2</v>
       </c>
-      <c r="AH3" s="3" cm="1">
-        <f t="array" ref="AH3">IF(
+      <c r="AB3" s="3" cm="1">
+        <f t="array" ref="AB3">IF(
   JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
   "",
   _xlfn.LET(
@@ -3143,8 +3138,8 @@
 )</f>
         <v>12744000</v>
       </c>
-      <c r="AI3" s="3" t="str" cm="1">
-        <f t="array" ref="AI3">IFERROR(
+      <c r="AC3" s="3" t="str" cm="1">
+        <f t="array" ref="AC3">IFERROR(
     _xlfn.IFS(
         JiraDataset[[#This Row],[IssueType]] = cfg_type_comment,"SKIP",
         JiraDataset[[#This Row],[IssueType]] = cfg_type_skip,"SKIP",
@@ -3154,12 +3149,12 @@
 )</f>
         <v>WorkItem</v>
       </c>
-      <c r="AJ3" s="3"/>
+      <c r="AD3" s="3"/>
     </row>
   </sheetData>
   <protectedRanges>
-    <protectedRange sqref="C1:AB2 A1:A1048576 P3:AD1048576 D3:N1048576" name="User Input"/>
-    <protectedRange algorithmName="SHA-512" hashValue="tpheD+JLADkhiyalt6vInlMwkILPZx4PVQN/k2vmwjOBdYUuHaXCrwtObHeFz5dJh9f853O84pZ1Rn9Ujz33+A==" saltValue="9ir5NB4CJc/69S/Eh84/mA==" spinCount="100000" sqref="AC1:AI2 AE3:AK1048576" name="Computed values"/>
+    <protectedRange sqref="A1:A1048576 L4:L1048576 C1:E2 D3:E1048576 F1:J3 G4:J1048576 K1:U2 Q4:Z1048576 K3:W3 N4:O1048576" name="User Input"/>
+    <protectedRange algorithmName="SHA-512" hashValue="tpheD+JLADkhiyalt6vInlMwkILPZx4PVQN/k2vmwjOBdYUuHaXCrwtObHeFz5dJh9f853O84pZ1Rn9Ujz33+A==" saltValue="9ir5NB4CJc/69S/Eh84/mA==" spinCount="100000" sqref="V1:AC2 X3:AE3 AA4:AH1048576" name="Computed values"/>
   </protectedRanges>
   <phoneticPr fontId="18" type="noConversion"/>
   <conditionalFormatting sqref="A2:A3 C2:C3">
@@ -3181,7 +3176,7 @@
       <formula>LEN(TRIM(A2))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:AJ3">
+  <conditionalFormatting sqref="A2:AD3">
     <cfRule type="expression" dxfId="10" priority="409" stopIfTrue="1">
       <formula>$B2=cfg_type_comment</formula>
     </cfRule>
@@ -3206,7 +3201,7 @@
       <formula>LEN(TRIM(B2))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2:AJ3">
+  <conditionalFormatting sqref="B2:AD3">
     <cfRule type="expression" dxfId="3" priority="1">
       <formula>$B2="Epic"</formula>
     </cfRule>
@@ -3219,61 +3214,59 @@
       <formula>LEN(TRIM(C2))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:L3">
+  <conditionalFormatting sqref="L2:M3">
     <cfRule type="containsBlanks" dxfId="0" priority="412">
-      <formula>LEN(TRIM(K2))=0</formula>
+      <formula>LEN(TRIM(L2))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations xWindow="1573" yWindow="665" count="23">
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" prompt="It must be a number (integer). This reference is only used during the import process." sqref="K2:L2" xr:uid="{005E18F2-4447-4781-8F18-5A58920A4F75}">
+  <dataValidations xWindow="1573" yWindow="665" count="22">
+    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" prompt="It must be a number (integer). This reference is only used during the import process." sqref="L2:M2" xr:uid="{005E18F2-4447-4781-8F18-5A58920A4F75}">
       <formula1>1</formula1>
       <formula2>1000</formula2>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="It must be a number (integer). This reference is only used during the import process." sqref="K1" xr:uid="{9C637146-F2E3-4D08-87A8-F70FD358E47E}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Use the Issue ID value to link this work item to an Epic_x000a__x000a_Story Issues are not Child-Issues and should have Epic Link instead. " sqref="M1" xr:uid="{A61138FD-C2B2-49D2-810B-69EAE2230B73}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="This field should be the Issue ID or Issue Key of the child tasks. (upstream linkage is not possible)._x000a__x000a__x000a_To link Epics and Stories, use the Epic Link from the Story Issue." sqref="O1:Q1" xr:uid="{BE6B7503-A11A-4130-9D63-988F0CFED80E}"/>
-    <dataValidation allowBlank="1" showErrorMessage="1" promptTitle="Warning" prompt="Field only used for Epic Issues, so they can be referenced in Story Issues via the Epic Link field.," sqref="L2 N2" xr:uid="{541AD292-0123-4B65-9663-081991FDF0C1}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Field only used for Epic Issues, so they can be referenced in Story Issues via the Epic Link field.," sqref="L1" xr:uid="{64C73155-DEE7-497D-8A98-01E54655ACA8}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="It must be a number (integer) or the Work Item key. This reference is only used during the import process to set the parent." sqref="L1" xr:uid="{8A2BE248-5762-43AD-9C47-C5A92A2E2357}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Field only used for Epic work item, so they can be referenced in Story work items via the Epic Link field. _x000a_DC Only" sqref="N1" xr:uid="{E8F6E005-1F9B-40F3-B24C-E2A3D286C532}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="J2:J3" xr:uid="{386E3B68-2486-4DDE-BEB1-45F897521149}"/>
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" promptTitle="Warning" prompt="This field should be the Issue ID or Issue Key of the child tasks. (upstream linkage is not possible)._x000a__x000a__x000a_To link Epics and Stories, use the Epic Link from the Story Issue." sqref="O2:Q3" xr:uid="{D7BD960D-9CEA-4120-B2E3-2AE0D4661093}">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="It must be a number (integer). This reference is only used during the import process." sqref="L1" xr:uid="{9C637146-F2E3-4D08-87A8-F70FD358E47E}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Use the Issue ID value to link this work item to an Epic_x000a__x000a_Story Issues are not Child-Issues and should have Epic Link instead. " sqref="N1" xr:uid="{A61138FD-C2B2-49D2-810B-69EAE2230B73}"/>
+    <dataValidation allowBlank="1" showErrorMessage="1" promptTitle="Warning" prompt="Field only used for Epic Issues, so they can be referenced in Story Issues via the Epic Link field.," sqref="M2 O2" xr:uid="{541AD292-0123-4B65-9663-081991FDF0C1}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Field only used for Epic Issues, so they can be referenced in Story Issues via the Epic Link field.," sqref="M1" xr:uid="{64C73155-DEE7-497D-8A98-01E54655ACA8}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="It must be a number (integer) or the Work Item key. This reference is only used during the import process to set the parent." sqref="M1" xr:uid="{8A2BE248-5762-43AD-9C47-C5A92A2E2357}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Field only used for Epic work item, so they can be referenced in Story work items via the Epic Link field. _x000a_DC Only, this field is ignored when importing in Jira Cloud" sqref="O1" xr:uid="{E8F6E005-1F9B-40F3-B24C-E2A3D286C532}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="I2:I3" xr:uid="{386E3B68-2486-4DDE-BEB1-45F897521149}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Note" prompt="The content of this column will be ignored during the Jira import." sqref="AD2:AD3" xr:uid="{2DA3EDB6-7635-4349-8860-B614B5B71275}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Permissions" prompt="Updating Existing Issues requires global admin permissions" sqref="D2:D3" xr:uid="{D5E4A4BB-53C8-42DF-9B52-F5E00AC6407B}"/>
+    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" promptTitle="Warning" prompt="Use the Issue ID value to link this work item to an Epic_x000a__x000a_Story Issues are not Child-Issues and should have Epic Link instead. " sqref="N2:N3" xr:uid="{16C14239-D6AA-4935-8809-57760481D8F1}">
       <formula1>1</formula1>
       <formula2>1000</formula2>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Note" prompt="The content of this column will be ignored during the Jira import." sqref="AJ2:AJ3" xr:uid="{2DA3EDB6-7635-4349-8860-B614B5B71275}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Permissions" prompt="Updating Existing Issues requires global admin permissions" sqref="D2:D3" xr:uid="{D5E4A4BB-53C8-42DF-9B52-F5E00AC6407B}"/>
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" promptTitle="Warning" prompt="Use the Issue ID value to link this work item to an Epic_x000a__x000a_Story Issues are not Child-Issues and should have Epic Link instead. " sqref="M2:M3" xr:uid="{16C14239-D6AA-4935-8809-57760481D8F1}">
-      <formula1>1</formula1>
-      <formula2>1000</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="AUTOMATIC FIELD" prompt="Do not manually edit these!" sqref="AC2:AC3 AF1:AH3" xr:uid="{893DA5FE-9FD0-4D28-BBD0-3D7AEDECEACB}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="H2:H3" xr:uid="{65EDED96-6789-400B-B504-6BC3F5A79E70}">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="AUTOMATIC FIELD" prompt="Do not manually edit these!" sqref="V2:V3 Y1:AB3" xr:uid="{893DA5FE-9FD0-4D28-BBD0-3D7AEDECEACB}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="G2:G3" xr:uid="{65EDED96-6789-400B-B504-6BC3F5A79E70}">
       <formula1>INDIRECT("CfgComponents[Component.Name]")</formula1>
     </dataValidation>
-    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" error="must be a valid fixversion" sqref="G2:G3" xr:uid="{44FDC20A-8BF5-49B5-9D2C-3A1FE5A7D835}">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" error="must be a valid fixversion" sqref="F2:F3" xr:uid="{44FDC20A-8BF5-49B5-9D2C-3A1FE5A7D835}">
       <formula1>INDIRECT("CfgAssignees[Assignee.Name]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="I2:I3" xr:uid="{A898E2E7-BC45-4B88-BA1E-4AAA377361D4}">
-      <formula1>INDIRECT("CfgSprints[Sprint.Name]")</formula1>
-    </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="Creation Marker (Config Sheet)" prompt="Do not manually edit these!" sqref="AD1:AD3 AE2:AE3" xr:uid="{412C516D-E091-4DDD-9C14-C33AC653C143}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="Feature Pod Label (Config Sheet)" prompt="Do not manually edit these!" sqref="AE1" xr:uid="{D2234141-379F-4413-AB08-6835BD9FF967}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="AUTOMATIC FIELD" prompt="Do not manually edit these! SKIP types won't be imported into Jira" sqref="AI1:AI3" xr:uid="{5A336857-7D14-4900-8734-BED680BE5154}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="Creation Marker (Config Sheet)" prompt="Do not manually edit these!" sqref="W1:W3 X2:X3" xr:uid="{412C516D-E091-4DDD-9C14-C33AC653C143}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="Feature Pod Label (Config Sheet)" prompt="Do not manually edit these!" sqref="X1" xr:uid="{D2234141-379F-4413-AB08-6835BD9FF967}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" promptTitle="AUTOMATIC FIELD" prompt="Do not manually edit these! SKIP types won't be imported into Jira" sqref="AC1:AC3" xr:uid="{5A336857-7D14-4900-8734-BED680BE5154}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Issue Type" sqref="B2:B3" xr:uid="{28BF52BF-C0B0-4D22-B02F-F1408D5A055B}">
       <formula1>INDIRECT("CfgIssueTypeList")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" sqref="F2:F3" xr:uid="{7708D6E2-1D6B-41D8-A9EE-0E87219BA8EA}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" sqref="K2:K3" xr:uid="{7708D6E2-1D6B-41D8-A9EE-0E87219BA8EA}">
       <formula1>INDIRECT("CfgFixVersions[FixVersion.Name]")</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A3" xr:uid="{5EEBB8D5-878D-4D0E-9267-0919B5A1B925}">
       <formula1>INDIRECT("CfgPriorities[Priority.Name]")</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="H2:I3" xr:uid="{A5F34B19-946D-4921-8173-A4364233D328}">
+      <formula1>INDIRECT("CfgTeams[Team.Name]")</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="J2:K3" xr:uid="{A898E2E7-BC45-4B88-BA1E-4AAA377361D4}">
+      <formula1>INDIRECT("CfgSprints[Sprint.Name]")</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="F2" calculatedColumn="1"/>
+    <ignoredError sqref="K2" calculatedColumn="1"/>
   </ignoredErrors>
   <legacyDrawing r:id="rId2"/>
   <tableParts count="1">
@@ -3296,7 +3289,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -3304,40 +3297,40 @@
         <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
       <c r="D4" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="B5" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="E5" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="B6">
         <v>1</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -3345,13 +3338,13 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -3359,13 +3352,13 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="16" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="B8">
         <v>1</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -3373,13 +3366,13 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -3387,13 +3380,13 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="B10">
         <v>1</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="E10">
         <v>2</v>
@@ -3401,7 +3394,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="16" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -3409,7 +3402,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="B12">
         <v>2</v>
@@ -3435,14 +3428,14 @@
   <sheetData>
     <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="18" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="B2" s="17"/>
       <c r="C2" t="str">
@@ -3452,47 +3445,47 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="B3" s="17"/>
       <c r="C3" s="12" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="B4" s="17"/>
       <c r="C4" s="12" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="B5" s="17"/>
       <c r="C5" s="12" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="B6" s="17"/>
       <c r="C6" s="12" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="B7" s="17"/>
       <c r="C7" s="12" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -3501,19 +3494,19 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="B9" s="17">
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B10" s="17"/>
       <c r="C10" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -3521,13 +3514,13 @@
         <v>2</v>
       </c>
       <c r="C11" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B12" s="17"/>
       <c r="C12" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -3547,17 +3540,17 @@
     </row>
     <row r="19" spans="1:3" ht="21" x14ac:dyDescent="0.35">
       <c r="A19" s="18" t="s">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="B19" s="18"/>
       <c r="C19" s="18"/>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="B21" t="s">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="C21" t="s">
         <v>4</v>
@@ -3565,13 +3558,13 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>112</v>
+        <v>103</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -3580,21 +3573,21 @@
         <v>CfgBasic</v>
       </c>
       <c r="B23" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="C23" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>114</v>
+        <v>105</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -3603,10 +3596,10 @@
         <v>CfgAssignees</v>
       </c>
       <c r="B25" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="C25" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -3615,10 +3608,10 @@
         <v>CfgSprints</v>
       </c>
       <c r="B26" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="C26" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -3627,10 +3620,10 @@
         <v>CfgFixVersions</v>
       </c>
       <c r="B27" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="C27" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -3639,10 +3632,10 @@
         <v>CfgIssueTypes</v>
       </c>
       <c r="B28" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="C28" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -3651,10 +3644,10 @@
         <v>CfgComponents</v>
       </c>
       <c r="B29" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="C29" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -3663,21 +3656,21 @@
         <v>CfgPriorities</v>
       </c>
       <c r="B30" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="C30" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="11" t="s">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -3686,10 +3679,10 @@
         <v>CfgAdvanced</v>
       </c>
       <c r="B32" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="C32" t="s">
-        <v>117</v>
+        <v>108</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -3698,21 +3691,21 @@
         <v>CfgCustomFields</v>
       </c>
       <c r="B33" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="C33" t="s">
-        <v>119</v>
+        <v>110</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="11" t="s">
-        <v>120</v>
+        <v>111</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>123</v>
+        <v>114</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -3721,10 +3714,10 @@
         <v>CfgSettings</v>
       </c>
       <c r="B35" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="C35" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -3733,21 +3726,21 @@
         <v>CfgAutofieldValues</v>
       </c>
       <c r="B36" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="C36" t="s">
-        <v>122</v>
+        <v>113</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="B37" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="C37" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -3756,15 +3749,15 @@
         <v>cfg_type_note</v>
       </c>
       <c r="B38" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="C38" t="s">
-        <v>118</v>
+        <v>109</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C45" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -3804,105 +3797,105 @@
   <sheetData>
     <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="18" t="s">
-        <v>105</v>
+        <v>96</v>
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
       <c r="E1" s="18" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
       <c r="F1" s="18"/>
       <c r="G1" s="18"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="19" t="s">
-        <v>105</v>
+        <v>96</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="8"/>
       <c r="E2" s="19" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="F2" s="19"/>
       <c r="G2" s="19"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="B3" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="C3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="E3" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="F3" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="G3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="B4" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="E4" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="F4" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="B5" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="E5" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="F5" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="B6" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="B7" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="C7" s="7"/>
     </row>
@@ -3942,97 +3935,99 @@
   <sheetData>
     <row r="1" spans="1:13" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="18" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="B1" s="18"/>
       <c r="D1" s="18" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="E1" s="18"/>
       <c r="G1" s="18" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="H1" s="18"/>
       <c r="J1" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="L1" s="6" t="s">
-        <v>49</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="L1" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="M1" s="18"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="19" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="B2" s="19"/>
       <c r="D2" s="19" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="E2" s="19"/>
       <c r="G2" s="19" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="H2" s="19"/>
       <c r="J2" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="L2" s="9" t="s">
-        <v>75</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="L2" s="19" t="s">
+        <v>185</v>
+      </c>
+      <c r="M2" s="19"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="D3" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
       <c r="E3" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="G3" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="H3" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="J3" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="L3" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="M3" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="B4" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="D4" t="s">
-        <v>155</v>
+        <v>184</v>
       </c>
       <c r="E4" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="H4">
         <v>97</v>
       </c>
       <c r="J4" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="L4" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="M4">
         <v>3</v>
@@ -4040,19 +4035,19 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>156</v>
+        <v>147</v>
       </c>
       <c r="B5" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
       <c r="D5" t="s">
-        <v>156</v>
+        <v>181</v>
       </c>
       <c r="E5" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
       <c r="L5" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="M5">
         <v>3</v>
@@ -4060,21 +4055,21 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="B6" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="D6" t="s">
-        <v>157</v>
+        <v>182</v>
       </c>
       <c r="E6" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
       <c r="L6" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="M6">
         <v>3</v>
@@ -4082,21 +4077,21 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="B7" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="D7" t="s">
-        <v>158</v>
+        <v>183</v>
       </c>
       <c r="E7" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
       <c r="L7" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="M7">
         <v>2</v>
@@ -4104,21 +4099,15 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="B8" t="s">
-        <v>164</v>
-      </c>
-      <c r="D8" t="s">
-        <v>159</v>
-      </c>
-      <c r="E8" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
       <c r="L8" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="M8">
         <v>4</v>
@@ -4172,83 +4161,85 @@
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
       <c r="J20" s="6" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
     </row>
     <row r="21" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J21" s="9" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="L21" s="9" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
     </row>
     <row r="22" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J22" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="L22" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="23" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J23" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="L23" s="1" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
     </row>
     <row r="24" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J24" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
     </row>
     <row r="25" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J25" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
     </row>
     <row r="26" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J26" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="L26" s="1" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
     </row>
     <row r="27" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J27" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="L27" s="1" t="s">
-        <v>97</v>
+        <v>88</v>
       </c>
     </row>
     <row r="28" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J28" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="L28" s="1" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
     </row>
     <row r="29" spans="7:12" x14ac:dyDescent="0.25">
       <c r="J29" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="8">
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="L2:M2"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="G1:H1"/>
@@ -4274,7 +4265,7 @@
   <sheetPr>
     <tabColor theme="5" tint="0.39997558519241921"/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="44.7109375" customWidth="1"/>
@@ -4285,12 +4276,12 @@
   <sheetData>
     <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="18" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
       <c r="E1" s="18" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="F1" s="18"/>
       <c r="G1" s="18"/>
@@ -4300,61 +4291,104 @@
       <c r="A2" s="19"/>
       <c r="B2" s="19"/>
       <c r="C2" s="8"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
+      <c r="E2" s="21" t="s">
+        <v>198</v>
+      </c>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="B3" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="C3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="E3" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="F3" t="s">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="G3" t="s">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="H3" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="B4" t="s">
-        <v>93</v>
+        <v>84</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>98</v>
+        <v>89</v>
+      </c>
+      <c r="E4" t="s">
+        <v>186</v>
+      </c>
+      <c r="F4" t="s">
+        <v>187</v>
+      </c>
+      <c r="G4" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="B5" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>146</v>
+        <v>137</v>
+      </c>
+      <c r="E5" t="s">
+        <v>189</v>
+      </c>
+      <c r="F5" t="s">
+        <v>190</v>
+      </c>
+      <c r="G5" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E6" t="s">
+        <v>192</v>
+      </c>
+      <c r="F6" t="s">
+        <v>193</v>
+      </c>
+      <c r="G6" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E7" t="s">
+        <v>195</v>
+      </c>
+      <c r="F7" t="s">
+        <v>196</v>
+      </c>
+      <c r="G7" t="s">
+        <v>197</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="E1:H1"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:B2"/>
+    <mergeCell ref="E2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="2">
@@ -4381,46 +4415,46 @@
   <sheetData>
     <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="C1" s="18" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="D1" s="18"/>
       <c r="F1" s="18" t="s">
-        <v>108</v>
+        <v>99</v>
       </c>
       <c r="G1" s="18"/>
       <c r="I1" s="6" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="I2" s="8" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="C3" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="D3" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="F3" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="G3" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="I3" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -4429,13 +4463,13 @@
         <v>Story</v>
       </c>
       <c r="C4" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="D4">
         <v>8</v>
       </c>
       <c r="I4" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -4444,14 +4478,14 @@
         <v>Task</v>
       </c>
       <c r="C5" t="s">
-        <v>107</v>
+        <v>98</v>
       </c>
       <c r="D5" t="str" cm="1">
         <f t="array" aca="1" ref="D5" ca="1">"[" &amp; _xlfn.TEXTJOIN(",",TRUE,_xlfn.MAP(_xlfn._xlws.FILTER(INDIRECT("CfgIgnoreList[IgnoreList.Name]"),INDIRECT("CfgIgnoreList[IgnoreList.Name]")&lt;&gt;""),_xlfn.LAMBDA(_xlpm.x,"""" &amp; SUBSTITUTE(_xlpm.x,"""","""""") &amp; """"))) &amp; "]"</f>
         <v>["Comment","Skip","Note","WorkItem"]</v>
       </c>
       <c r="I5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -4460,7 +4494,7 @@
         <v>Bug</v>
       </c>
       <c r="I6" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -4469,7 +4503,7 @@
         <v>Epic</v>
       </c>
       <c r="I7" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -4504,7 +4538,7 @@
     </row>
     <row r="13" spans="1:9" ht="21" x14ac:dyDescent="0.35">
       <c r="C13" s="18" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="D13" s="18"/>
       <c r="E13" s="18"/>
@@ -4513,7 +4547,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C14" s="20" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="D14" s="20"/>
       <c r="E14" s="20"/>
@@ -4667,12 +4701,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4905,20 +4941,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c471fd26-9765-4fbe-b6fd-c17c1e55c974">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9df69692-83aa-4c55-88c1-62abad05f4fe" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FFE630F-6530-4863-AB67-8477539A0000}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
+    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4943,12 +4980,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FFE630F-6530-4863-AB67-8477539A0000}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{156C3F15-3876-4FBB-8F24-692088DE8D9F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c471fd26-9765-4fbe-b6fd-c17c1e55c974"/>
-    <ds:schemaRef ds:uri="9df69692-83aa-4c55-88c1-62abad05f4fe"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
JT-67 Fix Excel template row behavior
ensure data validation propagates to new JiraDataset rows
remove unintended fixVersion formula propagation
</commit_message>
<xml_diff>
--- a/resources/templates/ImportTemplate.xlsx
+++ b/resources/templates/ImportTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workdir\DeerHide\sources\jira-toolkit\resources\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12369D8C-D85F-47D4-A1D7-BC151129C134}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16B68D21-5867-4D97-B166-F646694B05B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1845" yWindow="4695" windowWidth="33615" windowHeight="23445" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="31920" xr2:uid="{1FA076D1-0294-4A97-AB8C-3ADE2BC9CEA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset" sheetId="1" r:id="rId1"/>
@@ -247,7 +247,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="200">
   <si>
     <t>IssueType</t>
   </si>
@@ -1432,11 +1432,11 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="16" applyAlignment="1">
       <alignment horizontal="left" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="16" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" shrinkToFit="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -1484,7 +1484,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="52">
+  <dxfs count="148">
     <dxf>
       <fill>
         <patternFill patternType="darkUp"/>
@@ -1628,6 +1628,925 @@
       </fill>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill patternType="darkUp"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDAF2D0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2CEEF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <color theme="0" tint="-0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFF9B1AB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF99CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF6699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="darkUp"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDAF2D0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2CEEF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <color theme="0" tint="-0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFF9B1AB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF99CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF6699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="darkUp"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDAF2D0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2CEEF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <color theme="0" tint="-0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFF9B1AB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF99CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF6699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="darkUp"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDAF2D0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2CEEF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <color theme="0" tint="-0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFF9B1AB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF99CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF6699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="darkUp"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDAF2D0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2CEEF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <color theme="0" tint="-0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFF9B1AB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF99CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF6699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="darkUp"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDAF2D0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2CEEF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.89996032593768116"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <color theme="0" tint="-0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFF9B1AB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF99CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF6699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top"/>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
       </font>
@@ -1641,83 +2560,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
     </dxf>
     <dxf>
       <alignment vertical="top"/>
@@ -1762,7 +2605,16 @@
       <alignment vertical="top"/>
     </dxf>
     <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2272,53 +3124,51 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" name="JiraDataset" displayName="JiraDataset" ref="A1:AD3" totalsRowShown="0" headerRowDxfId="50" dataDxfId="49">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}" name="JiraDataset" displayName="JiraDataset" ref="A1:AD3" totalsRowShown="0" headerRowDxfId="143" dataDxfId="142">
   <autoFilter ref="A1:AD3" xr:uid="{933FCFD5-1AB1-4076-B5DD-E2B69F5EB3F2}"/>
   <tableColumns count="30">
-    <tableColumn id="3" xr3:uid="{AF2EC907-349C-4651-852D-6E39C61E17FF}" name="Priority" dataDxfId="48"/>
-    <tableColumn id="2" xr3:uid="{E90C51F2-4386-421F-A3E4-E2CA9D43D396}" name="IssueType" dataDxfId="47"/>
-    <tableColumn id="1" xr3:uid="{BBAD373B-BA13-47E4-9F74-565F4D9E9680}" name="Summary" dataDxfId="46"/>
-    <tableColumn id="4" xr3:uid="{026E5B97-FAFC-4E46-860E-0B0C976B1148}" name="Issue Key" dataDxfId="45"/>
-    <tableColumn id="5" xr3:uid="{A2C262E8-D544-4669-99F1-151EDE081654}" name="Description" dataDxfId="44"/>
-    <tableColumn id="28" xr3:uid="{07F3030C-7187-4B16-BBDB-798304851975}" name="Assignee.Name" dataDxfId="43"/>
-    <tableColumn id="8" xr3:uid="{8C7FB8DB-A85B-4189-93D8-0F0D4EEEF81B}" name="Component" dataDxfId="42"/>
-    <tableColumn id="31" xr3:uid="{BB70BDE8-70CB-404D-896E-075FB6ED93B1}" name="Team.Name" dataDxfId="20"/>
-    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="17"/>
-    <tableColumn id="9" xr3:uid="{DC5101A8-1204-44D2-BC2C-FEE1A4EFE7C1}" name="Sprint Name" dataDxfId="18"/>
-    <tableColumn id="7" xr3:uid="{0FAD1ACC-432E-462C-8B89-71540710BCB5}" name="FixVersion" dataDxfId="16">
-      <calculatedColumnFormula>'Config - Mappings'!$J$4</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="41"/>
-    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="40"/>
-    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="39"/>
-    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="38">
+    <tableColumn id="3" xr3:uid="{AF2EC907-349C-4651-852D-6E39C61E17FF}" name="Priority" dataDxfId="141"/>
+    <tableColumn id="2" xr3:uid="{E90C51F2-4386-421F-A3E4-E2CA9D43D396}" name="IssueType" dataDxfId="140"/>
+    <tableColumn id="1" xr3:uid="{BBAD373B-BA13-47E4-9F74-565F4D9E9680}" name="Summary" dataDxfId="139"/>
+    <tableColumn id="4" xr3:uid="{026E5B97-FAFC-4E46-860E-0B0C976B1148}" name="Issue Key" dataDxfId="138"/>
+    <tableColumn id="5" xr3:uid="{A2C262E8-D544-4669-99F1-151EDE081654}" name="Description" dataDxfId="137"/>
+    <tableColumn id="28" xr3:uid="{07F3030C-7187-4B16-BBDB-798304851975}" name="Assignee.Name" dataDxfId="136"/>
+    <tableColumn id="8" xr3:uid="{8C7FB8DB-A85B-4189-93D8-0F0D4EEEF81B}" name="Component" dataDxfId="135"/>
+    <tableColumn id="31" xr3:uid="{BB70BDE8-70CB-404D-896E-075FB6ED93B1}" name="Team.Name" dataDxfId="134"/>
+    <tableColumn id="40" xr3:uid="{1F406792-7ED2-4476-8FF4-4C6ABA231C97}" name="Estimate" dataDxfId="133"/>
+    <tableColumn id="9" xr3:uid="{DC5101A8-1204-44D2-BC2C-FEE1A4EFE7C1}" name="Sprint Name" dataDxfId="132"/>
+    <tableColumn id="7" xr3:uid="{0FAD1ACC-432E-462C-8B89-71540710BCB5}" name="FixVersion" dataDxfId="131"/>
+    <tableColumn id="10" xr3:uid="{70B7C471-B624-430B-8992-4711F27BB17E}" name="Issue ID" dataDxfId="130"/>
+    <tableColumn id="30" xr3:uid="{938D6CA2-8309-4146-9B62-E8CDFAB7B1C9}" name="Parent" dataDxfId="129"/>
+    <tableColumn id="11" xr3:uid="{594BD56F-7D1D-408F-BEDC-6BB9854C71A1}" name="Epic Link" dataDxfId="128"/>
+    <tableColumn id="33" xr3:uid="{3A94D4B2-1A5B-4BBF-B398-E56D2BB7F948}" name="Epic Name" dataDxfId="127">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[IssueType]]="Epic",JiraDataset[[#This Row],[Summary]],"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="37"/>
-    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="36"/>
-    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="35"/>
-    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="34"/>
-    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="33"/>
-    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="32"/>
-    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="22">
+    <tableColumn id="12" xr3:uid="{0699B70E-673B-4238-8A66-12FC943A4812}" name="Labels" dataDxfId="126"/>
+    <tableColumn id="13" xr3:uid="{9840B81F-2CA6-4708-8C93-3E7C8F72A676}" name="Labels1" dataDxfId="125"/>
+    <tableColumn id="14" xr3:uid="{D4A99C0B-46B7-484A-842E-D62E9D5D9341}" name="Labels2" dataDxfId="124"/>
+    <tableColumn id="15" xr3:uid="{1D1C275E-5C65-4393-9663-6C5F617591E1}" name="Labels3" dataDxfId="123"/>
+    <tableColumn id="16" xr3:uid="{D823FA91-7106-42D3-9DBC-B337C509EB09}" name="Labels4" dataDxfId="122"/>
+    <tableColumn id="17" xr3:uid="{05A07F85-1763-4A66-9CBB-4A760BD03D27}" name="Labels5" dataDxfId="121"/>
+    <tableColumn id="21" xr3:uid="{105F2D0F-70C1-4517-A55F-4C1DDFE85301}" name="Sprint" dataDxfId="120">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], CfgSprints[], 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="31">
+    <tableColumn id="22" xr3:uid="{D5984986-D838-4F87-A554-5DC4CA005452}" name="Labels0001" dataDxfId="119">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgMisc[Name], CfgMisc[Value],"",1))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="30">
+    <tableColumn id="39" xr3:uid="{C24E9ADD-96A8-4DBB-86A0-08D41975D750}" name="Labels0002" dataDxfId="118">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Work Group", CfgMisc[Name], CfgMisc[Value],"",1))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="21">
+    <tableColumn id="6" xr3:uid="{A6D8D5A6-43EE-415C-80C1-30372C7FE5BF}" name="Assignee" dataDxfId="117">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Assignee.Name]], CfgAssignees[], 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="32" xr3:uid="{B9236297-6F08-4471-BC00-A337F6321979}" name="Team" dataDxfId="19">
+    <tableColumn id="32" xr3:uid="{B9236297-6F08-4471-BC00-A337F6321979}" name="Team" dataDxfId="116">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Team.Name]], CfgTeams[], 2, FALSE), ""))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="29">
+    <tableColumn id="23" xr3:uid="{51D4B5F4-C6D3-4EEC-8B1B-7BEC6E526A64}" name="Project Key" dataDxfId="115">
       <calculatedColumnFormula>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("jira.project.key", CfgBasic[Name], CfgBasic[Value]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="28">
+    <tableColumn id="42" xr3:uid="{82B78F0D-CAEF-4615-B12A-B15ACF33913C}" name="OrigEst" dataDxfId="114">
       <calculatedColumnFormula array="1">IF(
   JiraDataset[[#This Row],[RowType]]=cfg_type_skip,
   "",
@@ -2334,7 +3184,7 @@
   )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="27">
+    <tableColumn id="44" xr3:uid="{C92FD7EC-0EAB-4967-A0E5-D2427E3A55B4}" name="RowType" dataDxfId="113">
       <calculatedColumnFormula array="1">IFERROR(
     _xlfn.IFS(
         JiraDataset[[#This Row],[IssueType]] = cfg_type_comment,"SKIP",
@@ -2344,7 +3194,7 @@
     cfg_type_workitem
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="26"/>
+    <tableColumn id="24" xr3:uid="{B63E8FC4-20B3-4755-92F2-EA1F700CA72E}" name="Note" dataDxfId="112"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2354,7 +3204,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}" name="CfgPriorities" displayName="CfgPriorities" ref="L22:L28" totalsRowShown="0">
   <autoFilter ref="L22:L28" xr:uid="{A6C0EE44-3F60-4588-BF11-75C3DD021846}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="51"/>
+    <tableColumn id="1" xr3:uid="{3B3BE2ED-38C4-410B-B0BF-4A9BD9B4B974}" name="Priority.Name" dataDxfId="145"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2390,7 +3240,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{724752C0-2EB0-4307-9766-E95D142383BC}" name="Name"/>
     <tableColumn id="2" xr3:uid="{1B4D7FE1-60C9-4319-8B9F-E66C19764AEE}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{F0634D25-384E-480B-B675-9F8463C0D844}" name="Note" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{F0634D25-384E-480B-B675-9F8463C0D844}" name="Note" dataDxfId="144"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2446,7 +3296,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{D4E1611F-A2CF-465D-A219-1759EA66687D}" name="Name"/>
     <tableColumn id="2" xr3:uid="{174D0D86-B1AA-4BF7-AC91-FCACFC898851}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Note" dataDxfId="25"/>
+    <tableColumn id="3" xr3:uid="{4D0493E3-2ED0-412B-9468-835FC91C2910}" name="Note" dataDxfId="147"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2458,7 +3308,7 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{19232286-858A-4316-B524-2259E904D535}" name="Name"/>
     <tableColumn id="2" xr3:uid="{E6137B31-22A5-4579-8A81-0FBB4015A668}" name="Value"/>
-    <tableColumn id="3" xr3:uid="{03DA91C8-48E1-4BFC-B993-8C1071BAA534}" name="Note" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{03DA91C8-48E1-4BFC-B993-8C1071BAA534}" name="Note" dataDxfId="146"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2837,7 +3687,7 @@
   <sheetPr>
     <tabColor theme="4"/>
   </sheetPr>
-  <dimension ref="A1:AP3"/>
+  <dimension ref="A1:AD3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
@@ -2854,12 +3704,12 @@
     <col min="15" max="15" width="14.42578125" hidden="1" customWidth="1" outlineLevel="1"/>
     <col min="16" max="16" width="14.28515625" customWidth="1" collapsed="1"/>
     <col min="17" max="21" width="14.28515625" customWidth="1"/>
-    <col min="22" max="22" width="14.28515625" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="23" max="24" width="13.140625" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="25" max="26" width="28.140625" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="27" max="27" width="13.42578125" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="28" max="29" width="28.140625" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="30" max="30" width="21.140625" customWidth="1" collapsed="1"/>
+    <col min="22" max="22" width="14.28515625" customWidth="1" outlineLevel="1"/>
+    <col min="23" max="24" width="13.140625" customWidth="1" outlineLevel="1"/>
+    <col min="25" max="26" width="28.140625" customWidth="1" outlineLevel="1"/>
+    <col min="27" max="27" width="13.42578125" customWidth="1" outlineLevel="1"/>
+    <col min="28" max="29" width="28.140625" customWidth="1" outlineLevel="1"/>
+    <col min="30" max="30" width="21.140625" customWidth="1"/>
     <col min="31" max="31" width="14" customWidth="1"/>
     <col min="32" max="32" width="12.5703125" customWidth="1"/>
     <col min="33" max="34" width="13.7109375" customWidth="1"/>
@@ -3065,19 +3915,12 @@
       <c r="G3" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="H3" s="3" t="s">
-        <v>181</v>
-      </c>
+      <c r="H3" s="3"/>
       <c r="I3" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="J3" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="K3" s="3" t="str">
-        <f>'Config - Mappings'!$J$4</f>
-        <v>JITTP Version 1</v>
-      </c>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>
       <c r="N3" s="3"/>
@@ -3097,9 +3940,9 @@
       <c r="S3" s="3"/>
       <c r="T3" s="3"/>
       <c r="U3" s="3"/>
-      <c r="V3" s="3">
+      <c r="V3" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Sprint Name]], CfgSprints[], 2, FALSE), ""))</f>
-        <v>97</v>
+        <v/>
       </c>
       <c r="W3" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("Creation Marker", CfgMisc[Name], CfgMisc[Value],"",1))</f>
@@ -3115,7 +3958,7 @@
       </c>
       <c r="Z3" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",IFERROR(VLOOKUP(JiraDataset[[#This Row],[Team.Name]], CfgTeams[], 2, FALSE), ""))</f>
-        <v>712020:09876543212345678902</v>
+        <v/>
       </c>
       <c r="AA3" s="3" t="str">
         <f>IF(JiraDataset[[#This Row],[RowType]]=cfg_type_skip,"",_xlfn.XLOOKUP("jira.project.key", CfgBasic[Name], CfgBasic[Value]))</f>
@@ -3153,7 +3996,7 @@
     </row>
   </sheetData>
   <protectedRanges>
-    <protectedRange sqref="A1:A1048576 L4:L1048576 C1:E2 D3:E1048576 F1:J3 G4:J1048576 K1:U2 Q4:Z1048576 K3:W3 N4:O1048576" name="User Input"/>
+    <protectedRange sqref="L4:L1048576 C1:E2 F1:J3 G4:J1048576 K1:U2 Q4:Z1048576 K3:W3 N4:O1048576 A1:A1048576 D3:E1048576" name="User Input"/>
     <protectedRange algorithmName="SHA-512" hashValue="tpheD+JLADkhiyalt6vInlMwkILPZx4PVQN/k2vmwjOBdYUuHaXCrwtObHeFz5dJh9f853O84pZ1Rn9Ujz33+A==" saltValue="9ir5NB4CJc/69S/Eh84/mA==" spinCount="100000" sqref="V1:AC2 X3:AE3 AA4:AH1048576" name="Computed values"/>
   </protectedRanges>
   <phoneticPr fontId="18" type="noConversion"/>
@@ -3219,7 +4062,7 @@
       <formula>LEN(TRIM(L2))=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations xWindow="1573" yWindow="665" count="22">
+  <dataValidations xWindow="1573" yWindow="665" count="23">
     <dataValidation type="whole" allowBlank="1" showErrorMessage="1" prompt="It must be a number (integer). This reference is only used during the import process." sqref="L2:M2" xr:uid="{005E18F2-4447-4781-8F18-5A58920A4F75}">
       <formula1>1</formula1>
       <formula2>1000</formula2>
@@ -3250,24 +4093,24 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Issue Type" sqref="B2:B3" xr:uid="{28BF52BF-C0B0-4D22-B02F-F1408D5A055B}">
       <formula1>INDIRECT("CfgIssueTypeList")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid fixversion" sqref="K2:K3" xr:uid="{7708D6E2-1D6B-41D8-A9EE-0E87219BA8EA}">
-      <formula1>INDIRECT("CfgFixVersions[FixVersion.Name]")</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A3" xr:uid="{5EEBB8D5-878D-4D0E-9267-0919B5A1B925}">
       <formula1>INDIRECT("CfgPriorities[Priority.Name]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="H2:I3" xr:uid="{A5F34B19-946D-4921-8173-A4364233D328}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="I2:I3" xr:uid="{A5F34B19-946D-4921-8173-A4364233D328}">
       <formula1>INDIRECT("CfgTeams[Team.Name]")</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="J2:K3" xr:uid="{A898E2E7-BC45-4B88-BA1E-4AAA377361D4}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="must be a valid component" sqref="J2:J3" xr:uid="{A898E2E7-BC45-4B88-BA1E-4AAA377361D4}">
       <formula1>INDIRECT("CfgSprints[Sprint.Name]")</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="must be a valid component" sqref="H2:H3" xr:uid="{7B68C246-CBB3-46A9-A050-68D1E898B8E3}">
+      <formula1>INDIRECT("CfgTeams[Team.Name]")</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K3" xr:uid="{C49FC18E-7E95-4F52-B450-E61F830A5C7D}">
+      <formula1>INDIRECT("CfgFixVersions[FixVersion.Name]")</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
-  <ignoredErrors>
-    <ignoredError sqref="K2" calculatedColumn="1"/>
-  </ignoredErrors>
   <legacyDrawing r:id="rId2"/>
   <tableParts count="1">
     <tablePart r:id="rId3"/>
@@ -4291,12 +5134,12 @@
       <c r="A2" s="19"/>
       <c r="B2" s="19"/>
       <c r="C2" s="8"/>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="20" t="s">
         <v>198</v>
       </c>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -4546,13 +5389,13 @@
       <c r="G13" s="18"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C14" s="20" t="s">
+      <c r="C14" s="21" t="s">
         <v>164</v>
       </c>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="20"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="21"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="21"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C15" t="str" cm="1">

</xml_diff>